<commit_message>
modified to allow for two different dead storage values
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8FFAD0-BBCF-7C4A-9F46-9354CAB76C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75A060D-8C3C-5A4B-A9D3-F7AC49307262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="500" windowWidth="33680" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="2520" yWindow="760" windowWidth="33680" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1097,7 +1097,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1159,31 +1159,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1208,9 +1183,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1234,19 +1206,46 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1783,60 +1782,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="24" t="s">
+      <c r="B1" s="41"/>
+      <c r="C1" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="23" t="s">
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="23"/>
-      <c r="H1" s="24" t="s">
+      <c r="G1" s="41"/>
+      <c r="H1" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="23" t="s">
+      <c r="I1" s="42"/>
+      <c r="J1" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="23"/>
-      <c r="L1" s="25" t="s">
+      <c r="K1" s="41"/>
+      <c r="L1" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="M1" s="25"/>
-      <c r="N1" s="27" t="s">
+      <c r="M1" s="44"/>
+      <c r="N1" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="25" t="s">
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25"/>
-      <c r="U1" s="26" t="s">
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="45" t="s">
         <v>44</v>
       </c>
-      <c r="V1" s="26"/>
+      <c r="V1" s="45"/>
       <c r="W1" s="4" t="s">
         <v>46</v>
       </c>
       <c r="X1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AC1" s="23" t="s">
+      <c r="AC1" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="23"/>
-      <c r="AG1" s="23"/>
-      <c r="AH1" s="23"/>
+      <c r="AD1" s="41"/>
+      <c r="AE1" s="41"/>
+      <c r="AF1" s="41"/>
+      <c r="AG1" s="41"/>
+      <c r="AH1" s="41"/>
       <c r="AI1" s="7" t="s">
         <v>37</v>
       </c>
@@ -6373,16 +6372,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AC1:AH1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="R1:T1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="N1:Q1"/>
-    <mergeCell ref="AC1:AH1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="R1:T1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6393,9 +6392,9 @@
   <dimension ref="A1:AN159"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="62.1640625" style="33" customWidth="1"/>
-    <col min="2" max="2" width="14" style="36" customWidth="1"/>
-    <col min="3" max="3" width="4.1640625" style="32" customWidth="1"/>
+    <col min="1" max="1" width="62.1640625" style="24" customWidth="1"/>
+    <col min="2" max="2" width="14" style="27" customWidth="1"/>
+    <col min="3" max="3" width="4.1640625" style="23" customWidth="1"/>
     <col min="4" max="4" width="27" style="22" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="44" style="10" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="11" style="4" customWidth="1"/>
@@ -6414,7 +6413,7 @@
     <col min="22" max="22" width="12.5" style="4" customWidth="1"/>
     <col min="23" max="23" width="9.1640625" style="5" customWidth="1"/>
     <col min="24" max="25" width="13.33203125" style="4" customWidth="1"/>
-    <col min="26" max="26" width="62.1640625" style="33" customWidth="1"/>
+    <col min="26" max="26" width="62.1640625" style="24" customWidth="1"/>
     <col min="27" max="29" width="14.6640625" customWidth="1"/>
     <col min="30" max="32" width="14.1640625" customWidth="1"/>
     <col min="33" max="33" width="4.1640625" customWidth="1"/>
@@ -6422,9 +6421,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="33"/>
-      <c r="B1" s="36"/>
-      <c r="C1" s="32"/>
+      <c r="A1" s="24"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="23"/>
       <c r="D1" s="22"/>
       <c r="E1" s="10"/>
       <c r="F1" s="5" t="s">
@@ -6453,12 +6452,12 @@
       <c r="W1" s="5"/>
       <c r="X1" s="5"/>
       <c r="Y1" s="5"/>
-      <c r="Z1" s="33"/>
+      <c r="Z1" s="24"/>
     </row>
     <row r="2" spans="1:40" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="33"/>
-      <c r="B2" s="36"/>
-      <c r="C2" s="32"/>
+      <c r="A2" s="24"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="23"/>
       <c r="D2" s="22"/>
       <c r="E2" s="10"/>
       <c r="F2" s="5" t="s">
@@ -6467,10 +6466,10 @@
       <c r="G2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="27">
+      <c r="H2" s="43">
         <v>150</v>
       </c>
-      <c r="I2" s="27"/>
+      <c r="I2" s="43"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
@@ -6489,22 +6488,22 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
       <c r="Y2" s="5"/>
-      <c r="Z2" s="33"/>
+      <c r="Z2" s="24"/>
     </row>
     <row r="3" spans="1:40" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="33"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="32"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="23"/>
       <c r="D3" s="22"/>
       <c r="E3" s="10"/>
       <c r="F3" s="5"/>
       <c r="G3" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="43">
         <v>30</v>
       </c>
-      <c r="I3" s="27"/>
+      <c r="I3" s="43"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
@@ -6521,7 +6520,7 @@
       <c r="W3" s="5"/>
       <c r="X3" s="5"/>
       <c r="Y3" s="5"/>
-      <c r="Z3" s="33"/>
+      <c r="Z3" s="24"/>
     </row>
     <row r="4" spans="1:40" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F4" s="8">
@@ -6558,11 +6557,11 @@
         <v>6</v>
       </c>
       <c r="Y4" s="20"/>
-      <c r="AD4" s="30" t="s">
+      <c r="AD4" s="51" t="s">
         <v>89</v>
       </c>
-      <c r="AE4" s="30"/>
-      <c r="AF4" s="30"/>
+      <c r="AE4" s="51"/>
+      <c r="AF4" s="51"/>
       <c r="AK4" t="s">
         <v>94</v>
       </c>
@@ -6577,51 +6576,51 @@
       </c>
     </row>
     <row r="5" spans="1:40" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="E5" s="31" t="s">
+      <c r="E5" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="G5" s="29"/>
+      <c r="G5" s="52"/>
       <c r="H5" s="17"/>
-      <c r="I5" s="29" t="s">
+      <c r="I5" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="J5" s="29"/>
-      <c r="L5" s="29" t="s">
+      <c r="J5" s="52"/>
+      <c r="L5" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="M5" s="29"/>
-      <c r="O5" s="29" t="s">
+      <c r="M5" s="52"/>
+      <c r="O5" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="P5" s="29"/>
-      <c r="R5" s="29" t="s">
+      <c r="P5" s="52"/>
+      <c r="R5" s="52" t="s">
         <v>83</v>
       </c>
-      <c r="S5" s="29"/>
-      <c r="U5" s="29" t="s">
+      <c r="S5" s="52"/>
+      <c r="U5" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="V5" s="29"/>
-      <c r="X5" s="29" t="s">
+      <c r="V5" s="52"/>
+      <c r="X5" s="52" t="s">
         <v>135</v>
       </c>
-      <c r="Y5" s="29"/>
-      <c r="Z5" s="33" t="s">
+      <c r="Y5" s="52"/>
+      <c r="Z5" s="24" t="s">
         <v>284</v>
       </c>
-      <c r="AC5" s="46" t="s">
+      <c r="AC5" s="36" t="s">
         <v>234</v>
       </c>
       <c r="AD5" s="21" t="s">
@@ -6647,7 +6646,7 @@
       </c>
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="B6" s="39"/>
+      <c r="B6" s="30"/>
       <c r="F6" s="4" t="s">
         <v>24</v>
       </c>
@@ -6714,10 +6713,10 @@
       </c>
     </row>
     <row r="7" spans="1:40" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="49" t="s">
+      <c r="A7" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E7" s="10" t="s">
@@ -6777,7 +6776,7 @@
         <f>MAX(V7-V9,0)</f>
         <v>249360</v>
       </c>
-      <c r="Z7" s="49" t="s">
+      <c r="Z7" s="38" t="s">
         <v>285</v>
       </c>
       <c r="AD7" s="19">
@@ -6804,10 +6803,10 @@
       </c>
     </row>
     <row r="8" spans="1:40" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E8" s="10" t="s">
@@ -6869,7 +6868,7 @@
         <f>V8-V9+V12</f>
         <v>249801</v>
       </c>
-      <c r="Z8" s="49" t="s">
+      <c r="Z8" s="38" t="s">
         <v>286</v>
       </c>
       <c r="AD8" s="19">
@@ -6896,10 +6895,10 @@
       </c>
     </row>
     <row r="9" spans="1:40" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="38" t="s">
         <v>224</v>
       </c>
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E9" s="10" t="s">
@@ -6947,7 +6946,7 @@
       <c r="Y9" s="4">
         <v>116</v>
       </c>
-      <c r="Z9" s="49" t="s">
+      <c r="Z9" s="38" t="s">
         <v>288</v>
       </c>
       <c r="AD9" s="19">
@@ -6974,10 +6973,10 @@
       </c>
     </row>
     <row r="10" spans="1:40" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="38" t="s">
         <v>223</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E10" s="10" t="s">
@@ -7011,7 +7010,7 @@
         <f>-MIN(Y7-Y9,0)</f>
         <v>0</v>
       </c>
-      <c r="Z10" s="49" t="s">
+      <c r="Z10" s="38" t="s">
         <v>289</v>
       </c>
       <c r="AD10" s="19">
@@ -7026,10 +7025,10 @@
       </c>
     </row>
     <row r="11" spans="1:40" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="49" t="s">
+      <c r="A11" s="38" t="s">
         <v>221</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E11" s="10" t="s">
@@ -7063,7 +7062,7 @@
         <f>MAX(Y10-Y25,0)</f>
         <v>0</v>
       </c>
-      <c r="Z11" s="49" t="s">
+      <c r="Z11" s="38" t="s">
         <v>290</v>
       </c>
       <c r="AD11" s="19">
@@ -7078,10 +7077,10 @@
       </c>
     </row>
     <row r="12" spans="1:40" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="49" t="s">
+      <c r="A12" s="38" t="s">
         <v>222</v>
       </c>
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E12" s="10" t="s">
@@ -7108,7 +7107,7 @@
       <c r="Y12" s="4">
         <v>110</v>
       </c>
-      <c r="Z12" s="49" t="s">
+      <c r="Z12" s="38" t="s">
         <v>287</v>
       </c>
       <c r="AD12" s="19">
@@ -7123,10 +7122,10 @@
       </c>
     </row>
     <row r="13" spans="1:40" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="49" t="s">
+      <c r="A13" s="38" t="s">
         <v>158</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E13" s="10" t="s">
@@ -7188,7 +7187,7 @@
         <f>MAX(Y7-Y9,0)</f>
         <v>249244</v>
       </c>
-      <c r="Z13" s="49" t="s">
+      <c r="Z13" s="38" t="s">
         <v>291</v>
       </c>
       <c r="AD13" s="19"/>
@@ -7196,10 +7195,10 @@
       <c r="AF13" s="19"/>
     </row>
     <row r="14" spans="1:40" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="49" t="s">
+      <c r="A14" s="38" t="s">
         <v>225</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E14" s="10" t="s">
@@ -7226,7 +7225,7 @@
       <c r="X14" s="4">
         <v>0.7</v>
       </c>
-      <c r="Z14" s="49" t="s">
+      <c r="Z14" s="38" t="s">
         <v>292</v>
       </c>
       <c r="AD14" s="19">
@@ -7241,10 +7240,10 @@
       </c>
     </row>
     <row r="15" spans="1:40" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="49" t="s">
+      <c r="A15" s="38" t="s">
         <v>249</v>
       </c>
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="31" t="s">
         <v>162</v>
       </c>
       <c r="D15" s="22" t="s">
@@ -7295,7 +7294,7 @@
       <c r="Y15" s="4">
         <v>9</v>
       </c>
-      <c r="Z15" s="49" t="s">
+      <c r="Z15" s="38" t="s">
         <v>296</v>
       </c>
       <c r="AD15" s="19"/>
@@ -7303,10 +7302,10 @@
       <c r="AF15" s="19"/>
     </row>
     <row r="16" spans="1:40" ht="51" x14ac:dyDescent="0.2">
-      <c r="A16" s="49" t="s">
+      <c r="A16" s="38" t="s">
         <v>226</v>
       </c>
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E16" s="10" t="s">
@@ -7315,25 +7314,7 @@
       <c r="F16" s="4">
         <v>1E-3</v>
       </c>
-      <c r="I16" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="L16" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="O16" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="R16" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="U16" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="X16" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="Z16" s="49" t="s">
+      <c r="Z16" s="38" t="s">
         <v>293</v>
       </c>
       <c r="AD16" s="19">
@@ -7348,13 +7329,13 @@
       </c>
     </row>
     <row r="17" spans="1:32" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="49" t="s">
+      <c r="A17" s="38" t="s">
         <v>227</v>
       </c>
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="49" t="s">
         <v>118</v>
       </c>
       <c r="E17" s="10" t="s">
@@ -7363,7 +7344,7 @@
       <c r="F17" s="4">
         <v>0.2</v>
       </c>
-      <c r="Z17" s="49" t="s">
+      <c r="Z17" s="38" t="s">
         <v>294</v>
       </c>
       <c r="AD17" s="19">
@@ -7378,20 +7359,20 @@
       </c>
     </row>
     <row r="18" spans="1:32" ht="51" x14ac:dyDescent="0.2">
-      <c r="A18" s="49" t="s">
+      <c r="A18" s="38" t="s">
         <v>228</v>
       </c>
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="D18" s="28"/>
+      <c r="D18" s="49"/>
       <c r="E18" s="10" t="s">
         <v>138</v>
       </c>
       <c r="F18" s="4">
         <v>0.67</v>
       </c>
-      <c r="Z18" s="53" t="s">
+      <c r="Z18" s="40" t="s">
         <v>295</v>
       </c>
       <c r="AD18" s="19">
@@ -7406,10 +7387,10 @@
       </c>
     </row>
     <row r="19" spans="1:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="49" t="s">
+      <c r="A19" s="38" t="s">
         <v>230</v>
       </c>
-      <c r="B19" s="41" t="s">
+      <c r="B19" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E19" s="10" t="s">
@@ -7421,7 +7402,7 @@
       <c r="G19" s="4">
         <v>100</v>
       </c>
-      <c r="Z19" s="49" t="s">
+      <c r="Z19" s="38" t="s">
         <v>297</v>
       </c>
       <c r="AD19" s="19">
@@ -7436,10 +7417,10 @@
       </c>
     </row>
     <row r="20" spans="1:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" s="49" t="s">
+      <c r="A20" s="38" t="s">
         <v>232</v>
       </c>
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E20" s="10" t="s">
@@ -7451,7 +7432,7 @@
       <c r="G20" s="4">
         <v>0.25</v>
       </c>
-      <c r="Z20" s="49" t="s">
+      <c r="Z20" s="38" t="s">
         <v>298</v>
       </c>
       <c r="AD20" s="19"/>
@@ -7459,10 +7440,10 @@
       <c r="AF20" s="19"/>
     </row>
     <row r="21" spans="1:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="49" t="s">
+      <c r="A21" s="38" t="s">
         <v>280</v>
       </c>
-      <c r="B21" s="42" t="s">
+      <c r="B21" s="32" t="s">
         <v>174</v>
       </c>
       <c r="E21" s="10" t="s">
@@ -7476,7 +7457,7 @@
         <f>G$19*$F$16</f>
         <v>0.1</v>
       </c>
-      <c r="Z21" s="49"/>
+      <c r="Z21" s="38"/>
       <c r="AD21" s="19">
         <v>12</v>
       </c>
@@ -7489,10 +7470,10 @@
       </c>
     </row>
     <row r="22" spans="1:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="49" t="s">
+      <c r="A22" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="32" t="s">
         <v>174</v>
       </c>
       <c r="E22" s="10" t="s">
@@ -7506,7 +7487,7 @@
         <f>G19-G21</f>
         <v>99.9</v>
       </c>
-      <c r="Z22" s="49" t="s">
+      <c r="Z22" s="38" t="s">
         <v>299</v>
       </c>
       <c r="AD22" s="19">
@@ -7533,10 +7514,10 @@
       </c>
     </row>
     <row r="24" spans="1:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="A24" s="49" t="s">
+      <c r="A24" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E24" s="10" t="s">
@@ -7584,7 +7565,7 @@
       <c r="Y24" s="4">
         <v>49500</v>
       </c>
-      <c r="Z24" s="49"/>
+      <c r="Z24" s="38"/>
       <c r="AD24" s="19">
         <v>10</v>
       </c>
@@ -7597,10 +7578,10 @@
       </c>
     </row>
     <row r="25" spans="1:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="A25" s="49" t="s">
+      <c r="A25" s="38" t="s">
         <v>279</v>
       </c>
-      <c r="B25" s="43" t="s">
+      <c r="B25" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E25" s="14" t="s">
@@ -7634,7 +7615,7 @@
         <f>MAX(Y$24-Y$13, 0)</f>
         <v>0</v>
       </c>
-      <c r="Z25" s="49"/>
+      <c r="Z25" s="38"/>
       <c r="AD25" s="19">
         <v>6</v>
       </c>
@@ -7647,10 +7628,10 @@
       </c>
     </row>
     <row r="26" spans="1:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" s="49" t="s">
+      <c r="A26" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E26" s="14" t="s">
@@ -7712,7 +7693,7 @@
         <f>MIN(Y13,Y24)</f>
         <v>49500</v>
       </c>
-      <c r="Z26" s="49"/>
+      <c r="Z26" s="38"/>
       <c r="AD26" s="19">
         <v>3</v>
       </c>
@@ -7754,16 +7735,16 @@
       </c>
     </row>
     <row r="28" spans="1:32" ht="73" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="49" t="s">
+      <c r="A28" s="38" t="s">
         <v>278</v>
       </c>
-      <c r="B28" s="41" t="s">
+      <c r="B28" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="D28" s="28" t="s">
+      <c r="D28" s="49" t="s">
         <v>170</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="25" t="s">
         <v>68</v>
       </c>
       <c r="F28" s="4">
@@ -7772,17 +7753,17 @@
       <c r="G28" s="4">
         <v>0.92</v>
       </c>
-      <c r="Z28" s="49"/>
+      <c r="Z28" s="38"/>
     </row>
     <row r="29" spans="1:32" ht="73" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="49" t="s">
+      <c r="A29" s="38" t="s">
         <v>233</v>
       </c>
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="32" t="s">
         <v>174</v>
       </c>
-      <c r="D29" s="28"/>
-      <c r="E29" s="34" t="s">
+      <c r="D29" s="49"/>
+      <c r="E29" s="25" t="s">
         <v>171</v>
       </c>
       <c r="F29" s="4">
@@ -7793,10 +7774,10 @@
         <f>F29</f>
         <v>2E-3</v>
       </c>
-      <c r="Z29" s="49"/>
+      <c r="Z29" s="38"/>
     </row>
     <row r="30" spans="1:32" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D30" s="35"/>
+      <c r="D30" s="26"/>
     </row>
     <row r="31" spans="1:32" ht="17" x14ac:dyDescent="0.2">
       <c r="E31" s="15" t="s">
@@ -7818,10 +7799,10 @@
       <c r="Y31" s="8"/>
     </row>
     <row r="32" spans="1:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" s="49" t="s">
+      <c r="A32" s="38" t="s">
         <v>168</v>
       </c>
-      <c r="B32" s="41" t="s">
+      <c r="B32" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E32" s="10" t="s">
@@ -7848,7 +7829,7 @@
       <c r="X32" s="4">
         <v>2520000</v>
       </c>
-      <c r="Z32" s="49"/>
+      <c r="Z32" s="38"/>
     </row>
     <row r="34" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="E34" s="11" t="s">
@@ -7891,7 +7872,7 @@
       </c>
     </row>
     <row r="36" spans="1:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" s="33" t="s">
+      <c r="A36" s="24" t="s">
         <v>179</v>
       </c>
       <c r="E36" s="14" t="s">
@@ -7944,10 +7925,10 @@
       </c>
     </row>
     <row r="37" spans="1:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="A37" s="47" t="s">
+      <c r="A37" s="46" t="s">
         <v>180</v>
       </c>
-      <c r="B37" s="37" t="s">
+      <c r="B37" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E37" s="14" t="s">
@@ -8032,11 +8013,11 @@
         <f>V37-X37</f>
         <v>85</v>
       </c>
-      <c r="Z37" s="51"/>
+      <c r="Z37" s="37"/>
     </row>
     <row r="38" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="48"/>
-      <c r="B38" s="37"/>
+      <c r="B38" s="47"/>
       <c r="E38" s="14" t="s">
         <v>69</v>
       </c>
@@ -8118,11 +8099,11 @@
         <f>V38-X38</f>
         <v>80</v>
       </c>
-      <c r="Z38" s="49"/>
+      <c r="Z38" s="38"/>
     </row>
     <row r="39" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="48"/>
-      <c r="B39" s="37"/>
+      <c r="B39" s="47"/>
       <c r="E39" s="14" t="s">
         <v>79</v>
       </c>
@@ -8203,11 +8184,11 @@
         <f>V39-X39</f>
         <v>92</v>
       </c>
-      <c r="Z39" s="49"/>
+      <c r="Z39" s="38"/>
     </row>
     <row r="40" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="48"/>
-      <c r="B40" s="37"/>
+      <c r="B40" s="47"/>
       <c r="E40" s="14" t="s">
         <v>80</v>
       </c>
@@ -8287,7 +8268,7 @@
         <f>V40-X40</f>
         <v>43</v>
       </c>
-      <c r="Z40" s="49"/>
+      <c r="Z40" s="38"/>
     </row>
     <row r="41" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="E41" s="14" t="s">
@@ -8301,7 +8282,7 @@
       <c r="A42" s="48" t="s">
         <v>191</v>
       </c>
-      <c r="B42" s="37" t="s">
+      <c r="B42" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E42" s="14" t="s">
@@ -8334,11 +8315,11 @@
         <f>IF(V37=0, 0, V95*X37/V37)</f>
         <v>0</v>
       </c>
-      <c r="Z42" s="49"/>
+      <c r="Z42" s="38"/>
     </row>
     <row r="43" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="48"/>
-      <c r="B43" s="37"/>
+      <c r="B43" s="47"/>
       <c r="E43" s="14" t="s">
         <v>196</v>
       </c>
@@ -8369,11 +8350,11 @@
         <f>IF(V38=0, 0, V96*X38/V38)</f>
         <v>0</v>
       </c>
-      <c r="Z43" s="49"/>
+      <c r="Z43" s="38"/>
     </row>
     <row r="44" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="48"/>
-      <c r="B44" s="37"/>
+      <c r="B44" s="47"/>
       <c r="E44" s="14" t="s">
         <v>197</v>
       </c>
@@ -8404,11 +8385,11 @@
         <f>IF(V39=0, 0, V97*X39/V39)</f>
         <v>0</v>
       </c>
-      <c r="Z44" s="49"/>
+      <c r="Z44" s="38"/>
     </row>
     <row r="45" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="48"/>
-      <c r="B45" s="37"/>
+      <c r="B45" s="47"/>
       <c r="E45" s="14" t="s">
         <v>198</v>
       </c>
@@ -8439,13 +8420,13 @@
         <f>IF(V40=0, 0, V98*X40/V40)</f>
         <v>0</v>
       </c>
-      <c r="Z45" s="49"/>
+      <c r="Z45" s="38"/>
     </row>
     <row r="46" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A46" s="49" t="s">
+      <c r="A46" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="B46" s="40" t="s">
+      <c r="B46" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E46" s="14"/>
@@ -8477,7 +8458,7 @@
         <f>SUM(Y42:Y45)</f>
         <v>0</v>
       </c>
-      <c r="Z46" s="49"/>
+      <c r="Z46" s="38"/>
     </row>
     <row r="47" spans="1:27" ht="17" x14ac:dyDescent="0.2">
       <c r="E47" s="14" t="s">
@@ -8491,10 +8472,10 @@
       <c r="A48" s="48" t="s">
         <v>263</v>
       </c>
-      <c r="B48" s="37" t="s">
+      <c r="B48" s="47" t="s">
         <v>174</v>
       </c>
-      <c r="D48" s="28" t="s">
+      <c r="D48" s="49" t="s">
         <v>251</v>
       </c>
       <c r="E48" s="14" t="s">
@@ -8528,12 +8509,12 @@
         <f>MIN(Y42,Y$15*X37)</f>
         <v>0</v>
       </c>
-      <c r="Z48" s="49"/>
+      <c r="Z48" s="38"/>
     </row>
     <row r="49" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="48"/>
-      <c r="B49" s="37"/>
-      <c r="D49" s="28"/>
+      <c r="B49" s="47"/>
+      <c r="D49" s="49"/>
       <c r="E49" s="14" t="s">
         <v>252</v>
       </c>
@@ -8565,12 +8546,12 @@
         <f t="shared" ref="Y49" si="8">MIN(Y43,Y$15*X38)</f>
         <v>0</v>
       </c>
-      <c r="Z49" s="49"/>
+      <c r="Z49" s="38"/>
     </row>
     <row r="50" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="48"/>
-      <c r="B50" s="37"/>
-      <c r="D50" s="28"/>
+      <c r="B50" s="47"/>
+      <c r="D50" s="49"/>
       <c r="E50" s="14" t="s">
         <v>253</v>
       </c>
@@ -8602,12 +8583,12 @@
         <f>MIN(Y44,Y$15*X39)</f>
         <v>0</v>
       </c>
-      <c r="Z50" s="49"/>
+      <c r="Z50" s="38"/>
     </row>
     <row r="51" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="48"/>
-      <c r="B51" s="37"/>
-      <c r="D51" s="28"/>
+      <c r="B51" s="47"/>
+      <c r="D51" s="49"/>
       <c r="E51" s="14" t="s">
         <v>254</v>
       </c>
@@ -8639,13 +8620,13 @@
         <f>MIN(Y45,Y$15*X40)</f>
         <v>0</v>
       </c>
-      <c r="Z51" s="49"/>
+      <c r="Z51" s="38"/>
     </row>
     <row r="52" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A52" s="49" t="s">
+      <c r="A52" s="38" t="s">
         <v>264</v>
       </c>
-      <c r="B52" s="40" t="s">
+      <c r="B52" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E52" s="14"/>
@@ -8677,13 +8658,13 @@
         <f>SUM(Y48:Y51)</f>
         <v>0</v>
       </c>
-      <c r="Z52" s="49"/>
+      <c r="Z52" s="38"/>
     </row>
     <row r="53" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A53" s="49" t="s">
+      <c r="A53" s="38" t="s">
         <v>266</v>
       </c>
-      <c r="B53" s="40"/>
+      <c r="B53" s="28"/>
       <c r="E53" s="14"/>
       <c r="G53" s="4">
         <f>G46-G52</f>
@@ -8713,7 +8694,7 @@
         <f>Y46-Y52</f>
         <v>0</v>
       </c>
-      <c r="Z53" s="49"/>
+      <c r="Z53" s="38"/>
     </row>
     <row r="54" spans="1:26" x14ac:dyDescent="0.2">
       <c r="E54" s="14"/>
@@ -8722,7 +8703,7 @@
       <c r="A55" s="48" t="s">
         <v>193</v>
       </c>
-      <c r="B55" s="37" t="s">
+      <c r="B55" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E55" s="14" t="s">
@@ -8756,11 +8737,11 @@
         <f>Y42*$G$20</f>
         <v>0</v>
       </c>
-      <c r="Z55" s="49"/>
+      <c r="Z55" s="38"/>
     </row>
     <row r="56" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A56" s="48"/>
-      <c r="B56" s="37"/>
+      <c r="B56" s="47"/>
       <c r="E56" s="14" t="s">
         <v>200</v>
       </c>
@@ -8792,11 +8773,11 @@
         <f>Y43*$G$20</f>
         <v>0</v>
       </c>
-      <c r="Z56" s="49"/>
+      <c r="Z56" s="38"/>
     </row>
     <row r="57" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A57" s="48"/>
-      <c r="B57" s="37"/>
+      <c r="B57" s="47"/>
       <c r="E57" s="14" t="s">
         <v>201</v>
       </c>
@@ -8828,11 +8809,11 @@
         <f>Y44*$G$20</f>
         <v>0</v>
       </c>
-      <c r="Z57" s="49"/>
+      <c r="Z57" s="38"/>
     </row>
     <row r="58" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="48"/>
-      <c r="B58" s="37"/>
+      <c r="B58" s="47"/>
       <c r="E58" s="14" t="s">
         <v>202</v>
       </c>
@@ -8864,13 +8845,13 @@
         <f>Y45*$G$20</f>
         <v>0</v>
       </c>
-      <c r="Z58" s="49"/>
+      <c r="Z58" s="38"/>
     </row>
     <row r="59" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A59" s="49" t="s">
+      <c r="A59" s="38" t="s">
         <v>194</v>
       </c>
-      <c r="B59" s="40" t="s">
+      <c r="B59" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E59" s="14"/>
@@ -8902,7 +8883,7 @@
         <f>SUM(Y55:Y58)</f>
         <v>0</v>
       </c>
-      <c r="Z59" s="49"/>
+      <c r="Z59" s="38"/>
     </row>
     <row r="60" spans="1:26" x14ac:dyDescent="0.2">
       <c r="E60" s="14"/>
@@ -8911,7 +8892,7 @@
       <c r="A61" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="B61" s="37" t="s">
+      <c r="B61" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E61" s="14" t="s">
@@ -8945,11 +8926,11 @@
         <f>AD14</f>
         <v>0.6</v>
       </c>
-      <c r="Z61" s="49"/>
+      <c r="Z61" s="38"/>
     </row>
     <row r="62" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="48"/>
-      <c r="B62" s="37"/>
+      <c r="B62" s="47"/>
       <c r="E62" s="14" t="s">
         <v>91</v>
       </c>
@@ -8979,11 +8960,11 @@
         <f>AD12</f>
         <v>0.36</v>
       </c>
-      <c r="Z62" s="49"/>
+      <c r="Z62" s="38"/>
     </row>
     <row r="63" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="48"/>
-      <c r="B63" s="37"/>
+      <c r="B63" s="47"/>
       <c r="E63" s="14" t="s">
         <v>92</v>
       </c>
@@ -9012,11 +8993,11 @@
         <f>AD11</f>
         <v>0.2</v>
       </c>
-      <c r="Z63" s="49"/>
+      <c r="Z63" s="38"/>
     </row>
     <row r="64" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="48"/>
-      <c r="B64" s="37"/>
+      <c r="B64" s="47"/>
       <c r="E64" s="14" t="s">
         <v>93</v>
       </c>
@@ -9044,7 +9025,7 @@
         <f>AD9</f>
         <v>0.12</v>
       </c>
-      <c r="Z64" s="49"/>
+      <c r="Z64" s="38"/>
     </row>
     <row r="65" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="E65" s="14" t="s">
@@ -9058,7 +9039,7 @@
       <c r="A67" s="48" t="s">
         <v>238</v>
       </c>
-      <c r="B67" s="37" t="s">
+      <c r="B67" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E67" s="14" t="s">
@@ -9092,11 +9073,11 @@
         <f>V67*(1- $F$29)+Y37*Y61</f>
         <v>113.66742611453597</v>
       </c>
-      <c r="Z67" s="49"/>
+      <c r="Z67" s="38"/>
     </row>
     <row r="68" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="48"/>
-      <c r="B68" s="37"/>
+      <c r="B68" s="47"/>
       <c r="E68" s="14" t="s">
         <v>110</v>
       </c>
@@ -9124,12 +9105,12 @@
         <f>V68*(1- $F$29)+Y38*Y62</f>
         <v>59.099305542412793</v>
       </c>
-      <c r="Z68" s="49"/>
+      <c r="Z68" s="38"/>
     </row>
     <row r="69" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="48"/>
-      <c r="B69" s="37"/>
-      <c r="D69" s="28"/>
+      <c r="B69" s="47"/>
+      <c r="D69" s="49"/>
       <c r="E69" s="14" t="s">
         <v>111</v>
       </c>
@@ -9153,12 +9134,12 @@
         <f>V69*(1- $F$29)+Y39*Y63</f>
         <v>34.91402943264</v>
       </c>
-      <c r="Z69" s="49"/>
+      <c r="Z69" s="38"/>
     </row>
     <row r="70" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="48"/>
-      <c r="B70" s="37"/>
-      <c r="D70" s="28"/>
+      <c r="B70" s="47"/>
+      <c r="D70" s="49"/>
       <c r="E70" s="14" t="s">
         <v>112</v>
       </c>
@@ -9182,17 +9163,17 @@
         <f>V70*(1- $F$29)+Y40*Y64</f>
         <v>7.7339817200000001</v>
       </c>
-      <c r="Z70" s="49"/>
+      <c r="Z70" s="38"/>
     </row>
     <row r="71" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="D71" s="28"/>
+      <c r="D71" s="49"/>
       <c r="E71" s="14"/>
     </row>
     <row r="72" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" s="48" t="s">
         <v>235</v>
       </c>
-      <c r="B72" s="37" t="s">
+      <c r="B72" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E72" s="14" t="s">
@@ -9225,11 +9206,11 @@
         <f>INT(X$4-$AF$6 &gt; $D80)*MAX(V95-$G$21*V37-Y42,0)</f>
         <v>30.582999999999998</v>
       </c>
-      <c r="Z72" s="49"/>
+      <c r="Z72" s="38"/>
     </row>
     <row r="73" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="48"/>
-      <c r="B73" s="37"/>
+      <c r="B73" s="47"/>
       <c r="E73" s="14" t="s">
         <v>128</v>
       </c>
@@ -9260,12 +9241,12 @@
         <f>INT(X$4-$AF$6 &gt; $D81)*MAX(V96-$G$21*V38-Y43,0)</f>
         <v>15.984000000000002</v>
       </c>
-      <c r="Z73" s="49"/>
+      <c r="Z73" s="38"/>
     </row>
     <row r="74" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="48"/>
-      <c r="B74" s="37"/>
-      <c r="D74" s="28" t="s">
+      <c r="B74" s="47"/>
+      <c r="D74" s="49" t="s">
         <v>152</v>
       </c>
       <c r="E74" s="14" t="s">
@@ -9298,12 +9279,12 @@
         <f>INT(X$4-$AF$6 &gt; $D82)*MAX(V97-$G$21*V39-Y44,0)</f>
         <v>7.3471236799999975</v>
       </c>
-      <c r="Z74" s="49"/>
+      <c r="Z74" s="38"/>
     </row>
     <row r="75" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="48"/>
-      <c r="B75" s="37"/>
-      <c r="D75" s="28"/>
+      <c r="B75" s="47"/>
+      <c r="D75" s="49"/>
       <c r="E75" s="14" t="s">
         <v>130</v>
       </c>
@@ -9334,16 +9315,16 @@
         <f>INT(X$4-$AF$6 &gt; $D83)*MAX(V98-$G$21*V40-Y45,0)</f>
         <v>0</v>
       </c>
-      <c r="Z75" s="49"/>
+      <c r="Z75" s="38"/>
     </row>
     <row r="76" spans="1:31" ht="17" x14ac:dyDescent="0.2">
-      <c r="A76" s="49" t="s">
+      <c r="A76" s="38" t="s">
         <v>236</v>
       </c>
-      <c r="B76" s="40" t="s">
+      <c r="B76" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="D76" s="28"/>
+      <c r="D76" s="49"/>
       <c r="E76" s="14" t="s">
         <v>147</v>
       </c>
@@ -9374,13 +9355,13 @@
         <f>SUM(Y72:Y75)</f>
         <v>53.914123679999996</v>
       </c>
-      <c r="Z76" s="49"/>
+      <c r="Z76" s="38"/>
       <c r="AE76" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="77" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="D77" s="28"/>
+      <c r="D77" s="49"/>
       <c r="E77" s="14"/>
       <c r="AC77" t="s">
         <v>85</v>
@@ -9393,7 +9374,7 @@
       <c r="A78" s="50" t="s">
         <v>237</v>
       </c>
-      <c r="B78" s="37" t="s">
+      <c r="B78" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E78" s="14" t="s">
@@ -9420,14 +9401,14 @@
       <c r="X78" s="4">
         <v>0</v>
       </c>
-      <c r="Z78" s="52"/>
+      <c r="Z78" s="39"/>
       <c r="AC78" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="79" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A79" s="50"/>
-      <c r="B79" s="37"/>
+      <c r="B79" s="47"/>
       <c r="E79" s="14" t="s">
         <v>148</v>
       </c>
@@ -9487,11 +9468,11 @@
         <f>IF(X79&gt;=X$131, IF(X78&lt;X$131, X$131-X78, 0),Y72)</f>
         <v>30.582999999999998</v>
       </c>
-      <c r="Z79" s="52"/>
+      <c r="Z79" s="39"/>
     </row>
     <row r="80" spans="1:31" ht="17" x14ac:dyDescent="0.2">
       <c r="A80" s="50"/>
-      <c r="B80" s="37"/>
+      <c r="B80" s="47"/>
       <c r="D80" s="22">
         <v>0</v>
       </c>
@@ -9554,11 +9535,11 @@
         <f>IF(X80&gt;=X$131, IF(X79&lt;X$131, X$131-X79, 0),Y73)</f>
         <v>15.984000000000002</v>
       </c>
-      <c r="Z80" s="52"/>
+      <c r="Z80" s="39"/>
     </row>
     <row r="81" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A81" s="50"/>
-      <c r="B81" s="37"/>
+      <c r="B81" s="47"/>
       <c r="D81" s="22">
         <v>1</v>
       </c>
@@ -9621,11 +9602,11 @@
         <f>IF(X81&gt;=X$131, IF(X80&lt;X$131, X$131-X80, 0),Y74)</f>
         <v>7.3471236799999957</v>
       </c>
-      <c r="Z81" s="52"/>
+      <c r="Z81" s="39"/>
     </row>
     <row r="82" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A82" s="50"/>
-      <c r="B82" s="37"/>
+      <c r="B82" s="47"/>
       <c r="D82" s="22">
         <v>2</v>
       </c>
@@ -9688,7 +9669,7 @@
         <f>IF(X82&gt;=X$131, IF(X81&lt;X$131, X$131-X81, 0),Y75)</f>
         <v>0</v>
       </c>
-      <c r="Z82" s="52"/>
+      <c r="Z82" s="39"/>
     </row>
     <row r="83" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D83" s="22">
@@ -9718,10 +9699,10 @@
       </c>
     </row>
     <row r="85" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A85" s="47" t="s">
+      <c r="A85" s="46" t="s">
         <v>181</v>
       </c>
-      <c r="B85" s="37" t="s">
+      <c r="B85" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E85" s="14" t="s">
@@ -9779,11 +9760,11 @@
         <f>Y61*X85</f>
         <v>0.5573184044275703</v>
       </c>
-      <c r="Z85" s="51"/>
+      <c r="Z85" s="37"/>
     </row>
     <row r="86" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A86" s="47"/>
-      <c r="B86" s="37"/>
+      <c r="A86" s="46"/>
+      <c r="B86" s="47"/>
       <c r="E86" s="14" t="s">
         <v>132</v>
       </c>
@@ -9839,11 +9820,11 @@
         <f>Y62</f>
         <v>0.36</v>
       </c>
-      <c r="Z86" s="51"/>
+      <c r="Z86" s="37"/>
     </row>
     <row r="87" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A87" s="47"/>
-      <c r="B87" s="37"/>
+      <c r="A87" s="46"/>
+      <c r="B87" s="47"/>
       <c r="E87" s="14" t="s">
         <v>133</v>
       </c>
@@ -9899,11 +9880,11 @@
         <f>Y63</f>
         <v>0.2</v>
       </c>
-      <c r="Z87" s="51"/>
+      <c r="Z87" s="37"/>
     </row>
     <row r="88" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A88" s="47"/>
-      <c r="B88" s="37"/>
+      <c r="A88" s="46"/>
+      <c r="B88" s="47"/>
       <c r="E88" s="14" t="s">
         <v>134</v>
       </c>
@@ -9959,16 +9940,16 @@
         <f>Y64</f>
         <v>0.12</v>
       </c>
-      <c r="Z88" s="51"/>
+      <c r="Z88" s="37"/>
     </row>
     <row r="89" spans="1:26" x14ac:dyDescent="0.2">
       <c r="E89" s="14"/>
     </row>
     <row r="90" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A90" s="47" t="s">
+      <c r="A90" s="46" t="s">
         <v>204</v>
       </c>
-      <c r="B90" s="37" t="s">
+      <c r="B90" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E90" s="14" t="s">
@@ -10002,11 +9983,11 @@
         <f>(V95-Y79-Y42)*$F$29</f>
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="Z90" s="51"/>
+      <c r="Z90" s="37"/>
     </row>
     <row r="91" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A91" s="47"/>
-      <c r="B91" s="37"/>
+      <c r="A91" s="46"/>
+      <c r="B91" s="47"/>
       <c r="E91" s="14" t="s">
         <v>206</v>
       </c>
@@ -10038,11 +10019,11 @@
         <f>(V96-Y80-Y43)*$F$29</f>
         <v>1.6E-2</v>
       </c>
-      <c r="Z91" s="51"/>
+      <c r="Z91" s="37"/>
     </row>
     <row r="92" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A92" s="47"/>
-      <c r="B92" s="37"/>
+      <c r="A92" s="46"/>
+      <c r="B92" s="47"/>
       <c r="E92" s="14" t="s">
         <v>207</v>
       </c>
@@ -10074,11 +10055,11 @@
         <f>(V97-Y81-Y44)*$F$29</f>
         <v>1.8400000000000007E-2</v>
       </c>
-      <c r="Z92" s="51"/>
+      <c r="Z92" s="37"/>
     </row>
     <row r="93" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A93" s="47"/>
-      <c r="B93" s="37"/>
+      <c r="A93" s="46"/>
+      <c r="B93" s="47"/>
       <c r="E93" s="14" t="s">
         <v>208</v>
       </c>
@@ -10110,16 +10091,16 @@
         <f>(V98-Y82-Y45)*$F$29</f>
         <v>5.1582799999999995E-3</v>
       </c>
-      <c r="Z93" s="51"/>
+      <c r="Z93" s="37"/>
     </row>
     <row r="94" spans="1:26" x14ac:dyDescent="0.2">
       <c r="E94" s="14"/>
     </row>
     <row r="95" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A95" s="47" t="s">
+      <c r="A95" s="46" t="s">
         <v>209</v>
       </c>
-      <c r="B95" s="37" t="s">
+      <c r="B95" s="47" t="s">
         <v>174</v>
       </c>
       <c r="E95" s="14" t="s">
@@ -10153,11 +10134,11 @@
         <f>V95 - Y79 - Y90 - Y42 + Y37*Y85</f>
         <v>55.855064376343478</v>
       </c>
-      <c r="Z95" s="51"/>
+      <c r="Z95" s="37"/>
     </row>
     <row r="96" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A96" s="47"/>
-      <c r="B96" s="37"/>
+      <c r="A96" s="46"/>
+      <c r="B96" s="47"/>
       <c r="E96" s="14" t="s">
         <v>71</v>
       </c>
@@ -10189,11 +10170,11 @@
         <f>V96 - Y80 - Y91 - Y43 + Y38*Y86</f>
         <v>36.783999999999999</v>
       </c>
-      <c r="Z96" s="51"/>
+      <c r="Z96" s="37"/>
     </row>
     <row r="97" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A97" s="47"/>
-      <c r="B97" s="37"/>
+      <c r="A97" s="46"/>
+      <c r="B97" s="47"/>
       <c r="E97" s="14" t="s">
         <v>72</v>
       </c>
@@ -10225,11 +10206,11 @@
         <f>V97 - Y81 - Y92 - Y44 + Y39*Y87</f>
         <v>27.581600000000005</v>
       </c>
-      <c r="Z97" s="51"/>
+      <c r="Z97" s="37"/>
     </row>
     <row r="98" spans="1:26" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="47"/>
-      <c r="B98" s="37"/>
+      <c r="A98" s="46"/>
+      <c r="B98" s="47"/>
       <c r="E98" s="14" t="s">
         <v>81</v>
       </c>
@@ -10261,20 +10242,20 @@
         <f>V98 - Y82 - Y93 - Y45 + Y40*Y88</f>
         <v>7.7339817200000001</v>
       </c>
-      <c r="Z98" s="51"/>
+      <c r="Z98" s="37"/>
     </row>
     <row r="99" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="D99" s="35"/>
+      <c r="D99" s="26"/>
       <c r="E99" s="14"/>
     </row>
     <row r="100" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A100" s="47" t="s">
+      <c r="A100" s="46" t="s">
         <v>210</v>
       </c>
-      <c r="B100" s="37" t="s">
+      <c r="B100" s="47" t="s">
         <v>174</v>
       </c>
-      <c r="D100" s="35"/>
+      <c r="D100" s="26"/>
       <c r="E100" s="14" t="s">
         <v>211</v>
       </c>
@@ -10306,12 +10287,12 @@
         <f>Y95*$G$20</f>
         <v>13.963766094085869</v>
       </c>
-      <c r="Z100" s="51"/>
+      <c r="Z100" s="37"/>
     </row>
     <row r="101" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A101" s="47"/>
-      <c r="B101" s="37"/>
-      <c r="D101" s="35"/>
+      <c r="A101" s="46"/>
+      <c r="B101" s="47"/>
+      <c r="D101" s="26"/>
       <c r="E101" s="14" t="s">
         <v>212</v>
       </c>
@@ -10343,12 +10324,12 @@
         <f t="shared" ref="Y101:Y103" si="15">Y96*$G$20</f>
         <v>9.1959999999999997</v>
       </c>
-      <c r="Z101" s="51"/>
+      <c r="Z101" s="37"/>
     </row>
     <row r="102" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A102" s="47"/>
-      <c r="B102" s="37"/>
-      <c r="D102" s="35"/>
+      <c r="A102" s="46"/>
+      <c r="B102" s="47"/>
+      <c r="D102" s="26"/>
       <c r="E102" s="14" t="s">
         <v>213</v>
       </c>
@@ -10380,12 +10361,12 @@
         <f>Y97*$G$20</f>
         <v>6.8954000000000013</v>
       </c>
-      <c r="Z102" s="51"/>
+      <c r="Z102" s="37"/>
     </row>
     <row r="103" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A103" s="47"/>
-      <c r="B103" s="37"/>
-      <c r="D103" s="35"/>
+      <c r="A103" s="46"/>
+      <c r="B103" s="47"/>
+      <c r="D103" s="26"/>
       <c r="E103" s="14" t="s">
         <v>214</v>
       </c>
@@ -10417,24 +10398,24 @@
         <f t="shared" si="15"/>
         <v>1.93349543</v>
       </c>
-      <c r="Z103" s="51"/>
+      <c r="Z103" s="37"/>
     </row>
     <row r="104" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A104" s="38"/>
-      <c r="B104" s="45"/>
-      <c r="D104" s="35"/>
+      <c r="A104" s="29"/>
+      <c r="B104" s="35"/>
+      <c r="D104" s="26"/>
       <c r="E104" s="14"/>
-      <c r="Z104" s="38"/>
+      <c r="Z104" s="29"/>
     </row>
     <row r="105" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A105" s="38"/>
-      <c r="B105" s="45"/>
-      <c r="D105" s="35"/>
+      <c r="A105" s="29"/>
+      <c r="B105" s="35"/>
+      <c r="D105" s="26"/>
       <c r="E105" s="14"/>
-      <c r="Z105" s="38"/>
+      <c r="Z105" s="29"/>
     </row>
     <row r="106" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="D106" s="35"/>
+      <c r="D106" s="26"/>
       <c r="E106" s="15" t="s">
         <v>140</v>
       </c>
@@ -10444,13 +10425,13 @@
       <c r="G106" s="8"/>
     </row>
     <row r="107" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A107" s="49" t="s">
+      <c r="A107" s="38" t="s">
         <v>239</v>
       </c>
-      <c r="B107" s="44" t="s">
+      <c r="B107" s="34" t="s">
         <v>182</v>
       </c>
-      <c r="D107" s="35"/>
+      <c r="D107" s="26"/>
       <c r="E107" s="14" t="s">
         <v>90</v>
       </c>
@@ -10510,13 +10491,13 @@
         <f>$G$28</f>
         <v>0.92</v>
       </c>
-      <c r="Z107" s="49"/>
+      <c r="Z107" s="38"/>
     </row>
     <row r="108" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A108" s="49" t="s">
+      <c r="A108" s="38" t="s">
         <v>240</v>
       </c>
-      <c r="B108" s="40" t="s">
+      <c r="B108" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E108" s="14" t="s">
@@ -10578,13 +10559,13 @@
         <f>Y7*$G$19</f>
         <v>24936000</v>
       </c>
-      <c r="Z108" s="49"/>
+      <c r="Z108" s="38"/>
     </row>
     <row r="109" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A109" s="49" t="s">
+      <c r="A109" s="38" t="s">
         <v>183</v>
       </c>
-      <c r="B109" s="40" t="s">
+      <c r="B109" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E109" s="14" t="s">
@@ -10644,13 +10625,13 @@
         <f>IF(V111=0,0,MIN(MAX((V111/V108-$F$16)/($F$18-$F$16), 0), 1))</f>
         <v>0.89478919993714923</v>
       </c>
-      <c r="Z109" s="49"/>
+      <c r="Z109" s="38"/>
     </row>
     <row r="110" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A110" s="49" t="s">
+      <c r="A110" s="38" t="s">
         <v>184</v>
       </c>
-      <c r="B110" s="43" t="s">
+      <c r="B110" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E110" s="14" t="s">
@@ -10712,13 +10693,13 @@
         <f>Y107*Y109</f>
         <v>0.82320606394217732</v>
       </c>
-      <c r="Z110" s="49"/>
+      <c r="Z110" s="38"/>
     </row>
     <row r="111" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A111" s="49" t="s">
+      <c r="A111" s="38" t="s">
         <v>241</v>
       </c>
-      <c r="B111" s="43" t="s">
+      <c r="B111" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E111" s="14" t="s">
@@ -10780,13 +10761,13 @@
         <f>V111 - V132 - V120 - V143 + Y110*Y7</f>
         <v>3187373.6439100648</v>
       </c>
-      <c r="Z111" s="49"/>
+      <c r="Z111" s="38"/>
     </row>
     <row r="112" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A112" s="49" t="s">
+      <c r="A112" s="38" t="s">
         <v>244</v>
       </c>
-      <c r="B112" s="43" t="s">
+      <c r="B112" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E112" s="14" t="s">
@@ -10848,13 +10829,13 @@
         <f>Y111/Y7</f>
         <v>12.782217051291566</v>
       </c>
-      <c r="Z112" s="49"/>
+      <c r="Z112" s="38"/>
     </row>
     <row r="113" spans="1:26" ht="34" x14ac:dyDescent="0.2">
-      <c r="A113" s="49" t="s">
+      <c r="A113" s="38" t="s">
         <v>282</v>
       </c>
-      <c r="B113" s="40" t="s">
+      <c r="B113" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E113" s="10" t="s">
@@ -10916,7 +10897,7 @@
         <f>MAX(Y112-$G21,0)</f>
         <v>12.682217051291566</v>
       </c>
-      <c r="Z113" s="49"/>
+      <c r="Z113" s="38"/>
     </row>
     <row r="114" spans="1:26" x14ac:dyDescent="0.2">
       <c r="E114" s="13"/>
@@ -10941,10 +10922,10 @@
       <c r="Y115" s="12"/>
     </row>
     <row r="116" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A116" s="49" t="s">
+      <c r="A116" s="38" t="s">
         <v>246</v>
       </c>
-      <c r="B116" s="44" t="s">
+      <c r="B116" s="34" t="s">
         <v>182</v>
       </c>
       <c r="E116" s="10" t="s">
@@ -11006,13 +10987,13 @@
         <f>Y112*Y7</f>
         <v>3187373.6439100648</v>
       </c>
-      <c r="Z116" s="49"/>
+      <c r="Z116" s="38"/>
     </row>
     <row r="117" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A117" s="49" t="s">
+      <c r="A117" s="38" t="s">
         <v>245</v>
       </c>
-      <c r="B117" s="43" t="s">
+      <c r="B117" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E117" s="10" t="s">
@@ -11046,13 +11027,13 @@
         <f>SUM(Y95:Y98)</f>
         <v>127.95464609634348</v>
       </c>
-      <c r="Z117" s="49"/>
+      <c r="Z117" s="38"/>
     </row>
     <row r="118" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A118" s="49" t="s">
+      <c r="A118" s="38" t="s">
         <v>242</v>
       </c>
-      <c r="B118" s="43" t="s">
+      <c r="B118" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E118" s="10" t="s">
@@ -11114,13 +11095,13 @@
         <f>Y116+Y117</f>
         <v>3187501.5985561614</v>
       </c>
-      <c r="Z118" s="49"/>
+      <c r="Z118" s="38"/>
     </row>
     <row r="119" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A119" s="49" t="s">
+      <c r="A119" s="38" t="s">
         <v>243</v>
       </c>
-      <c r="B119" s="43" t="s">
+      <c r="B119" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E119" s="10" t="s">
@@ -11182,13 +11163,13 @@
         <f>Y111*$G$20</f>
         <v>796843.41097751621</v>
       </c>
-      <c r="Z119" s="49"/>
+      <c r="Z119" s="38"/>
     </row>
     <row r="120" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A120" s="49" t="s">
+      <c r="A120" s="38" t="s">
         <v>281</v>
       </c>
-      <c r="B120" s="40" t="s">
+      <c r="B120" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E120" s="10" t="s">
@@ -11250,13 +11231,13 @@
         <f>Y9*Y112</f>
         <v>1482.7371779498217</v>
       </c>
-      <c r="Z120" s="49"/>
+      <c r="Z120" s="38"/>
     </row>
     <row r="121" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A121" s="49" t="s">
+      <c r="A121" s="38" t="s">
         <v>265</v>
       </c>
-      <c r="B121" s="40" t="s">
+      <c r="B121" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E121" s="10" t="s">
@@ -11318,13 +11299,13 @@
         <f>MIN(Y120,Y9*Y15)</f>
         <v>1044</v>
       </c>
-      <c r="Z121" s="49"/>
+      <c r="Z121" s="38"/>
     </row>
     <row r="122" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A122" s="49" t="s">
+      <c r="A122" s="38" t="s">
         <v>283</v>
       </c>
-      <c r="B122" s="40" t="s">
+      <c r="B122" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E122" s="10" t="s">
@@ -11386,13 +11367,13 @@
         <f>(Y120-Y121+Y53)*$F$14</f>
         <v>307.11602456487515</v>
       </c>
-      <c r="Z122" s="49"/>
+      <c r="Z122" s="38"/>
     </row>
     <row r="123" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A123" s="49" t="s">
+      <c r="A123" s="38" t="s">
         <v>258</v>
       </c>
-      <c r="B123" s="43" t="s">
+      <c r="B123" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E123" s="14" t="s">
@@ -11426,13 +11407,13 @@
         <f>MIN(X122+Y122, X32)</f>
         <v>5839.4603133048031</v>
       </c>
-      <c r="Z123" s="49"/>
+      <c r="Z123" s="38"/>
     </row>
     <row r="124" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A124" s="49" t="s">
+      <c r="A124" s="38" t="s">
         <v>259</v>
       </c>
-      <c r="B124" s="40" t="s">
+      <c r="B124" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E124" s="14" t="s">
@@ -11494,13 +11475,13 @@
         <f>Y122/(X122+Y122)</f>
         <v>5.2593220620942092E-2</v>
       </c>
-      <c r="Z124" s="49"/>
+      <c r="Z124" s="38"/>
     </row>
     <row r="125" spans="1:26" ht="34" x14ac:dyDescent="0.2">
-      <c r="A125" s="49" t="s">
+      <c r="A125" s="38" t="s">
         <v>185</v>
       </c>
-      <c r="B125" s="40" t="s">
+      <c r="B125" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E125" s="10" t="s">
@@ -11562,7 +11543,7 @@
         <f>MAX(Y13-Y26, 0)*Y113</f>
         <v>2533196.7626931826</v>
       </c>
-      <c r="Z125" s="49"/>
+      <c r="Z125" s="38"/>
     </row>
     <row r="127" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="E127" s="15" t="s">
@@ -11584,10 +11565,10 @@
       <c r="Y127" s="8"/>
     </row>
     <row r="128" spans="1:26" ht="17" x14ac:dyDescent="0.2">
-      <c r="A128" s="49" t="s">
+      <c r="A128" s="38" t="s">
         <v>260</v>
       </c>
-      <c r="B128" s="40" t="s">
+      <c r="B128" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E128" s="14" t="s">
@@ -11621,13 +11602,13 @@
         <f>MAX(X32-X123,0)</f>
         <v>2514160.5396866952</v>
       </c>
-      <c r="Z128" s="49"/>
+      <c r="Z128" s="38"/>
     </row>
     <row r="129" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A129" s="49" t="s">
+      <c r="A129" s="38" t="s">
         <v>261</v>
       </c>
-      <c r="B129" s="40" t="s">
+      <c r="B129" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E129" s="10" t="s">
@@ -11661,13 +11642,13 @@
         <f>MIN(X139,X128)</f>
         <v>1789059.8013981958</v>
       </c>
-      <c r="Z129" s="49"/>
+      <c r="Z129" s="38"/>
     </row>
     <row r="130" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A130" s="49" t="s">
+      <c r="A130" s="38" t="s">
         <v>272</v>
       </c>
-      <c r="B130" s="40" t="s">
+      <c r="B130" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E130" s="10" t="s">
@@ -11701,13 +11682,13 @@
         <f>X128-X129</f>
         <v>725100.73828849941</v>
       </c>
-      <c r="Z130" s="49"/>
+      <c r="Z130" s="38"/>
     </row>
     <row r="131" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A131" s="49" t="s">
+      <c r="A131" s="38" t="s">
         <v>216</v>
       </c>
-      <c r="B131" s="40" t="s">
+      <c r="B131" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E131" s="10" t="s">
@@ -11741,13 +11722,13 @@
         <f>MIN(X130,Y76)</f>
         <v>53.914123679999996</v>
       </c>
-      <c r="Z131" s="49"/>
+      <c r="Z131" s="38"/>
     </row>
     <row r="132" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A132" s="49" t="s">
+      <c r="A132" s="38" t="s">
         <v>268</v>
       </c>
-      <c r="B132" s="40" t="s">
+      <c r="B132" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E132" s="10" t="s">
@@ -11809,13 +11790,13 @@
         <f>Y140*X129</f>
         <v>1595269.5105861374</v>
       </c>
-      <c r="Z132" s="49"/>
+      <c r="Z132" s="38"/>
     </row>
     <row r="133" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A133" s="49" t="s">
+      <c r="A133" s="38" t="s">
         <v>273</v>
       </c>
-      <c r="B133" s="43" t="s">
+      <c r="B133" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E133" s="10" t="s">
@@ -11877,7 +11858,7 @@
         <f>Y132+X131</f>
         <v>1595323.4247098174</v>
       </c>
-      <c r="Z133" s="49"/>
+      <c r="Z133" s="38"/>
     </row>
     <row r="134" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="E134" s="15" t="s">
@@ -11899,10 +11880,10 @@
       <c r="Y134" s="8"/>
     </row>
     <row r="135" spans="1:29" ht="34" x14ac:dyDescent="0.2">
-      <c r="A135" s="49" t="s">
+      <c r="A135" s="38" t="s">
         <v>276</v>
       </c>
-      <c r="B135" s="40" t="s">
+      <c r="B135" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E135" s="10" t="s">
@@ -11964,7 +11945,7 @@
         <f>Y113/$G$22</f>
         <v>0.12694911963254821</v>
       </c>
-      <c r="Z135" s="49"/>
+      <c r="Z135" s="38"/>
       <c r="AA135">
         <v>0.5</v>
       </c>
@@ -11977,10 +11958,10 @@
       </c>
     </row>
     <row r="136" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A136" s="49" t="s">
+      <c r="A136" s="38" t="s">
         <v>186</v>
       </c>
-      <c r="B136" s="40" t="s">
+      <c r="B136" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E136" s="10" t="s">
@@ -12042,7 +12023,7 @@
         <f>MAX(MIN((Y135-$F$16)/$F$17, 1), 0)</f>
         <v>0.629745598162741</v>
       </c>
-      <c r="Z136" s="49"/>
+      <c r="Z136" s="38"/>
       <c r="AA136">
         <v>0.3</v>
       </c>
@@ -12055,8 +12036,8 @@
       </c>
     </row>
     <row r="137" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A137" s="49"/>
-      <c r="Z137" s="49"/>
+      <c r="A137" s="38"/>
+      <c r="Z137" s="38"/>
       <c r="AA137">
         <v>0.2</v>
       </c>
@@ -12069,10 +12050,10 @@
       </c>
     </row>
     <row r="138" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A138" s="49" t="s">
+      <c r="A138" s="38" t="s">
         <v>188</v>
       </c>
-      <c r="B138" s="40" t="s">
+      <c r="B138" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E138" s="10" t="s">
@@ -12134,7 +12115,7 @@
         <f>Y125*Y136</f>
         <v>1595269.5105861374</v>
       </c>
-      <c r="Z138" s="49"/>
+      <c r="Z138" s="38"/>
       <c r="AA138">
         <v>0.125</v>
       </c>
@@ -12147,10 +12128,10 @@
       </c>
     </row>
     <row r="139" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A139" s="49" t="s">
+      <c r="A139" s="38" t="s">
         <v>189</v>
       </c>
-      <c r="B139" s="40" t="s">
+      <c r="B139" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E139" s="10" t="s">
@@ -12212,13 +12193,13 @@
         <f>X139</f>
         <v>1789059.8013981958</v>
       </c>
-      <c r="Z139" s="49"/>
+      <c r="Z139" s="38"/>
     </row>
     <row r="140" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A140" s="49" t="s">
+      <c r="A140" s="38" t="s">
         <v>190</v>
       </c>
-      <c r="B140" s="40" t="s">
+      <c r="B140" s="28" t="s">
         <v>174</v>
       </c>
       <c r="E140" s="10" t="s">
@@ -12280,7 +12261,7 @@
         <f>Y138/Y139</f>
         <v>0.89168037275187428</v>
       </c>
-      <c r="Z140" s="49"/>
+      <c r="Z140" s="38"/>
     </row>
     <row r="142" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="E142" s="15" t="s">
@@ -12302,10 +12283,10 @@
       <c r="Y142" s="8"/>
     </row>
     <row r="143" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A143" s="49" t="s">
+      <c r="A143" s="38" t="s">
         <v>274</v>
       </c>
-      <c r="B143" s="43" t="s">
+      <c r="B143" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E143" s="10" t="s">
@@ -12367,13 +12348,13 @@
         <f>(Y111 - Y132 - Y120)*$G$29+SUM(Y90:Y93)</f>
         <v>3181.2993505719551</v>
       </c>
-      <c r="Z143" s="49"/>
+      <c r="Z143" s="38"/>
     </row>
     <row r="144" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A144" s="49" t="s">
+      <c r="A144" s="38" t="s">
         <v>275</v>
       </c>
-      <c r="B144" s="43" t="s">
+      <c r="B144" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E144" s="14" t="s">
@@ -12435,13 +12416,13 @@
         <f>(Y132+X131)*$G20</f>
         <v>398830.85617745435</v>
       </c>
-      <c r="Z144" s="49"/>
+      <c r="Z144" s="38"/>
     </row>
     <row r="145" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A145" s="49" t="s">
+      <c r="A145" s="38" t="s">
         <v>176</v>
       </c>
-      <c r="B145" s="43" t="s">
+      <c r="B145" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E145" s="10" t="s">
@@ -12503,13 +12484,13 @@
         <f>Y120-X123*Y124-Y121+Y53</f>
         <v>131.62115338494641</v>
       </c>
-      <c r="Z145" s="49"/>
+      <c r="Z145" s="38"/>
     </row>
     <row r="146" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A146" s="49" t="s">
+      <c r="A146" s="38" t="s">
         <v>177</v>
       </c>
-      <c r="B146" s="43" t="s">
+      <c r="B146" s="33" t="s">
         <v>163</v>
       </c>
       <c r="E146" s="10" t="s">
@@ -12571,10 +12552,10 @@
         <f>(Y120+Y53)*$G20</f>
         <v>370.68429448745542</v>
       </c>
-      <c r="Z146" s="49"/>
+      <c r="Z146" s="38"/>
     </row>
     <row r="149" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A149" s="33" t="s">
+      <c r="A149" s="24" t="s">
         <v>267</v>
       </c>
       <c r="F149" s="4">
@@ -12635,10 +12616,10 @@
       </c>
     </row>
     <row r="151" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A151" s="49" t="s">
+      <c r="A151" s="38" t="s">
         <v>277</v>
       </c>
-      <c r="B151" s="43" t="s">
+      <c r="B151" s="33" t="s">
         <v>163</v>
       </c>
       <c r="F151" s="4">
@@ -12669,7 +12650,7 @@
         <f>X123+X132+Y132</f>
         <v>1794899.2617115006</v>
       </c>
-      <c r="Z151" s="49"/>
+      <c r="Z151" s="38"/>
     </row>
     <row r="152" spans="1:29" x14ac:dyDescent="0.2">
       <c r="F152" s="4">
@@ -12739,37 +12720,6 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="A100:A103"/>
-    <mergeCell ref="B100:B103"/>
-    <mergeCell ref="A48:A51"/>
-    <mergeCell ref="B48:B51"/>
-    <mergeCell ref="D48:D51"/>
-    <mergeCell ref="A78:A82"/>
-    <mergeCell ref="B78:B82"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A61:A64"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="B85:B88"/>
-    <mergeCell ref="A95:A98"/>
-    <mergeCell ref="B95:B98"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B37:B40"/>
-    <mergeCell ref="A37:A40"/>
-    <mergeCell ref="B61:B64"/>
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="A72:A75"/>
-    <mergeCell ref="B72:B75"/>
-    <mergeCell ref="A85:A88"/>
-    <mergeCell ref="AD4:AF4"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="L5:M5"/>
     <mergeCell ref="D17:D18"/>
     <mergeCell ref="D69:D71"/>
     <mergeCell ref="D74:D77"/>
@@ -12778,6 +12728,37 @@
     <mergeCell ref="R5:S5"/>
     <mergeCell ref="U5:V5"/>
     <mergeCell ref="F5:G5"/>
+    <mergeCell ref="AD4:AF4"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B37:B40"/>
+    <mergeCell ref="A37:A40"/>
+    <mergeCell ref="B61:B64"/>
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A61:A64"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="A100:A103"/>
+    <mergeCell ref="B100:B103"/>
+    <mergeCell ref="A48:A51"/>
+    <mergeCell ref="B48:B51"/>
+    <mergeCell ref="D48:D51"/>
+    <mergeCell ref="A78:A82"/>
+    <mergeCell ref="B78:B82"/>
+    <mergeCell ref="B85:B88"/>
+    <mergeCell ref="A95:A98"/>
+    <mergeCell ref="B95:B98"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A72:A75"/>
+    <mergeCell ref="B72:B75"/>
+    <mergeCell ref="A85:A88"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated BCL to allow for forest-specific buffer zone (in py and excel) and updated additional variable retrieval functions for BCL setup
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75A060D-8C3C-5A4B-A9D3-F7AC49307262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB018337-E483-704D-B091-748AC3E41FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2520" yWindow="760" windowWidth="33680" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="260" yWindow="760" windowWidth="33680" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="301">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -944,6 +944,9 @@
   </si>
   <si>
     <t>k_{heav}</t>
+  </si>
+  <si>
+    <t>rrr</t>
   </si>
 </sst>
 </file>
@@ -7314,6 +7317,9 @@
       <c r="F16" s="4">
         <v>1E-3</v>
       </c>
+      <c r="G16" s="4">
+        <v>1E-3</v>
+      </c>
       <c r="Z16" s="38" t="s">
         <v>293</v>
       </c>
@@ -7344,6 +7350,9 @@
       <c r="F17" s="4">
         <v>0.2</v>
       </c>
+      <c r="G17" s="4">
+        <v>0.2</v>
+      </c>
       <c r="Z17" s="38" t="s">
         <v>294</v>
       </c>
@@ -7454,7 +7463,7 @@
         <v>0.15</v>
       </c>
       <c r="G21" s="4">
-        <f>G$19*$F$16</f>
+        <f>G$19*$G$16</f>
         <v>0.1</v>
       </c>
       <c r="Z21" s="38"/>
@@ -10582,7 +10591,7 @@
         <v>1</v>
       </c>
       <c r="J109" s="4">
-        <f>IF(G111=0,0,MIN(MAX((G111/G108-$F$16)/($F$18-$F$16), 0), 1))</f>
+        <f>IF(G111=0,0,MIN(MAX((G111/G108-$G$16)/($F$18-$G$16), 0), 1))</f>
         <v>1</v>
       </c>
       <c r="L109" s="4">
@@ -10590,7 +10599,7 @@
         <v>1</v>
       </c>
       <c r="M109" s="4">
-        <f>IF(J111=0,0,MIN(MAX((J111/J108-$F$16)/($F$18-$F$16), 0), 1))</f>
+        <f>IF(J111=0,0,MIN(MAX((J111/J108-$G$16)/($F$18-$G$16), 0), 1))</f>
         <v>1</v>
       </c>
       <c r="O109" s="4">
@@ -10598,7 +10607,7 @@
         <v>1</v>
       </c>
       <c r="P109" s="4">
-        <f>IF(M111=0,0,MIN(MAX((M111/M108-$F$16)/($F$18-$F$16), 0), 1))</f>
+        <f>IF(M111=0,0,MIN(MAX((M111/M108-$G$16)/($F$18-$G$16), 0), 1))</f>
         <v>1</v>
       </c>
       <c r="R109" s="4">
@@ -10606,7 +10615,7 @@
         <v>1</v>
       </c>
       <c r="S109" s="4">
-        <f>IF(P111=0,0,MIN(MAX((P111/P108-$F$16)/($F$18-$F$16), 0), 1))</f>
+        <f>IF(P111=0,0,MIN(MAX((P111/P108-$G$16)/($F$18-$G$16), 0), 1))</f>
         <v>1</v>
       </c>
       <c r="U109" s="4">
@@ -10614,7 +10623,7 @@
         <v>1</v>
       </c>
       <c r="V109" s="4">
-        <f>IF(S111=0,0,MIN(MAX((S111/S108-$F$16)/($F$18-$F$16), 0), 1))</f>
+        <f>IF(S111=0,0,MIN(MAX((S111/S108-$G$16)/($F$18-$G$16), 0), 1))</f>
         <v>1</v>
       </c>
       <c r="X109" s="4">
@@ -10622,10 +10631,12 @@
         <v>1</v>
       </c>
       <c r="Y109" s="4">
-        <f>IF(V111=0,0,MIN(MAX((V111/V108-$F$16)/($F$18-$F$16), 0), 1))</f>
+        <f>IF(V111=0,0,MIN(MAX((V111/V108-$G$16)/($F$18-$G$16), 0), 1))</f>
         <v>0.89478919993714923</v>
       </c>
-      <c r="Z109" s="38"/>
+      <c r="Z109" s="38" t="s">
+        <v>300</v>
+      </c>
     </row>
     <row r="110" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A110" s="38" t="s">
@@ -11972,7 +11983,7 @@
         <v>1</v>
       </c>
       <c r="G136" s="4">
-        <f>MAX(MIN((G135-$F$16)/$F$17, 1), 0)</f>
+        <f>MAX(MIN((G135-$G$16)/$G$17, 1), 0)</f>
         <v>1</v>
       </c>
       <c r="I136" s="4">
@@ -11980,7 +11991,7 @@
         <v>1</v>
       </c>
       <c r="J136" s="4">
-        <f>MAX(MIN((J135-$F$16)/$F$17, 1), 0)</f>
+        <f>MAX(MIN((J135-$G$16)/$G$17, 1), 0)</f>
         <v>1</v>
       </c>
       <c r="L136" s="4">
@@ -11988,7 +11999,7 @@
         <v>1</v>
       </c>
       <c r="M136" s="4">
-        <f>MAX(MIN((M135-$F$16)/$F$17, 1), 0)</f>
+        <f>MAX(MIN((M135-$G$16)/$G$17, 1), 0)</f>
         <v>1</v>
       </c>
       <c r="O136" s="4">
@@ -11996,7 +12007,7 @@
         <v>1</v>
       </c>
       <c r="P136" s="4">
-        <f>MAX(MIN((P135-$F$16)/$F$17, 1), 0)</f>
+        <f>MAX(MIN((P135-$G$16)/$G$17, 1), 0)</f>
         <v>1</v>
       </c>
       <c r="R136" s="4">
@@ -12004,7 +12015,7 @@
         <v>1</v>
       </c>
       <c r="S136" s="4">
-        <f>MAX(MIN((S135-$F$16)/$F$17, 1), 0)</f>
+        <f>MAX(MIN((S135-$G$16)/$G$17, 1), 0)</f>
         <v>1</v>
       </c>
       <c r="U136" s="4">
@@ -12012,7 +12023,7 @@
         <v>1</v>
       </c>
       <c r="V136" s="4">
-        <f>MAX(MIN((V135-$F$16)/$F$17, 1), 0)</f>
+        <f>MAX(MIN((V135-$G$16)/$G$17, 1), 0)</f>
         <v>1</v>
       </c>
       <c r="X136" s="4">
@@ -12020,7 +12031,7 @@
         <v>1</v>
       </c>
       <c r="Y136" s="4">
-        <f>MAX(MIN((Y135-$F$16)/$F$17, 1), 0)</f>
+        <f>MAX(MIN((Y135-$G$16)/$G$17, 1), 0)</f>
         <v>0.629745598162741</v>
       </c>
       <c r="Z136" s="38"/>

</xml_diff>

<commit_message>
updated below-ground biomass carbon emissions to account for preserved stock in converted class (based on conversion target classes)
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB018337-E483-704D-B091-748AC3E41FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD09B239-9DD4-0540-ADDC-8B25C9444167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="260" yWindow="760" windowWidth="33680" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="620" yWindow="500" windowWidth="37780" windowHeight="19040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7436,7 +7436,7 @@
         <v>173</v>
       </c>
       <c r="F20" s="4">
-        <v>0.3</v>
+        <v>0.21</v>
       </c>
       <c r="G20" s="4">
         <v>0.25</v>
@@ -11120,7 +11120,7 @@
       </c>
       <c r="F119" s="4">
         <f>F111*$F$20</f>
-        <v>450000</v>
+        <v>315000</v>
       </c>
       <c r="G119" s="4">
         <f>G111*$G$20</f>
@@ -11128,7 +11128,7 @@
       </c>
       <c r="I119" s="4">
         <f>I111*$F$20</f>
-        <v>426426.94265947182</v>
+        <v>298498.85986163025</v>
       </c>
       <c r="J119" s="4">
         <f>J111*$G$20</f>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="L119" s="4">
         <f>L111*$F$20</f>
-        <v>401729.40564975084</v>
+        <v>281210.58395482559</v>
       </c>
       <c r="M119" s="4">
         <f>M111*$G$20</f>
@@ -11144,7 +11144,7 @@
       </c>
       <c r="O119" s="4">
         <f>O111*$F$20</f>
-        <v>378689.78824255464</v>
+        <v>265082.85176978825</v>
       </c>
       <c r="P119" s="4">
         <f>P111*$G$20</f>
@@ -11152,7 +11152,7 @@
       </c>
       <c r="R119" s="4">
         <f>R111*$F$20</f>
-        <v>356485.31955472904</v>
+        <v>249539.7236883103</v>
       </c>
       <c r="S119" s="4">
         <f>S111*$G$20</f>
@@ -11160,7 +11160,7 @@
       </c>
       <c r="U119" s="4">
         <f>U111*$F$20</f>
-        <v>329374.48540307593</v>
+        <v>230562.13978215316</v>
       </c>
       <c r="V119" s="4">
         <f>V111*$G$20</f>
@@ -11168,7 +11168,7 @@
       </c>
       <c r="X119" s="4">
         <f>X111*$F$20</f>
-        <v>245972.17525771659</v>
+        <v>172180.5226804016</v>
       </c>
       <c r="Y119" s="4">
         <f>Y111*$G$20</f>
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F144" s="4">
         <f>F132*$F20</f>
-        <v>21365.788918364884</v>
+        <v>14956.05224285542</v>
       </c>
       <c r="G144" s="4">
         <f>(G132+F131)*$G20</f>
@@ -12381,7 +12381,7 @@
       </c>
       <c r="I144" s="4">
         <f>I132*$F20</f>
-        <v>22127.038759307754</v>
+        <v>15488.927131515427</v>
       </c>
       <c r="J144" s="4">
         <f>(J132+I131)*$G20</f>
@@ -12389,7 +12389,7 @@
       </c>
       <c r="L144" s="4">
         <f>L132*$F20</f>
-        <v>20810.770497264373</v>
+        <v>14567.539348085062</v>
       </c>
       <c r="M144" s="4">
         <f>(M132+L131)*$G20</f>
@@ -12397,7 +12397,7 @@
       </c>
       <c r="O144" s="4">
         <f>O132*$F20</f>
-        <v>19673.557629791878</v>
+        <v>13771.490340854314</v>
       </c>
       <c r="P144" s="4">
         <f>(P132+O131)*$G20</f>
@@ -12405,7 +12405,7 @@
       </c>
       <c r="R144" s="4">
         <f>R132*$F20</f>
-        <v>23669.393807170058</v>
+        <v>16568.575665019041</v>
       </c>
       <c r="S144" s="4">
         <f>(S132+R131)*$G20</f>
@@ -12413,7 +12413,7 @@
       </c>
       <c r="U144" s="4">
         <f>U132*$F20</f>
-        <v>80430.204256942568</v>
+        <v>56301.142979859804</v>
       </c>
       <c r="V144" s="4">
         <f>(V132+U131)*$G20</f>
@@ -12421,7 +12421,7 @@
       </c>
       <c r="X144" s="4">
         <f>X132*$F20</f>
-        <v>58137.087243617476</v>
+        <v>40695.961070532234</v>
       </c>
       <c r="Y144" s="4">
         <f>(Y132+X131)*$G20</f>
@@ -12508,60 +12508,60 @@
         <v>167</v>
       </c>
       <c r="F146" s="4">
-        <f>F120*$F20</f>
+        <f>(F120 - F121)*$F20</f>
+        <v>1522.5</v>
+      </c>
+      <c r="G146" s="4">
+        <f>(G120-G121+G53)*$G20</f>
         <v>2250</v>
       </c>
-      <c r="G146" s="4">
-        <f>(G120+G53)*$G20</f>
-        <v>2500</v>
-      </c>
       <c r="I146" s="4">
-        <f>I120*$F20</f>
-        <v>2657.1327080288697</v>
+        <f>(I120 - I121)*$F20</f>
+        <v>1793.5908956202086</v>
       </c>
       <c r="J146" s="4">
-        <f>(J120+J53)*$G20</f>
-        <v>2559.2229710466122</v>
+        <f>(J120-J121+J53)*$G20</f>
+        <v>2289.7229710466122</v>
       </c>
       <c r="L146" s="4">
-        <f>L120*$F20</f>
-        <v>2356.4224845960307</v>
+        <f>(L120 - L121)*$F20</f>
+        <v>1586.1597392172214</v>
       </c>
       <c r="M146" s="4">
-        <f>(M120+M53)*$G20</f>
-        <v>2019.8305166694299</v>
+        <f>(M120-M121+M53)*$G20</f>
+        <v>1789.53051666943</v>
       </c>
       <c r="O146" s="4">
-        <f>O120*$F20</f>
-        <v>2696.6719406896059</v>
+        <f>(O120 - O121)*$F20</f>
+        <v>1818.580358482724</v>
       </c>
       <c r="P146" s="4">
-        <f>(P120+P53)*$G20</f>
-        <v>3772.0021262214559</v>
+        <f>(P120-P121+P53)*$G20</f>
+        <v>3296.8021262214561</v>
       </c>
       <c r="R146" s="4">
-        <f>R120*$F20</f>
-        <v>3652.513520027961</v>
+        <f>(R120 - R121)*$F20</f>
+        <v>2447.5594640195727</v>
       </c>
       <c r="S146" s="4">
-        <f>(S120+S53)*$G20</f>
-        <v>690.59087551194818</v>
+        <f>(S120-S121+S53)*$G20</f>
+        <v>592.11587551194816</v>
       </c>
       <c r="U146" s="4">
-        <f>U120*$F20</f>
-        <v>3341.4802866978721</v>
+        <f>(U120 - U121)*$F20</f>
+        <v>2254.6582006885105</v>
       </c>
       <c r="V146" s="4">
-        <f>(V120+V53)*$G20</f>
-        <v>1573.9866837396262</v>
+        <f>(V120-V121+V53)*$G20</f>
+        <v>1285.2366837396262</v>
       </c>
       <c r="X146" s="4">
-        <f>X120*$F20</f>
-        <v>2520.9446951742548</v>
+        <f>(X120 - X121)*$F20</f>
+        <v>1659.7032866219784</v>
       </c>
       <c r="Y146" s="4">
-        <f>(Y120+Y53)*$G20</f>
-        <v>370.68429448745542</v>
+        <f>(Y120-Y121+Y53)*$G20</f>
+        <v>109.68429448745542</v>
       </c>
       <c r="Z146" s="38"/>
     </row>

</xml_diff>

<commit_message>
minor updates to ledger
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD09B239-9DD4-0540-ADDC-8B25C9444167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A80088C-E4B0-914A-82C9-BC19D659508B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="620" yWindow="500" windowWidth="37780" windowHeight="19040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="6860" yWindow="760" windowWidth="33680" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added some output variables to carbon ledger for tracking biomass growth and updated available output variables in FRST. Started building variable extraction and conversion in AFOLU
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F350A9A-DF78-DF44-80EF-AAEC8D1A81A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8C1182-B23A-DD4C-B000-5DF68ADA57A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="760" windowWidth="23640" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="240" yWindow="760" windowWidth="23640" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="303">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -950,6 +950,9 @@
   </si>
   <si>
     <t>arr_biomass_c_average_bg_stock_in_conversion_targets</t>
+  </si>
+  <si>
+    <t>arr_biomass_c_total_growth</t>
   </si>
 </sst>
 </file>
@@ -6395,7 +6398,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40F0562-A765-A442-B9DB-CF71D123E451}">
-  <dimension ref="A1:AN160"/>
+  <dimension ref="A1:AN161"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="62.1640625" style="24" customWidth="1"/>
@@ -12204,7 +12207,7 @@
         <v>0.125</v>
       </c>
       <c r="AB139">
-        <f>SUM(AA$6:AA157)</f>
+        <f>SUM(AA$6:AA158)</f>
         <v>1.125</v>
       </c>
       <c r="AC139">
@@ -12638,153 +12641,206 @@
       </c>
       <c r="Z147" s="38"/>
     </row>
-    <row r="150" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A150" s="24" t="s">
+    <row r="148" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A148" s="38" t="s">
+        <v>302</v>
+      </c>
+      <c r="B148" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="F148" s="4">
+        <f>I111*I7*(1+$F21)</f>
+        <v>3880.5</v>
+      </c>
+      <c r="G148" s="4">
+        <f>(J111*J7+SUMPRODUCT(G38:G41,G86:G89))*(1+$G21)</f>
+        <v>287385</v>
+      </c>
+      <c r="I148" s="4">
+        <f>L111*L7*(1+$F21)</f>
+        <v>3856.32</v>
+      </c>
+      <c r="J148" s="4">
+        <f>(M111*M7+SUMPRODUCT(J38:J41,J86:J89))*(1+$G21)</f>
+        <v>287259.5625</v>
+      </c>
+      <c r="L148" s="4">
+        <f>O111*O7*(1+$F21)</f>
+        <v>3833.7000000000003</v>
+      </c>
+      <c r="M148" s="4">
+        <f>(P111*P7+SUMPRODUCT(M38:M41,M86:M89))*(1+$G21)</f>
+        <v>287156.71250000002</v>
+      </c>
+      <c r="O148" s="4">
+        <f>R111*R7*(1+$F21)</f>
+        <v>3806.4</v>
+      </c>
+      <c r="P148" s="4">
+        <f>(S111*S7+SUMPRODUCT(P38:P41,P86:P89))*(1+$G21)</f>
+        <v>286948.5</v>
+      </c>
+      <c r="R148" s="4">
+        <f>U111*U7*(1+$F21)</f>
+        <v>3767.4</v>
+      </c>
+      <c r="S148" s="4">
+        <f>(V111*V7+SUMPRODUCT(S38:S41,S86:S89))*(1+$G21)</f>
+        <v>286924.28750000003</v>
+      </c>
+      <c r="U148" s="4">
+        <f>X111*X7*(1+$F21)</f>
+        <v>3327.4969606347436</v>
+      </c>
+      <c r="V148" s="4">
+        <f>(Y111*Y7+SUMPRODUCT(V38:V41,V86:V89))*(1+$G21)</f>
+        <v>243889.44739455794</v>
+      </c>
+      <c r="X148" s="4">
+        <f>AA111*AA7*(1+$F21)</f>
+        <v>0</v>
+      </c>
+      <c r="Y148" s="4">
+        <f>(AB111*AB7+SUMPRODUCT(Y38:Y41,Y86:Y89))*(1+$G21)</f>
+        <v>129.19999999999999</v>
+      </c>
+      <c r="Z148" s="38"/>
+    </row>
+    <row r="151" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A151" s="24" t="s">
         <v>267</v>
       </c>
-      <c r="F150" s="4">
+      <c r="F151" s="4">
         <f>F146+F122</f>
         <v>2425</v>
       </c>
-      <c r="G150" s="4">
+      <c r="G151" s="4">
         <f>G146+G122</f>
         <v>3700</v>
       </c>
-      <c r="I150" s="4">
+      <c r="I151" s="4">
         <f>I146+I122</f>
         <v>2838.8826284504194</v>
       </c>
-      <c r="J150" s="4">
+      <c r="J151" s="4">
         <f>J146+J122</f>
         <v>3791.9939124902994</v>
       </c>
-      <c r="L150" s="4">
+      <c r="L151" s="4">
         <f>L146+L122</f>
         <v>2492.7872894169086</v>
       </c>
-      <c r="M150" s="4">
+      <c r="M151" s="4">
         <f>M146+M122</f>
         <v>3013.8800374053144</v>
       </c>
-      <c r="O150" s="4">
+      <c r="O151" s="4">
         <f>O146+O122</f>
         <v>2742.4739452429521</v>
       </c>
-      <c r="P150" s="4">
+      <c r="P151" s="4">
         <f>P146+P122</f>
         <v>5703.0215606406946</v>
       </c>
-      <c r="R150" s="4">
+      <c r="R151" s="4">
         <f>R146+R122</f>
         <v>3536.5429221318309</v>
       </c>
-      <c r="S150" s="4">
+      <c r="S151" s="4">
         <f>S146+S122</f>
         <v>1067.0339396766713</v>
       </c>
-      <c r="U150" s="4">
+      <c r="U151" s="4">
         <f>U146+U122</f>
         <v>3074.7284826043051</v>
       </c>
-      <c r="V150" s="4">
+      <c r="V151" s="4">
         <f>V146+V122</f>
         <v>2781.2436955233939</v>
       </c>
-      <c r="X150" s="4">
+      <c r="X151" s="4">
         <f>X146+X122</f>
         <v>3021.989935081745</v>
       </c>
-      <c r="Y150" s="4">
+      <c r="Y151" s="4">
         <f>Y146+Y122</f>
         <v>2878.3021373837346</v>
       </c>
     </row>
-    <row r="152" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A152" s="38" t="s">
+    <row r="153" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A153" s="38" t="s">
         <v>277</v>
       </c>
-      <c r="B152" s="33" t="s">
+      <c r="B153" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="F152" s="4">
+      <c r="F153" s="4">
         <f>F124+F133+G133+F132</f>
         <v>2000000</v>
       </c>
-      <c r="I152" s="4">
+      <c r="I153" s="4">
         <f>I124+I133+J133</f>
         <v>2050000</v>
       </c>
-      <c r="L152" s="4">
+      <c r="L153" s="4">
         <f>L124+L133+M133</f>
         <v>2110000.0000000005</v>
       </c>
-      <c r="O152" s="4">
+      <c r="O153" s="4">
         <f>O124+O133+P133</f>
         <v>2210000</v>
       </c>
-      <c r="R152" s="4">
+      <c r="R153" s="4">
         <f>R124+R133+S133</f>
         <v>1374131.5531552718</v>
       </c>
-      <c r="U152" s="4">
+      <c r="U153" s="4">
         <f>U124+U133+V133</f>
         <v>259692.40809697201</v>
       </c>
-      <c r="X152" s="4">
+      <c r="X153" s="4">
         <f>X124+X133+Y133</f>
         <v>91488.01273416965</v>
       </c>
-      <c r="Z152" s="38"/>
-    </row>
-    <row r="153" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="F153" s="4">
-        <f>F152/F33</f>
+      <c r="Z153" s="38"/>
+    </row>
+    <row r="154" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="F154" s="4">
+        <f>F153/F33</f>
         <v>1</v>
       </c>
-      <c r="I153" s="4">
-        <f>I152/I33</f>
+      <c r="I154" s="4">
+        <f>I153/I33</f>
         <v>1</v>
       </c>
-      <c r="L153" s="4">
-        <f>L152/L33</f>
+      <c r="L154" s="4">
+        <f>L153/L33</f>
         <v>1.0000000000000002</v>
       </c>
-      <c r="O153" s="4">
-        <f>O152/O33</f>
+      <c r="O154" s="4">
+        <f>O153/O33</f>
         <v>1</v>
       </c>
-      <c r="R153" s="4">
-        <f>R152/R33</f>
+      <c r="R154" s="4">
+        <f>R153/R33</f>
         <v>0.45804385105175727</v>
       </c>
-      <c r="U153" s="4">
-        <f>U152/U33</f>
+      <c r="U154" s="4">
+        <f>U153/U33</f>
         <v>1.038769632387888E-2</v>
       </c>
-      <c r="X153" s="4">
-        <f>X152/X33</f>
+      <c r="X154" s="4">
+        <f>X153/X33</f>
         <v>3.6304766958003831E-2</v>
-      </c>
-    </row>
-    <row r="158" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="AA158">
-        <v>0.1225</v>
-      </c>
-      <c r="AB158">
-        <f>SUM(AA$6:AA158)</f>
-        <v>1.2475000000000001</v>
-      </c>
-      <c r="AC158">
-        <v>20</v>
       </c>
     </row>
     <row r="159" spans="1:29" x14ac:dyDescent="0.2">
       <c r="AA159">
-        <v>0.12239999999999999</v>
+        <v>0.1225</v>
       </c>
       <c r="AB159">
         <f>SUM(AA$6:AA159)</f>
-        <v>1.3699000000000001</v>
+        <v>1.2475000000000001</v>
       </c>
       <c r="AC159">
         <v>20</v>
@@ -12792,13 +12848,25 @@
     </row>
     <row r="160" spans="1:29" x14ac:dyDescent="0.2">
       <c r="AA160">
-        <v>0.12230000000000001</v>
+        <v>0.12239999999999999</v>
       </c>
       <c r="AB160">
         <f>SUM(AA$6:AA160)</f>
+        <v>1.3699000000000001</v>
+      </c>
+      <c r="AC160">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="161" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA161">
+        <v>0.12230000000000001</v>
+      </c>
+      <c r="AB161">
+        <f>SUM(AA$6:AA161)</f>
         <v>1.4922000000000002</v>
       </c>
-      <c r="AC160">
+      <c r="AC161">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed some issues with units conversion in sequestration and added below-ground biomass loss to decompostion
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8C1182-B23A-DD4C-B000-5DF68ADA57A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8405E880-F68F-1F45-BDD6-B68CBF1F15C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="760" windowWidth="23640" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="780" yWindow="760" windowWidth="33780" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="cl_1" sheetId="2" r:id="rId2"/>
     <sheet name="cl_2" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="304">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -953,6 +954,9 @@
   </si>
   <si>
     <t>arr_biomass_c_total_growth</t>
+  </si>
+  <si>
+    <t>arr_biomass_c_bg_lost_decomposition</t>
   </si>
 </sst>
 </file>
@@ -6398,7 +6402,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40F0562-A765-A442-B9DB-CF71D123E451}">
-  <dimension ref="A1:AN161"/>
+  <dimension ref="A1:AN162"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="62.1640625" style="24" customWidth="1"/>
@@ -7848,12 +7852,12 @@
         <v>171</v>
       </c>
       <c r="F30" s="4">
-        <f>0.01327547</f>
-        <v>1.3275469999999999E-2</v>
+        <f>0.00157</f>
+        <v>1.57E-3</v>
       </c>
       <c r="G30" s="4">
         <f>F30</f>
-        <v>1.3275469999999999E-2</v>
+        <v>1.57E-3</v>
       </c>
       <c r="I30" s="4">
         <f>F29/F20</f>
@@ -9140,23 +9144,23 @@
       </c>
       <c r="M68" s="4">
         <f>J68*(1- $F$30)+M38*M62</f>
-        <v>5.0887158504999999</v>
+        <v>5.0986655000000001</v>
       </c>
       <c r="P68" s="4">
         <f>M68*(1- $F$30)+P38*P62</f>
-        <v>15.221160755888162</v>
+        <v>15.290660595165001</v>
       </c>
       <c r="S68" s="4">
         <f>P68*(1- $F$30)+S38*S62</f>
-        <v>32.019092692908188</v>
+        <v>32.266654258030592</v>
       </c>
       <c r="V68" s="4">
         <f>S68*(1- $F$30)+V38*V62</f>
-        <v>62.194024188436266</v>
+        <v>62.815995610845476</v>
       </c>
       <c r="Y68" s="4">
         <f>V68*(1- $F$30)+Y38*Y62</f>
-        <v>112.36836928614341</v>
+        <v>113.71737449773644</v>
       </c>
       <c r="Z68" s="38"/>
     </row>
@@ -9176,19 +9180,19 @@
       </c>
       <c r="P69" s="4">
         <f>M69*(1- $F$30)+P39*P63</f>
-        <v>4.7893796240000004</v>
+        <v>4.7987440000000001</v>
       </c>
       <c r="S69" s="4">
         <f>P69*(1- $F$30)+S39*S63</f>
-        <v>14.325798358482977</v>
+        <v>14.39120997192</v>
       </c>
       <c r="V69" s="4">
         <f>S69*(1- $F$30)+V39*V63</f>
-        <v>30.13561665214889</v>
+        <v>30.368615772264086</v>
       </c>
       <c r="Y69" s="4">
         <f>V69*(1- $F$30)+Y39*Y63</f>
-        <v>58.535552177351789</v>
+        <v>59.120937045501634</v>
       </c>
       <c r="Z69" s="38"/>
     </row>
@@ -9209,15 +9213,15 @@
       </c>
       <c r="S70" s="4">
         <f>P70*(1- $F$30)+S40*S64</f>
-        <v>5.5077865676000002</v>
+        <v>5.5185556000000009</v>
       </c>
       <c r="V70" s="4">
         <f>S70*(1- $F$30)+V40*V64</f>
-        <v>16.474668112255422</v>
+        <v>16.549891467708001</v>
       </c>
       <c r="Y70" s="4">
         <f>V70*(1- $F$30)+Y40*Y64</f>
-        <v>34.655959149971224</v>
+        <v>34.923908138103698</v>
       </c>
       <c r="Z70" s="38"/>
     </row>
@@ -9242,11 +9246,11 @@
       </c>
       <c r="V71" s="4">
         <f>S71*(1- $F$30)+V41*V65</f>
-        <v>2.5742915478999997</v>
+        <v>2.5793249</v>
       </c>
       <c r="Y71" s="4">
         <f>V71*(1- $F$30)+Y41*Y65</f>
-        <v>7.7001166176845999</v>
+        <v>7.7352753599069999</v>
       </c>
       <c r="Z71" s="38"/>
     </row>
@@ -10050,23 +10054,23 @@
       </c>
       <c r="M91" s="4">
         <f>(J96-M80-M43)*$F$30</f>
-        <v>1.1284149499999998E-2</v>
+        <v>1.3345E-3</v>
       </c>
       <c r="P91" s="4">
         <f>(M96-P80-P43)*$F$30</f>
-        <v>6.755509461183723E-2</v>
+        <v>8.0049048349999999E-3</v>
       </c>
       <c r="S91" s="4">
         <f>(P96-S80-S43)*$F$30</f>
-        <v>0.2020680629799706</v>
+        <v>2.4006337134409049E-2</v>
       </c>
       <c r="V91" s="4">
         <f>(S96-V80-V43)*$F$30</f>
-        <v>0.42506850447192185</v>
+        <v>5.0658647185108027E-2</v>
       </c>
       <c r="Y91" s="4">
         <f>(V96-Y80-Y43)*$F$30</f>
-        <v>0.82565490229285987</v>
+        <v>9.8621113109027395E-2</v>
       </c>
       <c r="Z91" s="37"/>
     </row>
@@ -10090,19 +10094,19 @@
       </c>
       <c r="P92" s="4">
         <f>(M97-P81-P44)*$F$30</f>
-        <v>1.0620376000000001E-2</v>
+        <v>1.2560000000000002E-3</v>
       </c>
       <c r="S92" s="4">
         <f>(P97-S81-S44)*$F$30</f>
-        <v>6.3581265517023283E-2</v>
+        <v>7.5340280800000005E-3</v>
       </c>
       <c r="V92" s="4">
         <f>(S97-V81-V44)*$F$30</f>
-        <v>0.19018170633409001</v>
+        <v>2.2594199655914398E-2</v>
       </c>
       <c r="Y92" s="4">
         <f>(V97-Y81-Y44)*$F$30</f>
-        <v>0.40006447479710294</v>
+        <v>4.7678726762454618E-2</v>
       </c>
       <c r="Z92" s="37"/>
     </row>
@@ -10130,15 +10134,15 @@
       </c>
       <c r="S93" s="4">
         <f>(P98-S82-S45)*$F$30</f>
-        <v>1.22134324E-2</v>
+        <v>1.4444E-3</v>
       </c>
       <c r="V93" s="4">
         <f>(S98-V82-V45)*$F$30</f>
-        <v>7.3118455344576769E-2</v>
+        <v>8.664132292000002E-3</v>
       </c>
       <c r="Y93" s="4">
         <f>(V98-Y82-Y45)*$F$30</f>
-        <v>0.21870896228420347</v>
+        <v>2.5983329604301563E-2</v>
       </c>
       <c r="Z93" s="37"/>
     </row>
@@ -10170,11 +10174,11 @@
       </c>
       <c r="V94" s="4">
         <f>(S99-V83-V46)*$F$30</f>
-        <v>5.7084520999999997E-3</v>
+        <v>6.7509999999999998E-4</v>
       </c>
       <c r="Y94" s="4">
         <f>(V99-Y83-Y46)*$F$30</f>
-        <v>3.417493021540001E-2</v>
+        <v>4.049540093E-3</v>
       </c>
       <c r="Z94" s="37"/>
     </row>
@@ -10201,23 +10205,23 @@
       </c>
       <c r="M96" s="4">
         <f>J96 - M80 - M91 - M43 + M38*M86</f>
-        <v>5.0887158504999999</v>
+        <v>5.0986655000000001</v>
       </c>
       <c r="P96" s="4">
         <f>M96 - P80 - P91 - P43 + P38*P86</f>
-        <v>15.221160755888162</v>
+        <v>15.290660595164999</v>
       </c>
       <c r="S96" s="4">
         <f>P96 - S80 - S91 - S43 + S38*S86</f>
-        <v>32.019092692908188</v>
+        <v>32.266654258030592</v>
       </c>
       <c r="V96" s="4">
         <f>S96 - V80 - V91 - V43 + V38*V86</f>
-        <v>62.194024188436259</v>
+        <v>62.815995610845476</v>
       </c>
       <c r="Y96" s="4">
         <f>V96 - Y80 - Y91 - Y43 + Y38*Y86</f>
-        <v>112.36836928614341</v>
+        <v>113.71737449773644</v>
       </c>
       <c r="Z96" s="37"/>
     </row>
@@ -10241,19 +10245,19 @@
       </c>
       <c r="P97" s="4">
         <f>M97 - P81 - P92 - P44 + P39*P87</f>
-        <v>4.7893796240000004</v>
+        <v>4.7987440000000001</v>
       </c>
       <c r="S97" s="4">
         <f>P97 - S81 - S92 - S44 + S39*S87</f>
-        <v>14.325798358482977</v>
+        <v>14.391209971919999</v>
       </c>
       <c r="V97" s="4">
         <f>S97 - V81 - V92 - V44 + V39*V87</f>
-        <v>30.135616652148887</v>
+        <v>30.368615772264086</v>
       </c>
       <c r="Y97" s="4">
         <f>V97 - Y81 - Y92 - Y44 + Y39*Y87</f>
-        <v>58.535552177351782</v>
+        <v>59.120937045501627</v>
       </c>
       <c r="Z97" s="37"/>
     </row>
@@ -10281,15 +10285,15 @@
       </c>
       <c r="S98" s="4">
         <f>P98 - S82 - S93 - S45 + S40*S88</f>
-        <v>5.5077865676000002</v>
+        <v>5.5185556000000009</v>
       </c>
       <c r="V98" s="4">
         <f>S98 - V82 - V93 - V45 + V40*V88</f>
-        <v>16.474668112255422</v>
+        <v>16.549891467708001</v>
       </c>
       <c r="Y98" s="4">
         <f>V98 - Y82 - Y93 - Y45 + Y40*Y88</f>
-        <v>34.655959149971224</v>
+        <v>34.923908138103698</v>
       </c>
       <c r="Z98" s="37"/>
     </row>
@@ -10321,11 +10325,11 @@
       </c>
       <c r="V99" s="4">
         <f>S99 - V83 - V94 - V46 + V41*V89</f>
-        <v>2.5742915478999997</v>
+        <v>2.5793249</v>
       </c>
       <c r="Y99" s="4">
         <f>V99 - Y83 - Y94 - Y46 + Y41*Y89</f>
-        <v>7.7001166176845999</v>
+        <v>7.7352753599069999</v>
       </c>
       <c r="Z99" s="37"/>
     </row>
@@ -10354,23 +10358,23 @@
       </c>
       <c r="M101" s="4">
         <f>M96*$G$21</f>
-        <v>1.272178962625</v>
+        <v>1.274666375</v>
       </c>
       <c r="P101" s="4">
         <f>P96*$G$21</f>
-        <v>3.8052901889720405</v>
+        <v>3.8226651487912497</v>
       </c>
       <c r="S101" s="4">
         <f>S96*$G$21</f>
-        <v>8.0047731732270471</v>
+        <v>8.0666635645076479</v>
       </c>
       <c r="V101" s="4">
         <f>V96*$G$21</f>
-        <v>15.548506047109065</v>
+        <v>15.703998902711369</v>
       </c>
       <c r="Y101" s="4">
         <f>Y96*$G$21</f>
-        <v>28.092092321535851</v>
+        <v>28.429343624434111</v>
       </c>
       <c r="Z101" s="37"/>
     </row>
@@ -10395,19 +10399,19 @@
       </c>
       <c r="P102" s="4">
         <f t="shared" ref="P102:P104" si="12">P97*$G$21</f>
-        <v>1.1973449060000001</v>
+        <v>1.199686</v>
       </c>
       <c r="S102" s="4">
         <f t="shared" ref="S102:S104" si="13">S97*$G$21</f>
-        <v>3.5814495896207443</v>
+        <v>3.5978024929799997</v>
       </c>
       <c r="V102" s="4">
         <f t="shared" ref="V102:V104" si="14">V97*$G$21</f>
-        <v>7.5339041630372217</v>
+        <v>7.5921539430660214</v>
       </c>
       <c r="Y102" s="4">
         <f t="shared" ref="Y102:Y104" si="15">Y97*$G$21</f>
-        <v>14.633888044337946</v>
+        <v>14.780234261375407</v>
       </c>
       <c r="Z102" s="37"/>
     </row>
@@ -10436,15 +10440,15 @@
       </c>
       <c r="S103" s="4">
         <f>S98*$G$21</f>
-        <v>1.3769466419</v>
+        <v>1.3796389000000002</v>
       </c>
       <c r="V103" s="4">
         <f>V98*$G$21</f>
-        <v>4.1186670280638555</v>
+        <v>4.1374728669270002</v>
       </c>
       <c r="Y103" s="4">
         <f>Y98*$G$21</f>
-        <v>8.663989787492806</v>
+        <v>8.7309770345259246</v>
       </c>
       <c r="Z103" s="37"/>
     </row>
@@ -10477,11 +10481,11 @@
       </c>
       <c r="V104" s="4">
         <f t="shared" si="14"/>
-        <v>0.64357288697499992</v>
+        <v>0.64483122500000001</v>
       </c>
       <c r="Y104" s="4">
         <f t="shared" si="15"/>
-        <v>1.92502915442115</v>
+        <v>1.93381883997675</v>
       </c>
       <c r="Z104" s="37"/>
     </row>
@@ -10704,11 +10708,11 @@
       </c>
       <c r="X110" s="4">
         <f>IF(U112=0,0,MIN(MAX((U112/U109-$F$17)/($F$19-$F$17), 0), 1))</f>
-        <v>0.89228649746988453</v>
+        <v>0.96349966843506474</v>
       </c>
       <c r="Y110" s="4">
         <f>IF(V112=0,0,MIN(MAX((V112/V109-$G$17)/($F$19-$G$17), 0), 1))</f>
-        <v>0.85022774788522248</v>
+        <v>0.86560925711218095</v>
       </c>
       <c r="Z110" s="38" t="s">
         <v>300</v>
@@ -10774,11 +10778,11 @@
       </c>
       <c r="X111" s="4">
         <f xml:space="preserve"> X108*X110</f>
-        <v>0.26768594924096534</v>
+        <v>0.28904990053051943</v>
       </c>
       <c r="Y111" s="4">
         <f>Y108*Y110</f>
-        <v>0.78220952805440469</v>
+        <v>0.7963605165432065</v>
       </c>
       <c r="Z111" s="38"/>
     </row>
@@ -10802,51 +10806,51 @@
       </c>
       <c r="I112" s="4">
         <f>F112 - F133 - F121 - F144+I111*I7</f>
-        <v>1400244.5781226705</v>
+        <v>1416820.2074666857</v>
       </c>
       <c r="J112" s="4">
         <f>G112 - G133 - G121 - G144 + J111*J7</f>
-        <v>23001355.719131082</v>
+        <v>23271492.408783317</v>
       </c>
       <c r="L112" s="4">
         <f>I112 - I133 - I121 - I144+L111*L7</f>
-        <v>1296616.445847953</v>
+        <v>1328540.482773518</v>
       </c>
       <c r="M112" s="4">
         <f>J112 - J133 - J121 - J144 + M111*M7</f>
-        <v>20984486.203669269</v>
+        <v>21500316.163346589</v>
       </c>
       <c r="O112" s="4">
         <f>L112 - L133 - L121 - L144+O111*O7</f>
-        <v>1175936.6610351533</v>
+        <v>1229960.5227370157</v>
       </c>
       <c r="P112" s="4">
         <f>M112 - M133 - M121 - M144 + P111*P7</f>
-        <v>18954620.865377408</v>
+        <v>19683424.583337996</v>
       </c>
       <c r="R112" s="4">
         <f>O112 - O133 - O121 - O144+R111*R7</f>
-        <v>1032133.964000222</v>
+        <v>1102712.6301399493</v>
       </c>
       <c r="S112" s="4">
         <f>P112 - P133 - P121 - P144 + S111*S7</f>
-        <v>16874657.962828044</v>
+        <v>17795064.508199312</v>
       </c>
       <c r="U112" s="4">
         <f>R112 - R133 - R121 - R144+U111*U7</f>
-        <v>917853.92999855743</v>
+        <v>952878.26623738057</v>
       </c>
       <c r="V112" s="4">
         <f>S112 - S133 - S121 - S144 + V111*V7</f>
-        <v>15623190.666785505</v>
+        <v>15735231.967631815</v>
       </c>
       <c r="X112" s="4">
         <f>U112 - U133 - U121 - U144+X111*X7</f>
-        <v>869078.45031468186</v>
+        <v>902055.81293937785</v>
       </c>
       <c r="Y112" s="4">
         <f>V112 - V133 - V121 - V144 + Y111*Y7</f>
-        <v>15387963.591322072</v>
+        <v>15603395.572368858</v>
       </c>
       <c r="Z112" s="38"/>
     </row>
@@ -10870,51 +10874,51 @@
       </c>
       <c r="I113" s="4">
         <f>I112/I7</f>
-        <v>140.72809830378597</v>
+        <v>142.39399070016941</v>
       </c>
       <c r="J113" s="4">
         <f>J112/J7</f>
-        <v>92.042239772433305</v>
+        <v>93.12321892270235</v>
       </c>
       <c r="L113" s="4">
         <f>L112/L7</f>
-        <v>131.13030398947745</v>
+        <v>134.35886759440919</v>
       </c>
       <c r="M113" s="4">
         <f>M112/M7</f>
-        <v>84.008511964727447</v>
+        <v>86.073566449203682</v>
       </c>
       <c r="O113" s="4">
         <f>O112/O7</f>
-        <v>119.62733072585486</v>
+        <v>125.12314575147667</v>
       </c>
       <c r="P113" s="4">
         <f>P112/P7</f>
-        <v>75.910790983345379</v>
+        <v>78.82955507231992</v>
       </c>
       <c r="R113" s="4">
         <f>R112/R7</f>
-        <v>105.75143073772767</v>
+        <v>112.98285144876529</v>
       </c>
       <c r="S113" s="4">
         <f>S112/S7</f>
-        <v>67.63281535698043</v>
+        <v>71.321760405441637</v>
       </c>
       <c r="U113" s="4">
         <f>U112/U7</f>
-        <v>95.015934782459368</v>
+        <v>98.641642467637737</v>
       </c>
       <c r="V113" s="4">
         <f>V112/V7</f>
-        <v>62.62678398486964</v>
+        <v>63.075910318609083</v>
       </c>
       <c r="X113" s="4">
         <f>X112/X7</f>
-        <v>90.888773302100176</v>
+        <v>94.337566716103098</v>
       </c>
       <c r="Y113" s="4">
         <f>Y112/Y7</f>
-        <v>61.709831534015365</v>
+        <v>62.573771143603061</v>
       </c>
       <c r="Z113" s="38"/>
     </row>
@@ -10938,51 +10942,51 @@
       </c>
       <c r="I114" s="4">
         <f>MAX(I113-$F22,0)</f>
-        <v>91.141540803785972</v>
+        <v>92.807433200169413</v>
       </c>
       <c r="J114" s="4">
         <f>MAX(J113-$G22,0)</f>
-        <v>54.241346772433303</v>
+        <v>55.322325922702348</v>
       </c>
       <c r="L114" s="4">
         <f>MAX(L113-$F22,0)</f>
-        <v>81.543746489477456</v>
+        <v>84.772310094409193</v>
       </c>
       <c r="M114" s="4">
         <f>MAX(M113-$G22,0)</f>
-        <v>46.207618964727445</v>
+        <v>48.27267344920368</v>
       </c>
       <c r="O114" s="4">
         <f>MAX(O113-$F22,0)</f>
-        <v>70.040773225854863</v>
+        <v>75.536588251476672</v>
       </c>
       <c r="P114" s="4">
         <f>MAX(P113-$G22,0)</f>
-        <v>38.109897983345377</v>
+        <v>41.028662072319918</v>
       </c>
       <c r="R114" s="4">
         <f>MAX(R113-$F22,0)</f>
-        <v>56.164873237727676</v>
+        <v>63.39629394876529</v>
       </c>
       <c r="S114" s="4">
         <f>MAX(S113-$G22,0)</f>
-        <v>29.831922356980428</v>
+        <v>33.520867405441635</v>
       </c>
       <c r="U114" s="4">
         <f>MAX(U113-$F22,0)</f>
-        <v>45.42937728245937</v>
+        <v>49.05508496763774</v>
       </c>
       <c r="V114" s="4">
         <f>MAX(V113-$G22,0)</f>
-        <v>24.825890984869638</v>
+        <v>25.275017318609081</v>
       </c>
       <c r="X114" s="4">
         <f>MAX(X113-$F22,0)</f>
-        <v>41.302215802100179</v>
+        <v>44.7510092161031</v>
       </c>
       <c r="Y114" s="4">
         <f>MAX(Y113-$G22,0)</f>
-        <v>23.908938534015363</v>
+        <v>24.772878143603059</v>
       </c>
       <c r="Z114" s="38"/>
     </row>
@@ -11028,51 +11032,51 @@
       </c>
       <c r="I117" s="4">
         <f>I113*I7</f>
-        <v>1400244.5781226703</v>
+        <v>1416820.2074666857</v>
       </c>
       <c r="J117" s="4">
         <f>J113*J7</f>
-        <v>23001355.719131082</v>
+        <v>23271492.408783317</v>
       </c>
       <c r="L117" s="4">
         <f>L113*L7</f>
-        <v>1296616.445847953</v>
+        <v>1328540.4827735182</v>
       </c>
       <c r="M117" s="4">
         <f>M113*M7</f>
-        <v>20984486.203669269</v>
+        <v>21500316.163346589</v>
       </c>
       <c r="O117" s="4">
         <f>O113*O7</f>
-        <v>1175936.6610351533</v>
+        <v>1229960.5227370157</v>
       </c>
       <c r="P117" s="4">
         <f>P113*P7</f>
-        <v>18954620.865377408</v>
+        <v>19683424.583337996</v>
       </c>
       <c r="R117" s="4">
         <f>R113*R7</f>
-        <v>1032133.964000222</v>
+        <v>1102712.6301399493</v>
       </c>
       <c r="S117" s="4">
         <f>S113*S7</f>
-        <v>16874657.962828044</v>
+        <v>17795064.508199312</v>
       </c>
       <c r="U117" s="4">
         <f>U113*U7</f>
-        <v>917853.92999855755</v>
+        <v>952878.26623738057</v>
       </c>
       <c r="V117" s="4">
         <f>V113*V7</f>
-        <v>15623190.666785505</v>
+        <v>15735231.967631815</v>
       </c>
       <c r="X117" s="4">
         <f>X113*X7</f>
-        <v>869078.45031468186</v>
+        <v>902055.81293937785</v>
       </c>
       <c r="Y117" s="4">
         <f>Y113*Y7</f>
-        <v>15387963.591322072</v>
+        <v>15603395.572368858</v>
       </c>
       <c r="Z117" s="38"/>
     </row>
@@ -11096,23 +11100,23 @@
       </c>
       <c r="M118" s="4">
         <f>SUM(M96:M99)</f>
-        <v>5.8887158504999997</v>
+        <v>5.8986654999999999</v>
       </c>
       <c r="P118" s="4">
         <f>SUM(P96:P99)</f>
-        <v>20.930540379888164</v>
+        <v>21.009404595165002</v>
       </c>
       <c r="S118" s="4">
         <f>SUM(S96:S99)</f>
-        <v>52.282677618991166</v>
+        <v>52.606419829950589</v>
       </c>
       <c r="V118" s="4">
         <f>SUM(V96:V99)</f>
-        <v>111.37860050074056</v>
+        <v>112.31382775081757</v>
       </c>
       <c r="Y118" s="4">
         <f>SUM(Y96:Y99)</f>
-        <v>213.25999723115103</v>
+        <v>215.49749504124878</v>
       </c>
       <c r="Z118" s="38"/>
     </row>
@@ -11136,51 +11140,51 @@
       </c>
       <c r="I119" s="4">
         <f>I117+I118</f>
-        <v>1400244.5781226703</v>
+        <v>1416820.2074666857</v>
       </c>
       <c r="J119" s="4">
         <f>J117+J118</f>
-        <v>23001356.569131084</v>
+        <v>23271493.258783318</v>
       </c>
       <c r="L119" s="4">
         <f>L117+L118</f>
-        <v>1296616.445847953</v>
+        <v>1328540.4827735182</v>
       </c>
       <c r="M119" s="4">
         <f>M117+M118</f>
-        <v>20984492.092385121</v>
+        <v>21500322.062012088</v>
       </c>
       <c r="O119" s="4">
         <f>O117+O118</f>
-        <v>1175936.6610351533</v>
+        <v>1229960.5227370157</v>
       </c>
       <c r="P119" s="4">
         <f>P117+P118</f>
-        <v>18954641.795917787</v>
+        <v>19683445.592742592</v>
       </c>
       <c r="R119" s="4">
         <f>R117+R118</f>
-        <v>1032133.964000222</v>
+        <v>1102712.6301399493</v>
       </c>
       <c r="S119" s="4">
         <f>S117+S118</f>
-        <v>16874710.245505664</v>
+        <v>17795117.114619143</v>
       </c>
       <c r="U119" s="4">
         <f>U117+U118</f>
-        <v>917853.92999855755</v>
+        <v>952878.26623738057</v>
       </c>
       <c r="V119" s="4">
         <f>V117+V118</f>
-        <v>15623302.045386005</v>
+        <v>15735344.281459566</v>
       </c>
       <c r="X119" s="4">
         <f>X117+X118</f>
-        <v>869078.45031468186</v>
+        <v>902055.81293937785</v>
       </c>
       <c r="Y119" s="4">
         <f>Y117+Y118</f>
-        <v>15388176.851319304</v>
+        <v>15603611.069863901</v>
       </c>
       <c r="Z119" s="38"/>
     </row>
@@ -11195,60 +11199,60 @@
         <v>220</v>
       </c>
       <c r="F120" s="4">
-        <f>F112*$F$21</f>
+        <f>F119*$F$21</f>
         <v>450000</v>
       </c>
       <c r="G120" s="4">
-        <f>G112*$G$21</f>
+        <f>G119*$G$21</f>
         <v>6250000</v>
       </c>
       <c r="I120" s="4">
-        <f>I112*$F$21</f>
-        <v>420073.37343680114</v>
+        <f>I119*$F$21</f>
+        <v>425046.0622400057</v>
       </c>
       <c r="J120" s="4">
-        <f>J112*$G$21</f>
-        <v>5750338.9297827706</v>
+        <f>J119*$G$21</f>
+        <v>5817873.3146958295</v>
       </c>
       <c r="L120" s="4">
-        <f>L112*$F$21</f>
-        <v>388984.93375438586</v>
+        <f>L119*$F$21</f>
+        <v>398562.14483205543</v>
       </c>
       <c r="M120" s="4">
-        <f>M112*$G$21</f>
-        <v>5246121.5509173172</v>
+        <f>M119*$G$21</f>
+        <v>5375080.5155030219</v>
       </c>
       <c r="O120" s="4">
-        <f>O112*$F$21</f>
-        <v>352780.99831054598</v>
+        <f>O119*$F$21</f>
+        <v>368988.1568211047</v>
       </c>
       <c r="P120" s="4">
-        <f>P112*$G$21</f>
-        <v>4738655.2163443519</v>
+        <f>P119*$G$21</f>
+        <v>4920861.398185648</v>
       </c>
       <c r="R120" s="4">
-        <f>R112*$F$21</f>
-        <v>309640.18920006661</v>
+        <f>R119*$F$21</f>
+        <v>330813.78904198477</v>
       </c>
       <c r="S120" s="4">
-        <f>S112*$G$21</f>
-        <v>4218664.490707011</v>
+        <f>S119*$G$21</f>
+        <v>4448779.2786547858</v>
       </c>
       <c r="U120" s="4">
-        <f>U112*$F$21</f>
-        <v>275356.17899956723</v>
+        <f>U119*$F$21</f>
+        <v>285863.47987121413</v>
       </c>
       <c r="V120" s="4">
-        <f>V112*$G$21</f>
-        <v>3905797.6666963762</v>
+        <f>V119*$G$21</f>
+        <v>3933836.0703648916</v>
       </c>
       <c r="X120" s="4">
-        <f>X112*$F$21</f>
-        <v>260723.53509440453</v>
+        <f>X119*$F$21</f>
+        <v>270616.74388181337</v>
       </c>
       <c r="Y120" s="4">
-        <f>Y112*$G$21</f>
-        <v>3846990.897830518</v>
+        <f>Y119*$G$21</f>
+        <v>3900902.7674659751</v>
       </c>
       <c r="Z120" s="38"/>
     </row>
@@ -11272,51 +11276,51 @@
       </c>
       <c r="I121" s="4">
         <f>I9*I113</f>
-        <v>8725.1420948347295</v>
+        <v>8828.4274234105033</v>
       </c>
       <c r="J121" s="4">
         <f>J9*J113</f>
-        <v>10124.646374967664</v>
+        <v>10243.554081497259</v>
       </c>
       <c r="L121" s="4">
         <f>L9*L113</f>
-        <v>7605.5576313896927</v>
+        <v>7792.8143204757334</v>
       </c>
       <c r="M121" s="4">
         <f>M9*M113</f>
-        <v>7896.8001246843796</v>
+        <v>8090.9152462251459</v>
       </c>
       <c r="O121" s="4">
         <f>O9*O113</f>
-        <v>8373.9131508098399</v>
+        <v>8758.6202026033661</v>
       </c>
       <c r="P121" s="4">
         <f>P9*P113</f>
-        <v>14574.871868802313</v>
+        <v>15135.274573885425</v>
       </c>
       <c r="R121" s="4">
         <f>R9*R113</f>
-        <v>10575.143073772768</v>
+        <v>11298.285144876529</v>
       </c>
       <c r="S121" s="4">
         <f>S9*S113</f>
-        <v>2637.6797989222368</v>
+        <v>2781.5486558122238</v>
       </c>
       <c r="U121" s="4">
         <f>U9*U113</f>
-        <v>9311.5616086810187</v>
+        <v>9666.8809618284977</v>
       </c>
       <c r="V121" s="4">
         <f>V9*V113</f>
-        <v>6575.8123184113119</v>
+        <v>6622.9705834539536</v>
       </c>
       <c r="X121" s="4">
         <f>X9*X113</f>
-        <v>8907.0997836058177</v>
+        <v>9245.0815381781031</v>
       </c>
       <c r="Y121" s="4">
         <f>Y9*Y113</f>
-        <v>7158.340457945782</v>
+        <v>7258.5574526579549</v>
       </c>
       <c r="Z121" s="38"/>
     </row>
@@ -11408,51 +11412,51 @@
       </c>
       <c r="I123" s="4">
         <f>(I121-I122)*$F$14</f>
-        <v>5886.2594663843101</v>
+        <v>5958.5591963873512</v>
       </c>
       <c r="J123" s="4">
         <f>(J121-J122+J54)*$F$14</f>
-        <v>6332.6524624773647</v>
+        <v>6415.8878570480811</v>
       </c>
       <c r="L123" s="4">
         <f>(L121-L122)*$F$14</f>
-        <v>5112.7703419727841</v>
+        <v>5243.8500243330127</v>
       </c>
       <c r="M123" s="4">
         <f>(M121-M122+M54)*$F$14</f>
-        <v>4882.9200872790652</v>
+        <v>5018.8006723576018</v>
       </c>
       <c r="O123" s="4">
         <f>(O121-O122)*$F$14</f>
-        <v>5631.4392055668877</v>
+        <v>5900.7341418223559</v>
       </c>
       <c r="P123" s="4">
         <f>(P121-P122+P54)*$F$14</f>
-        <v>8871.8503081616182</v>
+        <v>9264.1322017197963</v>
       </c>
       <c r="R123" s="4">
         <f>(R121-R122)*$F$14</f>
-        <v>7038.6001516409369</v>
+        <v>7544.7996014135697</v>
       </c>
       <c r="S123" s="4">
         <f>(S121-S122+S54)*$F$14</f>
-        <v>1570.6458592455656</v>
+        <v>1671.3540590685566</v>
       </c>
       <c r="U123" s="4">
         <f>(U121-U122)*$F$14</f>
-        <v>6236.8331260767136</v>
+        <v>6485.5566732799489</v>
       </c>
       <c r="V123" s="4">
         <f>(V121-V122+V54)*$F$14</f>
-        <v>3794.5686228879181</v>
+        <v>3827.5794084177674</v>
       </c>
       <c r="X123" s="4">
         <f>(X121-X122)*$F$14</f>
-        <v>5885.1098485240727</v>
+        <v>6121.6970767246721</v>
       </c>
       <c r="Y123" s="4">
         <f>(Y121-Y122+Y54)*$F$14</f>
-        <v>4280.0383205620474</v>
+        <v>4350.1902168605684</v>
       </c>
       <c r="Z123" s="38"/>
     </row>
@@ -11472,27 +11476,27 @@
       </c>
       <c r="I124" s="4">
         <f>MIN(I123+J123, I33)</f>
-        <v>12218.911928861675</v>
+        <v>12374.447053435433</v>
       </c>
       <c r="L124" s="4">
         <f>MIN(L123+M123, L33)</f>
-        <v>9995.6904292518484</v>
+        <v>10262.650696690614</v>
       </c>
       <c r="O124" s="4">
         <f>MIN(O123+P123, O33)</f>
-        <v>14503.289513728505</v>
+        <v>15164.866343542151</v>
       </c>
       <c r="R124" s="4">
         <f>MIN(R123+S123, R33)</f>
-        <v>8609.2460108865016</v>
+        <v>9216.1536604821267</v>
       </c>
       <c r="U124" s="4">
         <f>MIN(U123+V123, U33)</f>
-        <v>10031.401748964632</v>
+        <v>10313.136081697716</v>
       </c>
       <c r="X124" s="4">
         <f>MIN(X123+Y123, X33)</f>
-        <v>10165.14816908612</v>
+        <v>10471.887293585241</v>
       </c>
       <c r="Z124" s="38"/>
     </row>
@@ -11516,51 +11520,51 @@
       </c>
       <c r="I125" s="4">
         <f>I123/(I123+J123)</f>
-        <v>0.48173352100858291</v>
+        <v>0.48152124863899409</v>
       </c>
       <c r="J125" s="4">
         <f>J123/(I123+J123)</f>
-        <v>0.51826647899141709</v>
+        <v>0.51847875136100585</v>
       </c>
       <c r="L125" s="4">
         <f>L123/(L123+M123)</f>
-        <v>0.51149746764971205</v>
+        <v>0.51096448464566679</v>
       </c>
       <c r="M125" s="4">
         <f>M123/(L123+M123)</f>
-        <v>0.48850253235028801</v>
+        <v>0.48903551535433326</v>
       </c>
       <c r="O125" s="4">
         <f>O123/(O123+P123)</f>
-        <v>0.3882870296587741</v>
+        <v>0.38910558181972643</v>
       </c>
       <c r="P125" s="4">
         <f>P123/(O123+P123)</f>
-        <v>0.61171297034122596</v>
+        <v>0.61089441818027368</v>
       </c>
       <c r="R125" s="4">
         <f>R123/(R123+S123)</f>
-        <v>0.81756290187788072</v>
+        <v>0.81864950166411143</v>
       </c>
       <c r="S125" s="4">
         <f>S123/(R123+S123)</f>
-        <v>0.18243709812211939</v>
+        <v>0.18135049833588848</v>
       </c>
       <c r="U125" s="4">
         <f>U123/(U123+V123)</f>
-        <v>0.62173096862763311</v>
+        <v>0.62886367656775044</v>
       </c>
       <c r="V125" s="4">
         <f>V123/(U123+V123)</f>
-        <v>0.37826903137236684</v>
+        <v>0.37113632343224967</v>
       </c>
       <c r="X125" s="4">
         <f>X123/(X123+Y123)</f>
-        <v>0.57894973596367783</v>
+        <v>0.58458393459549907</v>
       </c>
       <c r="Y125" s="4">
         <f>Y123/(X123+Y123)</f>
-        <v>0.42105026403632212</v>
+        <v>0.41541606540450088</v>
       </c>
       <c r="Z125" s="38"/>
     </row>
@@ -11584,51 +11588,51 @@
       </c>
       <c r="I126" s="4">
         <f>MAX(I13-I27, 0)*I114</f>
-        <v>445499.85144890583</v>
+        <v>453642.73348242807</v>
       </c>
       <c r="J126" s="4">
         <f>MAX(J13-J27, 0)*J114</f>
-        <v>10836878.67166445</v>
+        <v>11052847.496096702</v>
       </c>
       <c r="L126" s="4">
         <f>MAX(L13-L27, 0)*L114</f>
-        <v>353084.4222994374</v>
+        <v>367064.10270879179</v>
       </c>
       <c r="M126" s="4">
         <f>MAX(M13-M27, 0)*M114</f>
-        <v>9227476.6767802127</v>
+        <v>9639859.7971121781</v>
       </c>
       <c r="O126" s="4">
         <f>MAX(O13-O27, 0)*O114</f>
-        <v>263353.30732921429</v>
+        <v>284017.57182555227</v>
       </c>
       <c r="P126" s="4">
         <f>MAX(P13-P27, 0)*P114</f>
-        <v>7603077.087269336</v>
+        <v>8185382.1980761131</v>
       </c>
       <c r="R126" s="4">
         <f>MAX(R13-R27, 0)*R114</f>
-        <v>177480.99943121945</v>
+        <v>200332.2888780983</v>
       </c>
       <c r="S126" s="4">
         <f>MAX(S13-S27, 0)*S114</f>
-        <v>5980256.3152920818</v>
+        <v>6719760.6844318574</v>
       </c>
       <c r="U126" s="4">
         <f>MAX(U13-U27, 0)*U114</f>
-        <v>107304.18914116903</v>
+        <v>115868.11069356035</v>
       </c>
       <c r="V126" s="4">
         <f>MAX(V13-V27, 0)*V114</f>
-        <v>4961702.5722360462</v>
+        <v>5051464.9612972112</v>
       </c>
       <c r="X126" s="4">
         <f>MAX(X13-X27, 0)*X114</f>
-        <v>93508.216575954808</v>
+        <v>101316.28486525742</v>
       </c>
       <c r="Y126" s="4">
         <f>MAX(Y13-Y27, 0)*Y114</f>
-        <v>4775667.0185383642</v>
+        <v>4948233.7719158493</v>
       </c>
       <c r="Z126" s="38"/>
     </row>
@@ -11667,27 +11671,27 @@
       </c>
       <c r="I129" s="4">
         <f>MAX(I33-I124,0)</f>
-        <v>2037781.0880711384</v>
+        <v>2037625.5529465645</v>
       </c>
       <c r="L129" s="4">
         <f>MAX(L33-L124,0)</f>
-        <v>2100004.3095707484</v>
+        <v>2099737.3493033093</v>
       </c>
       <c r="O129" s="4">
         <f>MAX(O33-O124,0)</f>
-        <v>2195496.7104862714</v>
+        <v>2194835.133656458</v>
       </c>
       <c r="R129" s="4">
         <f>MAX(R33-R124,0)</f>
-        <v>2991390.7539891135</v>
+        <v>2990783.8463395177</v>
       </c>
       <c r="U129" s="4">
         <f>MAX(U33-U124,0)</f>
-        <v>24989968.598251034</v>
+        <v>24989686.863918301</v>
       </c>
       <c r="X129" s="4">
         <f>MAX(X33-X124,0)</f>
-        <v>2509834.8518309137</v>
+        <v>2509528.1127064149</v>
       </c>
       <c r="Z129" s="38"/>
     </row>
@@ -11707,27 +11711,27 @@
       </c>
       <c r="I130" s="4">
         <f>MIN(I140,I129)</f>
-        <v>2037781.0880711384</v>
+        <v>2037625.5529465645</v>
       </c>
       <c r="L130" s="4">
         <f>MIN(L140,L129)</f>
-        <v>2100004.3095707484</v>
+        <v>2099737.3493033093</v>
       </c>
       <c r="O130" s="4">
         <f>MIN(O140,O129)</f>
-        <v>2195496.7104862714</v>
+        <v>2194835.133656458</v>
       </c>
       <c r="R130" s="4">
         <f>MIN(R140,R129)</f>
-        <v>1365522.3071443853</v>
+        <v>2402116.7562237582</v>
       </c>
       <c r="U130" s="4">
         <f>MIN(U140,U129)</f>
-        <v>249661.00634800739</v>
+        <v>342075.56862017012</v>
       </c>
       <c r="X130" s="4">
         <f>MIN(X140,X129)</f>
-        <v>81322.864565083524</v>
+        <v>236958.69160889552</v>
       </c>
       <c r="Z130" s="38"/>
     </row>
@@ -11759,15 +11763,15 @@
       </c>
       <c r="R131" s="4">
         <f>R129-R130</f>
-        <v>1625868.4468447282</v>
+        <v>588667.09011575952</v>
       </c>
       <c r="U131" s="4">
         <f>U129-U130</f>
-        <v>24740307.591903027</v>
+        <v>24647611.295298129</v>
       </c>
       <c r="X131" s="4">
         <f>X129-X130</f>
-        <v>2428511.9872658299</v>
+        <v>2272569.4210975193</v>
       </c>
       <c r="Z131" s="38"/>
     </row>
@@ -11831,51 +11835,51 @@
       </c>
       <c r="I133" s="4">
         <f>I141*I130</f>
-        <v>80464.51997345034</v>
+        <v>80333.273414349693</v>
       </c>
       <c r="J133" s="4">
         <f>J141*I130</f>
-        <v>1957316.568097688</v>
+        <v>1957292.2795322149</v>
       </c>
       <c r="L133" s="4">
         <f>L141*L130</f>
-        <v>100241.7582597421</v>
+        <v>91806.708408756895</v>
       </c>
       <c r="M133" s="4">
         <f>M141*L130</f>
-        <v>1999762.5513110063</v>
+        <v>2007930.6408945527</v>
       </c>
       <c r="O133" s="4">
         <f>O141*O130</f>
-        <v>124509.76530548533</v>
+        <v>119687.89540326738</v>
       </c>
       <c r="P133" s="4">
         <f>P141*O130</f>
-        <v>2070986.9451807863</v>
+        <v>2075147.2382531904</v>
       </c>
       <c r="R133" s="4">
         <f>R141*R130</f>
-        <v>94293.001358187947</v>
+        <v>139940.26445123838</v>
       </c>
       <c r="S133" s="4">
         <f>S141*R130</f>
-        <v>1271229.3057861973</v>
+        <v>2262176.4917725199</v>
       </c>
       <c r="U133" s="4">
         <f>U141*U130</f>
-        <v>30365.318035164255</v>
+        <v>42505.359023831879</v>
       </c>
       <c r="V133" s="4">
         <f>V141*U130</f>
-        <v>219295.68831284312</v>
+        <v>299570.20959633822</v>
       </c>
       <c r="X133" s="4">
         <f>X141*X130</f>
-        <v>17535.251773675584</v>
+        <v>27081.188280169557</v>
       </c>
       <c r="Y133" s="4">
         <f>Y141*X130</f>
-        <v>63787.612791407948</v>
+        <v>209877.50332872596</v>
       </c>
       <c r="Z133" s="38"/>
     </row>
@@ -11899,51 +11903,51 @@
       </c>
       <c r="I134" s="4">
         <f>I133</f>
-        <v>80464.51997345034</v>
+        <v>80333.273414349693</v>
       </c>
       <c r="J134" s="4">
         <f>J133+I132</f>
-        <v>1957316.568097688</v>
+        <v>1957292.2795322149</v>
       </c>
       <c r="L134" s="4">
         <f>L133</f>
-        <v>100241.7582597421</v>
+        <v>91806.708408756895</v>
       </c>
       <c r="M134" s="4">
         <f>M133+L132</f>
-        <v>1999762.5513110063</v>
+        <v>2007930.6408945527</v>
       </c>
       <c r="O134" s="4">
         <f>O133</f>
-        <v>124509.76530548533</v>
+        <v>119687.89540326738</v>
       </c>
       <c r="P134" s="4">
         <f>P133+O132</f>
-        <v>2070986.9451807863</v>
+        <v>2075147.2382531904</v>
       </c>
       <c r="R134" s="4">
         <f>R133</f>
-        <v>94293.001358187947</v>
+        <v>139940.26445123838</v>
       </c>
       <c r="S134" s="4">
         <f>S133+R132</f>
-        <v>1271229.3057861973</v>
+        <v>2262176.4917725199</v>
       </c>
       <c r="U134" s="4">
         <f>U133</f>
-        <v>30365.318035164255</v>
+        <v>42505.359023831879</v>
       </c>
       <c r="V134" s="4">
         <f>V133+U132</f>
-        <v>219295.68831284312</v>
+        <v>299570.20959633822</v>
       </c>
       <c r="X134" s="4">
         <f>X133</f>
-        <v>17535.251773675584</v>
+        <v>27081.188280169557</v>
       </c>
       <c r="Y134" s="4">
         <f>Y133+X132</f>
-        <v>63787.612791407948</v>
+        <v>209877.50332872596</v>
       </c>
       <c r="Z134" s="38"/>
     </row>
@@ -11986,51 +11990,51 @@
       </c>
       <c r="I136" s="4">
         <f>I114/$F$23</f>
-        <v>0.90766274449544915</v>
+        <v>0.92425307697392622</v>
       </c>
       <c r="J136" s="4">
         <f>J114/$G$23</f>
-        <v>0.87205989585080868</v>
+        <v>0.8894392313816073</v>
       </c>
       <c r="L136" s="4">
         <f>L114/$F$23</f>
-        <v>0.81207998111883728</v>
+        <v>0.84423268422860009</v>
       </c>
       <c r="M136" s="4">
         <f>M114/$G$23</f>
-        <v>0.74289843043449877</v>
+        <v>0.77609913996359592</v>
       </c>
       <c r="O136" s="4">
         <f>O114/$F$23</f>
-        <v>0.69752387212354428</v>
+        <v>0.75225573758689401</v>
       </c>
       <c r="P136" s="4">
         <f>P114/$G$23</f>
-        <v>0.61270812108838446</v>
+        <v>0.65963426247132328</v>
       </c>
       <c r="R136" s="4">
         <f>R114/$F$23</f>
-        <v>0.55933619881349728</v>
+        <v>0.63135265926935324</v>
       </c>
       <c r="S136" s="4">
         <f>S114/$G$23</f>
-        <v>0.47961978548953171</v>
+        <v>0.5389284351854382</v>
       </c>
       <c r="U136" s="4">
         <f>U114/$F$23</f>
-        <v>0.45242326277638945</v>
+        <v>0.48853105467067059</v>
       </c>
       <c r="V136" s="4">
         <f>V114/$G$23</f>
-        <v>0.3991358105007784</v>
+        <v>0.4063565947756948</v>
       </c>
       <c r="X136" s="4">
         <f>X114/$F$23</f>
-        <v>0.41132157979844358</v>
+        <v>0.44566751325255183</v>
       </c>
       <c r="Y136" s="4">
         <f>Y114/$G$23</f>
-        <v>0.38439359803052098</v>
+        <v>0.39828350178087057</v>
       </c>
       <c r="Z136" s="38"/>
       <c r="AA136">
@@ -12076,39 +12080,39 @@
       </c>
       <c r="M137" s="4">
         <f>MAX(MIN((M136-$G$17)/$G$18, 1), 0)</f>
-        <v>0.76335289475554091</v>
+        <v>0.8328091484893303</v>
       </c>
       <c r="O137" s="4">
         <f>MAX(MIN((O136-$F$17)/$F$18, 1), 0)</f>
-        <v>0.85222104179390024</v>
+        <v>0.97933386739236106</v>
       </c>
       <c r="P137" s="4">
         <f>MAX(MIN((P136-$G$17)/$G$18, 1), 0)</f>
-        <v>0.49099331907540816</v>
+        <v>0.5891633289598236</v>
       </c>
       <c r="R137" s="4">
         <f>MAX(MIN((R136-$F$17)/$F$18, 1), 0)</f>
-        <v>0.53128504831712997</v>
+        <v>0.69854073566938424</v>
       </c>
       <c r="S137" s="4">
         <f>MAX(MIN((S136-$G$17)/$G$18, 1), 0)</f>
-        <v>0.2125710402304235</v>
+        <v>0.33664539527627274</v>
       </c>
       <c r="U137" s="4">
         <f>MAX(MIN((U136-$F$17)/$F$18, 1), 0)</f>
-        <v>0.28298352821263806</v>
+        <v>0.36684260034451582</v>
       </c>
       <c r="V137" s="4">
         <f>MAX(MIN((V136-$G$17)/$G$18, 1), 0)</f>
-        <v>4.4197669070279458E-2</v>
+        <v>5.9303630113552025E-2</v>
       </c>
       <c r="X137" s="4">
         <f>MAX(MIN((X136-$F$17)/$F$18, 1), 0)</f>
-        <v>0.18752632031466515</v>
+        <v>0.26729353840979642</v>
       </c>
       <c r="Y137" s="4">
         <f>MAX(MIN((Y136-$G$17)/$G$18, 1), 0)</f>
-        <v>1.3356796557170923E-2</v>
+        <v>4.2414629745244618E-2</v>
       </c>
       <c r="Z137" s="38"/>
       <c r="AA137">
@@ -12156,58 +12160,58 @@
       </c>
       <c r="I139" s="4">
         <f>I126*I137</f>
-        <v>445499.85144890583</v>
+        <v>453642.73348242807</v>
       </c>
       <c r="J139" s="4">
         <f>J126*J137</f>
-        <v>10836878.67166445</v>
+        <v>11052847.496096702</v>
       </c>
       <c r="L139" s="4">
         <f>L126*L137</f>
-        <v>353084.4222994374</v>
+        <v>367064.10270879179</v>
       </c>
       <c r="M139" s="4">
         <f>M126*M137</f>
-        <v>7043821.0325094145</v>
+        <v>8028163.4291895209</v>
       </c>
       <c r="O139" s="4">
         <f>O126*O137</f>
-        <v>224435.22993197219</v>
+        <v>278148.02702330577</v>
       </c>
       <c r="P139" s="4">
         <f>P126*P137</f>
-        <v>3733060.054264558</v>
+        <v>4822527.024627001</v>
       </c>
       <c r="R139" s="4">
         <f>R126*R137</f>
-        <v>94293.001358187947</v>
+        <v>139940.26445123838</v>
       </c>
       <c r="S139" s="4">
         <f>S126*S137</f>
-        <v>1271229.3057861973</v>
+        <v>2262176.4917725199</v>
       </c>
       <c r="U139" s="4">
         <f>U126*U137</f>
-        <v>30365.318035164255</v>
+        <v>42505.359023831879</v>
       </c>
       <c r="V139" s="4">
         <f>V126*V137</f>
-        <v>219295.68831284312</v>
+        <v>299570.20959633822</v>
       </c>
       <c r="X139" s="4">
         <f>X126*X137</f>
-        <v>17535.251773675584</v>
+        <v>27081.188280169557</v>
       </c>
       <c r="Y139" s="4">
         <f>Y126*Y137</f>
-        <v>63787.612791407948</v>
+        <v>209877.50332872596</v>
       </c>
       <c r="Z139" s="38"/>
       <c r="AA139">
         <v>0.125</v>
       </c>
       <c r="AB139">
-        <f>SUM(AA$6:AA158)</f>
+        <f>SUM(AA$6:AA159)</f>
         <v>1.125</v>
       </c>
       <c r="AC139">
@@ -12234,51 +12238,51 @@
       </c>
       <c r="I140" s="4">
         <f>I139+J139</f>
-        <v>11282378.523113357</v>
+        <v>11506490.22957913</v>
       </c>
       <c r="J140" s="4">
         <f>I140</f>
-        <v>11282378.523113357</v>
+        <v>11506490.22957913</v>
       </c>
       <c r="L140" s="4">
         <f>L139+M139</f>
-        <v>7396905.4548088517</v>
+        <v>8395227.5318983123</v>
       </c>
       <c r="M140" s="4">
         <f>L140</f>
-        <v>7396905.4548088517</v>
+        <v>8395227.5318983123</v>
       </c>
       <c r="O140" s="4">
         <f>O139+P139</f>
-        <v>3957495.28419653</v>
+        <v>5100675.0516503071</v>
       </c>
       <c r="P140" s="4">
         <f>O140</f>
-        <v>3957495.28419653</v>
+        <v>5100675.0516503071</v>
       </c>
       <c r="R140" s="4">
         <f>R139+S139</f>
-        <v>1365522.3071443853</v>
+        <v>2402116.7562237582</v>
       </c>
       <c r="S140" s="4">
         <f>R140</f>
-        <v>1365522.3071443853</v>
+        <v>2402116.7562237582</v>
       </c>
       <c r="U140" s="4">
         <f>U139+V139</f>
-        <v>249661.00634800739</v>
+        <v>342075.56862017012</v>
       </c>
       <c r="V140" s="4">
         <f>U140</f>
-        <v>249661.00634800739</v>
+        <v>342075.56862017012</v>
       </c>
       <c r="X140" s="4">
         <f>X139+Y139</f>
-        <v>81322.864565083524</v>
+        <v>236958.69160889552</v>
       </c>
       <c r="Y140" s="4">
         <f>X140</f>
-        <v>81322.864565083524</v>
+        <v>236958.69160889552</v>
       </c>
       <c r="Z140" s="38"/>
     </row>
@@ -12302,51 +12306,51 @@
       </c>
       <c r="I141" s="4">
         <f>I139/I140</f>
-        <v>3.9486341513559745E-2</v>
+        <v>3.9424944047340565E-2</v>
       </c>
       <c r="J141" s="4">
         <f>J139/J140</f>
-        <v>0.96051365848644021</v>
+        <v>0.96057505595265946</v>
       </c>
       <c r="L141" s="4">
         <f>L139/L140</f>
-        <v>4.773407264113283E-2</v>
+        <v>4.3722948700806917E-2</v>
       </c>
       <c r="M141" s="4">
         <f>M139/M140</f>
-        <v>0.95226592735886717</v>
+        <v>0.95627705129919316</v>
       </c>
       <c r="O141" s="4">
         <f>O139/O140</f>
-        <v>5.6711433322033163E-2</v>
+        <v>5.4531610856745689E-2</v>
       </c>
       <c r="P141" s="4">
         <f>P139/P140</f>
-        <v>0.9432885666779669</v>
+        <v>0.94546838914325426</v>
       </c>
       <c r="R141" s="4">
         <f>R139/R140</f>
-        <v>6.9052699369939879E-2</v>
+        <v>5.8257061855407535E-2</v>
       </c>
       <c r="S141" s="4">
         <f>S139/S140</f>
-        <v>0.93094730063006004</v>
+        <v>0.94174293814459253</v>
       </c>
       <c r="U141" s="4">
         <f>U139/U140</f>
-        <v>0.12162619417161781</v>
+        <v>0.12425721952399496</v>
       </c>
       <c r="V141" s="4">
         <f>V139/V140</f>
-        <v>0.87837380582838209</v>
+        <v>0.87574278047600496</v>
       </c>
       <c r="X141" s="4">
         <f>X139/X140</f>
-        <v>0.21562511192214512</v>
+        <v>0.11428653701746266</v>
       </c>
       <c r="Y141" s="4">
         <f>Y139/Y140</f>
-        <v>0.78437488807785494</v>
+        <v>0.88571346298253728</v>
       </c>
       <c r="Z141" s="38"/>
     </row>
@@ -12381,478 +12385,531 @@
       </c>
       <c r="F144" s="4">
         <f>(F112 - F133 - F121)*$F$30</f>
-        <v>18798.841062135314</v>
+        <v>2223.2117181201452</v>
       </c>
       <c r="G144" s="4">
         <f>(G112 - G133 - G121)*$G$30+SUM(G91:G94)</f>
-        <v>306368.86168411467</v>
+        <v>36232.172031879854</v>
       </c>
       <c r="I144" s="4">
         <f>(I112 - I133 - I121)*$F$30</f>
-        <v>17404.870206432512</v>
+        <v>2084.4238554074132</v>
       </c>
       <c r="J144" s="4">
         <f>(J112 - J133 - J121)*$G$30+SUM(J91:J94)</f>
-        <v>279235.1009891578</v>
+        <v>33447.211823016281</v>
       </c>
       <c r="L144" s="4">
         <f>(L112 - L133 - L121)*$F$30</f>
-        <v>15781.46892166788</v>
+        <v>1929.437307269528</v>
       </c>
       <c r="M144" s="4">
         <f>(M112 - M133 - M121)*$G$30+SUM(M91:M94)</f>
-        <v>251926.30685617079</v>
+        <v>30590.343867813121</v>
       </c>
       <c r="O144" s="4">
         <f>(O112 - O133 - O121)*$F$30</f>
-        <v>13847.018578636153</v>
+        <v>1729.3769911958977</v>
       </c>
       <c r="P144" s="4">
         <f>(P112 - P133 - P121)*$G$30+SUM(P91:P94)</f>
-        <v>223944.76549977509</v>
+        <v>27621.242311606977</v>
       </c>
       <c r="R144" s="4">
         <f>(R112 - R133 - R121)*$F$30</f>
-        <v>12309.889569703864</v>
+        <v>1493.8143064538199</v>
       </c>
       <c r="S144" s="4">
         <f>(S112 - S133 - S121)*$G$30+SUM(S91:S94)</f>
-        <v>207108.11045742003</v>
+        <v>24382.300139165654</v>
       </c>
       <c r="U144" s="4">
         <f>(U112 - U133 - U121)*$F$30</f>
-        <v>11658.213086672471</v>
+        <v>1414.1084612152006</v>
       </c>
       <c r="V144" s="4">
         <f>(V112 - V133 - V121)*$G$30+SUM(V91:V94)</f>
-        <v>204407.342747824</v>
+        <v>24223.673488378809</v>
       </c>
       <c r="X144" s="4">
         <f>(X112 - X133 - X121)*$F$30</f>
-        <v>11186.390249970907</v>
+        <v>1359.1953827000175</v>
       </c>
       <c r="Y144" s="4">
         <f>(Y112 - Y133 - Y121)*$G$30+SUM(Y91:Y94)</f>
-        <v>203342.08674697479</v>
+        <v>24156.603765901902</v>
       </c>
       <c r="Z144" s="38"/>
     </row>
-    <row r="145" spans="1:29" ht="17" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A145" s="38" t="s">
-        <v>275</v>
+        <v>303</v>
       </c>
       <c r="B145" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="E145" s="14" t="s">
+      <c r="F145" s="4">
+        <f>F144*$F21</f>
+        <v>666.96351543604351</v>
+      </c>
+      <c r="G145" s="4">
+        <f>G144*$G21</f>
+        <v>9058.0430079699636</v>
+      </c>
+      <c r="I145" s="4">
+        <f>I144*$F21</f>
+        <v>625.32715662222392</v>
+      </c>
+      <c r="J145" s="4">
+        <f>J144*$G21</f>
+        <v>8361.8029557540704</v>
+      </c>
+      <c r="L145" s="4">
+        <f>L144*$F21</f>
+        <v>578.83119218085835</v>
+      </c>
+      <c r="M145" s="4">
+        <f>M144*$G21</f>
+        <v>7647.5859669532801</v>
+      </c>
+      <c r="O145" s="4">
+        <f>O144*$F21</f>
+        <v>518.81309735876926</v>
+      </c>
+      <c r="P145" s="4">
+        <f>P144*$G21</f>
+        <v>6905.3105779017442</v>
+      </c>
+      <c r="R145" s="4">
+        <f>R144*$F21</f>
+        <v>448.14429193614598</v>
+      </c>
+      <c r="S145" s="4">
+        <f>S144*$G21</f>
+        <v>6095.5750347914136</v>
+      </c>
+      <c r="U145" s="4">
+        <f>U144*$F21</f>
+        <v>424.23253836456018</v>
+      </c>
+      <c r="V145" s="4">
+        <f>V144*$G21</f>
+        <v>6055.9183720947021</v>
+      </c>
+      <c r="X145" s="4">
+        <f>X144*$F21</f>
+        <v>407.75861481000521</v>
+      </c>
+      <c r="Y145" s="4">
+        <f>Y144*$G21</f>
+        <v>6039.1509414754755</v>
+      </c>
+      <c r="Z145" s="38"/>
+    </row>
+    <row r="146" spans="1:29" ht="17" x14ac:dyDescent="0.2">
+      <c r="A146" s="38" t="s">
+        <v>275</v>
+      </c>
+      <c r="B146" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="E146" s="14" t="s">
         <v>215</v>
       </c>
-      <c r="F145" s="4">
+      <c r="F146" s="4">
         <f>F133*$F21</f>
         <v>22932.474244558285</v>
       </c>
-      <c r="G145" s="4">
+      <c r="G146" s="4">
         <f>(G133+F132)*$G21</f>
         <v>478045.8547962014</v>
       </c>
-      <c r="I145" s="4">
+      <c r="I146" s="4">
         <f>I133*$F21</f>
-        <v>24139.3559920351</v>
-      </c>
-      <c r="J145" s="4">
+        <v>24099.982024304907</v>
+      </c>
+      <c r="J146" s="4">
         <f>(J133+I132)*$G21</f>
-        <v>489329.14202442201</v>
-      </c>
-      <c r="L145" s="4">
+        <v>489323.06988305371</v>
+      </c>
+      <c r="L146" s="4">
         <f>L133*$F21</f>
-        <v>30072.527477922627</v>
-      </c>
-      <c r="M145" s="4">
+        <v>27542.012522627068</v>
+      </c>
+      <c r="M146" s="4">
         <f>(M133+L132)*$G21</f>
-        <v>499940.63782775158</v>
-      </c>
-      <c r="O145" s="4">
+        <v>501982.66022363817</v>
+      </c>
+      <c r="O146" s="4">
         <f>O133*$F21</f>
-        <v>37352.929591645596</v>
-      </c>
-      <c r="P145" s="4">
+        <v>35906.368620980211</v>
+      </c>
+      <c r="P146" s="4">
         <f>(P133+O132)*$G21</f>
-        <v>517746.73629519658</v>
-      </c>
-      <c r="R145" s="4">
+        <v>518786.8095632976</v>
+      </c>
+      <c r="R146" s="4">
         <f>R133*$F21</f>
-        <v>28287.900407456382</v>
-      </c>
-      <c r="S145" s="4">
+        <v>41982.079335371513</v>
+      </c>
+      <c r="S146" s="4">
         <f>(S133+R132)*$G21</f>
-        <v>317807.32644654933</v>
-      </c>
-      <c r="U145" s="4">
+        <v>565544.12294312997</v>
+      </c>
+      <c r="U146" s="4">
         <f>U133*$F21</f>
-        <v>9109.5954105492765</v>
-      </c>
-      <c r="V145" s="4">
+        <v>12751.607707149564</v>
+      </c>
+      <c r="V146" s="4">
         <f>(V133+U132)*$G21</f>
-        <v>54823.92207821078</v>
-      </c>
-      <c r="X145" s="4">
+        <v>74892.552399084554</v>
+      </c>
+      <c r="X146" s="4">
         <f>X133*$F21</f>
-        <v>5260.5755321026745</v>
-      </c>
-      <c r="Y145" s="4">
+        <v>8124.356484050867</v>
+      </c>
+      <c r="Y146" s="4">
         <f>(Y133+X132)*$G21</f>
-        <v>15946.903197851987</v>
-      </c>
-      <c r="Z145" s="38"/>
-    </row>
-    <row r="146" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A146" s="38" t="s">
+        <v>52469.375832181489</v>
+      </c>
+      <c r="Z146" s="38"/>
+    </row>
+    <row r="147" spans="1:29" ht="17" x14ac:dyDescent="0.2">
+      <c r="A147" s="38" t="s">
         <v>176</v>
       </c>
-      <c r="B146" s="33" t="s">
+      <c r="B147" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="E146" s="10" t="s">
+      <c r="E147" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="F146" s="4">
+      <c r="F147" s="4">
         <f>F121-F124*F125-F122</f>
         <v>2175</v>
       </c>
-      <c r="G146" s="4">
+      <c r="G147" s="4">
         <f>G121-F124*G125-G122+G54</f>
         <v>2700</v>
       </c>
-      <c r="I146" s="4">
+      <c r="I147" s="4">
         <f>I121-I124*I125-I122</f>
-        <v>2522.6826284504195</v>
-      </c>
-      <c r="J146" s="4">
+        <v>2553.6682270231522</v>
+      </c>
+      <c r="J147" s="4">
         <f>J121-I124*J125-J122+J54</f>
-        <v>2713.9939124902994</v>
-      </c>
-      <c r="L146" s="4">
+        <v>2749.6662244491781</v>
+      </c>
+      <c r="L147" s="4">
         <f>L121-L124*L125-L122</f>
-        <v>2191.1872894169087</v>
-      </c>
-      <c r="M146" s="4">
+        <v>2247.3642961427208</v>
+      </c>
+      <c r="M147" s="4">
         <f>M121-L124*M125-M122+M54</f>
-        <v>2092.6800374053146</v>
-      </c>
-      <c r="O146" s="4">
+        <v>2150.9145738675443</v>
+      </c>
+      <c r="O147" s="4">
         <f>O121-O124*O125-O122</f>
-        <v>2413.4739452429521</v>
-      </c>
-      <c r="P146" s="4">
+        <v>2528.8860607810102</v>
+      </c>
+      <c r="P147" s="4">
         <f>P121-O124*P125-P122+P54</f>
-        <v>3802.2215606406944</v>
-      </c>
-      <c r="R146" s="4">
+        <v>3970.3423721656281</v>
+      </c>
+      <c r="R147" s="4">
         <f>R121-R124*R125-R122</f>
-        <v>3016.5429221318309</v>
-      </c>
-      <c r="S146" s="4">
+        <v>3233.485543462959</v>
+      </c>
+      <c r="S147" s="4">
         <f>S121-R124*S125-S122+S54</f>
-        <v>673.13393967667128</v>
-      </c>
-      <c r="U146" s="4">
+        <v>716.29459674366728</v>
+      </c>
+      <c r="U147" s="4">
         <f>U121-U124*U125-U122</f>
-        <v>2672.9284826043049</v>
-      </c>
-      <c r="V146" s="4">
+        <v>2779.5242885485477</v>
+      </c>
+      <c r="V147" s="4">
         <f>V121-U124*V125-V122+V54</f>
-        <v>1626.2436955233939</v>
-      </c>
-      <c r="X146" s="4">
+        <v>1640.3911750361863</v>
+      </c>
+      <c r="X147" s="4">
         <f>X121-X124*X125-X122</f>
-        <v>2522.1899350817448</v>
-      </c>
-      <c r="Y146" s="4">
+        <v>2623.5844614534308</v>
+      </c>
+      <c r="Y147" s="4">
         <f>Y121-X124*Y125-Y122+Y54</f>
-        <v>1834.3021373837346</v>
-      </c>
-      <c r="Z146" s="38"/>
-    </row>
-    <row r="147" spans="1:29" ht="17" x14ac:dyDescent="0.2">
-      <c r="A147" s="38" t="s">
+        <v>1864.3672357973865</v>
+      </c>
+      <c r="Z147" s="38"/>
+    </row>
+    <row r="148" spans="1:29" ht="17" x14ac:dyDescent="0.2">
+      <c r="A148" s="38" t="s">
         <v>177</v>
       </c>
-      <c r="B147" s="33" t="s">
+      <c r="B148" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="E147" s="10" t="s">
+      <c r="E148" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="F147" s="4">
+      <c r="F148" s="4">
         <f>MAX((F121 - F122)*$F21-F16*F9,0)</f>
         <v>2128.25</v>
       </c>
-      <c r="G147" s="4">
+      <c r="G148" s="4">
         <f>MAX((G121-G122+G54)*$G21-G16*G9,0)</f>
         <v>2058</v>
       </c>
-      <c r="I147" s="4">
+      <c r="I148" s="4">
         <f>MAX((I121 - I122)*$F21-I16*I9,0)</f>
-        <v>2463.5532284504188</v>
-      </c>
-      <c r="J147" s="4">
+        <v>2494.538827023151</v>
+      </c>
+      <c r="J148" s="4">
         <f>MAX((J121-J122+J54)*$G21-J16*J9,0)</f>
-        <v>2054.6855937419159</v>
-      </c>
-      <c r="L147" s="4">
+        <v>2084.4125203743147</v>
+      </c>
+      <c r="L148" s="4">
         <f>MAX((L121 - L122)*$F21-L16*L9,0)</f>
-        <v>2134.788089416908</v>
-      </c>
-      <c r="M147" s="4">
+        <v>2190.9650961427201</v>
+      </c>
+      <c r="M148" s="4">
         <f>MAX((M121-M122+M54)*$G21-M16*M9,0)</f>
-        <v>1567.0296311710949</v>
-      </c>
-      <c r="O147" s="4">
+        <v>1615.5584115562865</v>
+      </c>
+      <c r="O148" s="4">
         <f>MAX((O121 - O122)*$F21-O16*O9,0)</f>
-        <v>2351.9509452429515</v>
-      </c>
-      <c r="P147" s="4">
+        <v>2467.3630607810096</v>
+      </c>
+      <c r="P148" s="4">
         <f>MAX((P121-P122+P54)*$G21-P16*P9,0)</f>
-        <v>2803.5643672005781</v>
-      </c>
-      <c r="R147" s="4">
+        <v>2943.6650434713565</v>
+      </c>
+      <c r="R148" s="4">
         <f>MAX((R121 - R122)*$F21-R16*R9,0)</f>
-        <v>2919.3029221318302</v>
-      </c>
-      <c r="S147" s="4">
+        <v>3136.2455434629583</v>
+      </c>
+      <c r="S148" s="4">
         <f>MAX((S121-S122+S54)*$G21-S16*S9,0)</f>
-        <v>485.31614973055918</v>
-      </c>
-      <c r="U147" s="4">
+        <v>521.28336395305598</v>
+      </c>
+      <c r="U148" s="4">
         <f>MAX((U121 - U122)*$F21-U16*U9,0)</f>
-        <v>2597.791882604306</v>
-      </c>
-      <c r="V147" s="4">
+        <v>2704.3876885485497</v>
+      </c>
+      <c r="V148" s="4">
         <f>MAX((V121-V122+V54)*$G21-V16*V9,0)</f>
-        <v>1133.443079602828</v>
-      </c>
-      <c r="X147" s="4">
+        <v>1145.2326458634884</v>
+      </c>
+      <c r="X148" s="4">
         <f>MAX((X121 - X122)*$F21-X16*X9,0)</f>
-        <v>2428.7273350817454</v>
-      </c>
-      <c r="Y147" s="4">
+        <v>2530.1218614534314</v>
+      </c>
+      <c r="Y148" s="4">
         <f>MAX((Y121-Y122+Y54)*$G21-Y16*Y9,0)</f>
-        <v>1328.1371144864454</v>
-      </c>
-      <c r="Z147" s="38"/>
-    </row>
-    <row r="148" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A148" s="38" t="s">
+        <v>1353.1913631644886</v>
+      </c>
+      <c r="Z148" s="38"/>
+    </row>
+    <row r="149" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A149" s="38" t="s">
         <v>302</v>
       </c>
-      <c r="B148" s="33" t="s">
+      <c r="B149" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="F148" s="4">
+      <c r="F149" s="4">
         <f>I111*I7*(1+$F21)</f>
         <v>3880.5</v>
       </c>
-      <c r="G148" s="4">
+      <c r="G149" s="4">
         <f>(J111*J7+SUMPRODUCT(G38:G41,G86:G89))*(1+$G21)</f>
         <v>287385</v>
       </c>
-      <c r="I148" s="4">
+      <c r="I149" s="4">
         <f>L111*L7*(1+$F21)</f>
         <v>3856.32</v>
       </c>
-      <c r="J148" s="4">
+      <c r="J149" s="4">
         <f>(M111*M7+SUMPRODUCT(J38:J41,J86:J89))*(1+$G21)</f>
         <v>287259.5625</v>
       </c>
-      <c r="L148" s="4">
+      <c r="L149" s="4">
         <f>O111*O7*(1+$F21)</f>
         <v>3833.7000000000003</v>
       </c>
-      <c r="M148" s="4">
+      <c r="M149" s="4">
         <f>(P111*P7+SUMPRODUCT(M38:M41,M86:M89))*(1+$G21)</f>
         <v>287156.71250000002</v>
       </c>
-      <c r="O148" s="4">
+      <c r="O149" s="4">
         <f>R111*R7*(1+$F21)</f>
         <v>3806.4</v>
       </c>
-      <c r="P148" s="4">
+      <c r="P149" s="4">
         <f>(S111*S7+SUMPRODUCT(P38:P41,P86:P89))*(1+$G21)</f>
         <v>286948.5</v>
       </c>
-      <c r="R148" s="4">
+      <c r="R149" s="4">
         <f>U111*U7*(1+$F21)</f>
         <v>3767.4</v>
       </c>
-      <c r="S148" s="4">
+      <c r="S149" s="4">
         <f>(V111*V7+SUMPRODUCT(S38:S41,S86:S89))*(1+$G21)</f>
         <v>286924.28750000003</v>
       </c>
-      <c r="U148" s="4">
+      <c r="U149" s="4">
         <f>X111*X7*(1+$F21)</f>
-        <v>3327.4969606347436</v>
-      </c>
-      <c r="V148" s="4">
+        <v>3593.0636935346747</v>
+      </c>
+      <c r="V149" s="4">
         <f>(Y111*Y7+SUMPRODUCT(V38:V41,V86:V89))*(1+$G21)</f>
-        <v>243889.44739455794</v>
-      </c>
-      <c r="X148" s="4">
+        <v>248300.31050651748</v>
+      </c>
+      <c r="X149" s="4">
         <f>AA111*AA7*(1+$F21)</f>
         <v>0</v>
       </c>
-      <c r="Y148" s="4">
+      <c r="Y149" s="4">
         <f>(AB111*AB7+SUMPRODUCT(Y38:Y41,Y86:Y89))*(1+$G21)</f>
         <v>129.19999999999999</v>
       </c>
-      <c r="Z148" s="38"/>
-    </row>
-    <row r="151" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A151" s="24" t="s">
+      <c r="Z149" s="38"/>
+    </row>
+    <row r="152" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A152" s="24" t="s">
         <v>267</v>
       </c>
-      <c r="F151" s="4">
-        <f>F146+F122</f>
+      <c r="F152" s="4">
+        <f>F147+F122</f>
         <v>2425</v>
       </c>
-      <c r="G151" s="4">
-        <f>G146+G122</f>
+      <c r="G152" s="4">
+        <f>G147+G122</f>
         <v>3700</v>
       </c>
-      <c r="I151" s="4">
-        <f>I146+I122</f>
-        <v>2838.8826284504194</v>
-      </c>
-      <c r="J151" s="4">
-        <f>J146+J122</f>
-        <v>3791.9939124902994</v>
-      </c>
-      <c r="L151" s="4">
-        <f>L146+L122</f>
-        <v>2492.7872894169086</v>
-      </c>
-      <c r="M151" s="4">
-        <f>M146+M122</f>
-        <v>3013.8800374053144</v>
-      </c>
-      <c r="O151" s="4">
-        <f>O146+O122</f>
-        <v>2742.4739452429521</v>
-      </c>
-      <c r="P151" s="4">
-        <f>P146+P122</f>
-        <v>5703.0215606406946</v>
-      </c>
-      <c r="R151" s="4">
-        <f>R146+R122</f>
-        <v>3536.5429221318309</v>
-      </c>
-      <c r="S151" s="4">
-        <f>S146+S122</f>
-        <v>1067.0339396766713</v>
-      </c>
-      <c r="U151" s="4">
-        <f>U146+U122</f>
-        <v>3074.7284826043051</v>
-      </c>
-      <c r="V151" s="4">
-        <f>V146+V122</f>
-        <v>2781.2436955233939</v>
-      </c>
-      <c r="X151" s="4">
-        <f>X146+X122</f>
-        <v>3021.989935081745</v>
-      </c>
-      <c r="Y151" s="4">
-        <f>Y146+Y122</f>
-        <v>2878.3021373837346</v>
-      </c>
-    </row>
-    <row r="153" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A153" s="38" t="s">
+      <c r="I152" s="4">
+        <f>I147+I122</f>
+        <v>2869.868227023152</v>
+      </c>
+      <c r="J152" s="4">
+        <f>J147+J122</f>
+        <v>3827.6662244491781</v>
+      </c>
+      <c r="L152" s="4">
+        <f>L147+L122</f>
+        <v>2548.9642961427207</v>
+      </c>
+      <c r="M152" s="4">
+        <f>M147+M122</f>
+        <v>3072.1145738675441</v>
+      </c>
+      <c r="O152" s="4">
+        <f>O147+O122</f>
+        <v>2857.8860607810102</v>
+      </c>
+      <c r="P152" s="4">
+        <f>P147+P122</f>
+        <v>5871.1423721656283</v>
+      </c>
+      <c r="R152" s="4">
+        <f>R147+R122</f>
+        <v>3753.485543462959</v>
+      </c>
+      <c r="S152" s="4">
+        <f>S147+S122</f>
+        <v>1110.1945967436673</v>
+      </c>
+      <c r="U152" s="4">
+        <f>U147+U122</f>
+        <v>3181.3242885485479</v>
+      </c>
+      <c r="V152" s="4">
+        <f>V147+V122</f>
+        <v>2795.3911750361863</v>
+      </c>
+      <c r="X152" s="4">
+        <f>X147+X122</f>
+        <v>3123.384461453431</v>
+      </c>
+      <c r="Y152" s="4">
+        <f>Y147+Y122</f>
+        <v>2908.3672357973865</v>
+      </c>
+    </row>
+    <row r="154" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A154" s="38" t="s">
         <v>277</v>
       </c>
-      <c r="B153" s="33" t="s">
+      <c r="B154" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="F153" s="4">
+      <c r="F154" s="4">
         <f>F124+F133+G133+F132</f>
         <v>2000000</v>
       </c>
-      <c r="I153" s="4">
+      <c r="I154" s="4">
         <f>I124+I133+J133</f>
         <v>2050000</v>
       </c>
-      <c r="L153" s="4">
+      <c r="L154" s="4">
         <f>L124+L133+M133</f>
-        <v>2110000.0000000005</v>
-      </c>
-      <c r="O153" s="4">
+        <v>2110000</v>
+      </c>
+      <c r="O154" s="4">
         <f>O124+O133+P133</f>
         <v>2210000</v>
       </c>
-      <c r="R153" s="4">
+      <c r="R154" s="4">
         <f>R124+R133+S133</f>
-        <v>1374131.5531552718</v>
-      </c>
-      <c r="U153" s="4">
+        <v>2411332.9098842405</v>
+      </c>
+      <c r="U154" s="4">
         <f>U124+U133+V133</f>
-        <v>259692.40809697201</v>
-      </c>
-      <c r="X153" s="4">
+        <v>352388.70470186783</v>
+      </c>
+      <c r="X154" s="4">
         <f>X124+X133+Y133</f>
-        <v>91488.01273416965</v>
-      </c>
-      <c r="Z153" s="38"/>
-    </row>
-    <row r="154" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="F154" s="4">
-        <f>F153/F33</f>
+        <v>247430.57890248077</v>
+      </c>
+      <c r="Z154" s="38"/>
+    </row>
+    <row r="155" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="F155" s="4">
+        <f>F154/F33</f>
         <v>1</v>
       </c>
-      <c r="I154" s="4">
-        <f>I153/I33</f>
+      <c r="I155" s="4">
+        <f>I154/I33</f>
         <v>1</v>
       </c>
-      <c r="L154" s="4">
-        <f>L153/L33</f>
-        <v>1.0000000000000002</v>
-      </c>
-      <c r="O154" s="4">
-        <f>O153/O33</f>
+      <c r="L155" s="4">
+        <f>L154/L33</f>
         <v>1</v>
       </c>
-      <c r="R154" s="4">
-        <f>R153/R33</f>
-        <v>0.45804385105175727</v>
-      </c>
-      <c r="U154" s="4">
-        <f>U153/U33</f>
-        <v>1.038769632387888E-2</v>
-      </c>
-      <c r="X154" s="4">
-        <f>X153/X33</f>
-        <v>3.6304766958003831E-2</v>
-      </c>
-    </row>
-    <row r="159" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="AA159">
-        <v>0.1225</v>
-      </c>
-      <c r="AB159">
-        <f>SUM(AA$6:AA159)</f>
-        <v>1.2475000000000001</v>
-      </c>
-      <c r="AC159">
-        <v>20</v>
+      <c r="O155" s="4">
+        <f>O154/O33</f>
+        <v>1</v>
+      </c>
+      <c r="R155" s="4">
+        <f>R154/R33</f>
+        <v>0.80377763662808011</v>
+      </c>
+      <c r="U155" s="4">
+        <f>U154/U33</f>
+        <v>1.4095548188074713E-2</v>
+      </c>
+      <c r="X155" s="4">
+        <f>X154/X33</f>
+        <v>9.8186737659714599E-2</v>
       </c>
     </row>
     <row r="160" spans="1:29" x14ac:dyDescent="0.2">
       <c r="AA160">
-        <v>0.12239999999999999</v>
+        <v>0.1225</v>
       </c>
       <c r="AB160">
         <f>SUM(AA$6:AA160)</f>
-        <v>1.3699000000000001</v>
+        <v>1.2475000000000001</v>
       </c>
       <c r="AC160">
         <v>20</v>
@@ -12860,13 +12917,25 @@
     </row>
     <row r="161" spans="27:29" x14ac:dyDescent="0.2">
       <c r="AA161">
-        <v>0.12230000000000001</v>
+        <v>0.12239999999999999</v>
       </c>
       <c r="AB161">
         <f>SUM(AA$6:AA161)</f>
+        <v>1.3699000000000001</v>
+      </c>
+      <c r="AC161">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="162" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA162">
+        <v>0.12230000000000001</v>
+      </c>
+      <c r="AB162">
+        <f>SUM(AA$6:AA162)</f>
         <v>1.4922000000000002</v>
       </c>
-      <c r="AC161">
+      <c r="AC162">
         <v>20</v>
       </c>
     </row>
@@ -12916,4 +12985,13 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40B7113C-E57E-E340-957C-77A5927B4CD4}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
began work on new approach for setting lvst diets to allocate residuals effictively and allow for energy residual accounting
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3312DB0-35BF-4B40-AD8A-44200E17485A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D2868BA-3FEB-C140-9630-268A0A3EB0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="760" windowWidth="33780" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="9040" yWindow="760" windowWidth="33780" windowHeight="19400" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
updated varnames in carbon ledger workboook
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6869E642-61B5-724A-9F9F-F3EAE8BE1752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36EE739-1C78-174B-BB96-7938DAAAF8C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="420" yWindow="760" windowWidth="34560" windowHeight="20040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="325">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -902,9 +902,6 @@
     <t>latex variable</t>
   </si>
   <si>
-    <t>A_r(t)</t>
-  </si>
-  <si>
     <t>A(t)</t>
   </si>
   <si>
@@ -920,9 +917,6 @@
     <t>a^{(y)}_{out}(t)</t>
   </si>
   <si>
-    <t>A_r(t + 1)</t>
-  </si>
-  <si>
     <t>\chi_(t)</t>
   </si>
   <si>
@@ -935,12 +929,6 @@
     <t>\hat{\alpha}(t)</t>
   </si>
   <si>
-    <t>\bar{S}_{targ}(t)</t>
-  </si>
-  <si>
-    <t>k_0</t>
-  </si>
-  <si>
     <t>\gamma</t>
   </si>
   <si>
@@ -963,6 +951,75 @@
   </si>
   <si>
     <t>this has been modified to use a logistic ramp rather than alinear</t>
+  </si>
+  <si>
+    <t>\overline{B}_{targ}(t)</t>
+  </si>
+  <si>
+    <t>\underline{B}_{targ}(t)</t>
+  </si>
+  <si>
+    <t>\overline{B}_0</t>
+  </si>
+  <si>
+    <t>\Delta B_0</t>
+  </si>
+  <si>
+    <t>\delta(t)</t>
+  </si>
+  <si>
+    <t>A_{protected}(t)</t>
+  </si>
+  <si>
+    <t>a_{protected}(t)</t>
+  </si>
+  <si>
+    <t>A^*(t)</t>
+  </si>
+  <si>
+    <t>A^*_{protected}(t)</t>
+  </si>
+  <si>
+    <t>d(t)</t>
+  </si>
+  <si>
+    <t>A^*(t + 1)</t>
+  </si>
+  <si>
+    <t>A_{young}(t, u)</t>
+  </si>
+  <si>
+    <t>\hat{A}_{young}(t, u)</t>
+  </si>
+  <si>
+    <t>L_{young}(t, u)</t>
+  </si>
+  <si>
+    <t>\overline{Y}_{conv}(t, u)</t>
+  </si>
+  <si>
+    <t>\overline{y}_{conv}(t)</t>
+  </si>
+  <si>
+    <t>\overline{Y}_{preserved\_in\_conv}(t, u)</t>
+  </si>
+  <si>
+    <t>\overline{y}_{preserved\_in\_conv}(t)</t>
+  </si>
+  <si>
+    <t>\overline{y}_{availble\_from\_conv}(t)</t>
+  </si>
+  <si>
+    <t>\underline{Y}_{conv}(t, u)</t>
+  </si>
+  <si>
+    <t>\underline{y}_{conv}(t)</t>
+  </si>
+  <si>
+    <t>Q_0(t, u)</t>
+  </si>
+  <si>
+    <t>\overline{Y}^*(t, u)</t>
   </si>
 </sst>
 </file>
@@ -1230,11 +1287,20 @@
     <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1242,17 +1308,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1826,12 +1883,12 @@
         <v>29</v>
       </c>
       <c r="M1" s="51"/>
-      <c r="N1" s="44" t="s">
+      <c r="N1" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="47"/>
+      <c r="Q1" s="47"/>
       <c r="R1" s="51" t="s">
         <v>48</v>
       </c>
@@ -6391,16 +6448,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AC1:AH1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="R1:T1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="N1:Q1"/>
-    <mergeCell ref="AC1:AH1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="R1:T1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6420,18 +6477,18 @@
     <col min="8" max="8" width="15.1640625" style="4" customWidth="1"/>
     <col min="9" max="9" width="11.5" style="5" customWidth="1"/>
     <col min="10" max="11" width="13.33203125" style="4" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" style="5" customWidth="1"/>
-    <col min="13" max="14" width="13.33203125" style="4" customWidth="1"/>
-    <col min="15" max="15" width="21.1640625" style="5" customWidth="1"/>
-    <col min="16" max="16" width="21.1640625" style="4" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" style="5" customWidth="1"/>
-    <col min="19" max="20" width="13.33203125" style="4" customWidth="1"/>
-    <col min="21" max="21" width="9.1640625" style="5" customWidth="1"/>
-    <col min="22" max="22" width="13.33203125" style="4" customWidth="1"/>
-    <col min="23" max="23" width="12.5" style="4" customWidth="1"/>
-    <col min="24" max="24" width="9.1640625" style="5" customWidth="1"/>
-    <col min="25" max="26" width="13.33203125" style="4" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" style="5" hidden="1" customWidth="1"/>
+    <col min="13" max="14" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="21.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="21.1640625" style="4" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" style="5" hidden="1" customWidth="1"/>
+    <col min="19" max="20" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="9.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="12.5" style="4" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="9.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="25" max="26" width="13.33203125" style="4" hidden="1" customWidth="1"/>
     <col min="27" max="27" width="62.1640625" style="24" customWidth="1"/>
     <col min="28" max="30" width="14.6640625" customWidth="1"/>
     <col min="31" max="33" width="14.1640625" customWidth="1"/>
@@ -6485,10 +6542,10 @@
       <c r="H2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="I2" s="44">
+      <c r="I2" s="47">
         <v>150</v>
       </c>
-      <c r="J2" s="44"/>
+      <c r="J2" s="47"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
@@ -6519,10 +6576,10 @@
       <c r="H3" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="I3" s="44">
+      <c r="I3" s="47">
         <v>30</v>
       </c>
-      <c r="J3" s="44"/>
+      <c r="J3" s="47"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
@@ -6576,11 +6633,11 @@
         <v>6</v>
       </c>
       <c r="Z4" s="20"/>
-      <c r="AE4" s="43" t="s">
+      <c r="AE4" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="AF4" s="43"/>
-      <c r="AG4" s="43"/>
+      <c r="AF4" s="46"/>
+      <c r="AG4" s="46"/>
       <c r="AL4" t="s">
         <v>94</v>
       </c>
@@ -6596,7 +6653,7 @@
     </row>
     <row r="5" spans="1:41" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>155</v>
@@ -6610,35 +6667,35 @@
       <c r="F5" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="G5" s="42" t="s">
+      <c r="G5" s="48" t="s">
         <v>51</v>
       </c>
-      <c r="H5" s="42"/>
+      <c r="H5" s="48"/>
       <c r="I5" s="17"/>
-      <c r="J5" s="42" t="s">
+      <c r="J5" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="K5" s="42"/>
-      <c r="M5" s="42" t="s">
+      <c r="K5" s="48"/>
+      <c r="M5" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="42"/>
-      <c r="P5" s="42" t="s">
+      <c r="N5" s="48"/>
+      <c r="P5" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="Q5" s="42"/>
-      <c r="S5" s="42" t="s">
+      <c r="Q5" s="48"/>
+      <c r="S5" s="48" t="s">
         <v>83</v>
       </c>
-      <c r="T5" s="42"/>
-      <c r="V5" s="42" t="s">
+      <c r="T5" s="48"/>
+      <c r="V5" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="W5" s="42"/>
-      <c r="Y5" s="42" t="s">
+      <c r="W5" s="48"/>
+      <c r="Y5" s="48" t="s">
         <v>135</v>
       </c>
-      <c r="Z5" s="42"/>
+      <c r="Z5" s="48"/>
       <c r="AA5" s="24" t="s">
         <v>284</v>
       </c>
@@ -6799,7 +6856,7 @@
         <v>249360</v>
       </c>
       <c r="AA7" s="38" t="s">
-        <v>285</v>
+        <v>309</v>
       </c>
       <c r="AE7" s="19">
         <v>0.01</v>
@@ -6891,7 +6948,7 @@
         <v>249801</v>
       </c>
       <c r="AA8" s="38" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="AE8" s="19">
         <v>0.05</v>
@@ -6969,7 +7026,7 @@
         <v>116</v>
       </c>
       <c r="AA9" s="38" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="AE9" s="19">
         <v>0.12</v>
@@ -7033,7 +7090,7 @@
         <v>0</v>
       </c>
       <c r="AA10" s="38" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="AE10" s="19">
         <v>0.2</v>
@@ -7085,7 +7142,7 @@
         <v>0</v>
       </c>
       <c r="AA11" s="38" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="AE11" s="19">
         <v>0.2</v>
@@ -7130,7 +7187,7 @@
         <v>110</v>
       </c>
       <c r="AA12" s="38" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="AE12" s="19">
         <v>0.36</v>
@@ -7210,7 +7267,7 @@
         <v>249244</v>
       </c>
       <c r="AA13" s="38" t="s">
-        <v>291</v>
+        <v>312</v>
       </c>
       <c r="AE13" s="19"/>
       <c r="AF13" s="19"/>
@@ -7248,7 +7305,7 @@
         <v>0.7</v>
       </c>
       <c r="AA14" s="38" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="AE14" s="19">
         <v>0.6</v>
@@ -7317,7 +7374,7 @@
         <v>9</v>
       </c>
       <c r="AA15" s="38" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="AE15" s="19"/>
       <c r="AF15" s="19"/>
@@ -7325,7 +7382,7 @@
     </row>
     <row r="16" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="38" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C16" s="31"/>
       <c r="G16" s="4">
@@ -7384,7 +7441,9 @@
         <f>Z15*0.192</f>
         <v>1.728</v>
       </c>
-      <c r="AA16" s="38"/>
+      <c r="AA16" s="38" t="s">
+        <v>303</v>
+      </c>
       <c r="AE16" s="19"/>
       <c r="AF16" s="19"/>
       <c r="AG16" s="19"/>
@@ -7406,7 +7465,7 @@
         <v>0.37800893000000002</v>
       </c>
       <c r="AA17" s="38" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="AE17" s="19">
         <v>1.8</v>
@@ -7426,7 +7485,7 @@
       <c r="C18" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E18" s="41" t="s">
+      <c r="E18" s="44" t="s">
         <v>118</v>
       </c>
       <c r="F18" s="10" t="s">
@@ -7439,7 +7498,7 @@
         <v>0.47800893</v>
       </c>
       <c r="AA18" s="38" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="AE18" s="19">
         <v>3</v>
@@ -7459,7 +7518,7 @@
       <c r="C19" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E19" s="41"/>
+      <c r="E19" s="44"/>
       <c r="F19" s="10" t="s">
         <v>138</v>
       </c>
@@ -7467,7 +7526,7 @@
         <v>0.67</v>
       </c>
       <c r="AA19" s="40" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="AE19" s="19">
         <v>6</v>
@@ -7497,7 +7556,7 @@
         <v>100</v>
       </c>
       <c r="AA20" s="38" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="AE20" s="19">
         <v>10</v>
@@ -7527,7 +7586,7 @@
         <v>0.25</v>
       </c>
       <c r="AA21" s="38" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="AE21" s="19"/>
       <c r="AF21" s="19"/>
@@ -7582,7 +7641,7 @@
         <v>62.199106999999998</v>
       </c>
       <c r="AA23" s="38" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="AE23" s="19">
         <v>13.5</v>
@@ -7659,7 +7718,9 @@
       <c r="Z25" s="4">
         <v>49500</v>
       </c>
-      <c r="AA25" s="38"/>
+      <c r="AA25" s="38" t="s">
+        <v>307</v>
+      </c>
       <c r="AE25" s="19">
         <v>10</v>
       </c>
@@ -7709,7 +7770,9 @@
         <f>MAX(Z$25-Z$13, 0)</f>
         <v>0</v>
       </c>
-      <c r="AA26" s="38"/>
+      <c r="AA26" s="38" t="s">
+        <v>308</v>
+      </c>
       <c r="AE26" s="19">
         <v>6</v>
       </c>
@@ -7787,7 +7850,9 @@
         <f>MIN(Z13,Z25)</f>
         <v>49500</v>
       </c>
-      <c r="AA27" s="38"/>
+      <c r="AA27" s="38" t="s">
+        <v>310</v>
+      </c>
       <c r="AE27" s="19">
         <v>3</v>
       </c>
@@ -7835,7 +7900,7 @@
       <c r="C29" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E29" s="41" t="s">
+      <c r="E29" s="44" t="s">
         <v>170</v>
       </c>
       <c r="F29" s="25" t="s">
@@ -7847,7 +7912,9 @@
       <c r="H29" s="4">
         <v>0.92</v>
       </c>
-      <c r="AA29" s="38"/>
+      <c r="AA29" s="38" t="s">
+        <v>305</v>
+      </c>
     </row>
     <row r="30" spans="2:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="38" t="s">
@@ -7856,7 +7923,7 @@
       <c r="C30" s="32" t="s">
         <v>174</v>
       </c>
-      <c r="E30" s="41"/>
+      <c r="E30" s="44"/>
       <c r="F30" s="25" t="s">
         <v>171</v>
       </c>
@@ -7872,7 +7939,9 @@
         <f>G29/G20</f>
         <v>2E-3</v>
       </c>
-      <c r="AA30" s="38"/>
+      <c r="AA30" s="38" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="31" spans="2:33" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E31" s="26"/>
@@ -7927,7 +7996,9 @@
       <c r="Y33" s="4">
         <v>2520000</v>
       </c>
-      <c r="AA33" s="38"/>
+      <c r="AA33" s="38" t="s">
+        <v>311</v>
+      </c>
     </row>
     <row r="35" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="F35" s="11" t="s">
@@ -8023,10 +8094,10 @@
       </c>
     </row>
     <row r="38" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B38" s="46" t="s">
+      <c r="B38" s="41" t="s">
         <v>180</v>
       </c>
-      <c r="C38" s="45" t="s">
+      <c r="C38" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F38" s="14" t="s">
@@ -8114,8 +8185,8 @@
       <c r="AA38" s="37"/>
     </row>
     <row r="39" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B39" s="47"/>
-      <c r="C39" s="45"/>
+      <c r="B39" s="43"/>
+      <c r="C39" s="42"/>
       <c r="F39" s="14" t="s">
         <v>69</v>
       </c>
@@ -8197,11 +8268,13 @@
         <f>W39-Y39</f>
         <v>80</v>
       </c>
-      <c r="AA39" s="38"/>
+      <c r="AA39" s="38" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="40" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B40" s="47"/>
-      <c r="C40" s="45"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="42"/>
       <c r="F40" s="14" t="s">
         <v>79</v>
       </c>
@@ -8282,11 +8355,13 @@
         <f>W40-Y40</f>
         <v>92</v>
       </c>
-      <c r="AA40" s="38"/>
+      <c r="AA40" s="38" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="41" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B41" s="47"/>
-      <c r="C41" s="45"/>
+      <c r="B41" s="43"/>
+      <c r="C41" s="42"/>
       <c r="F41" s="14" t="s">
         <v>80</v>
       </c>
@@ -8366,7 +8441,9 @@
         <f>W41-Y41</f>
         <v>43</v>
       </c>
-      <c r="AA41" s="38"/>
+      <c r="AA41" s="38" t="s">
+        <v>315</v>
+      </c>
     </row>
     <row r="42" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="F42" s="14" t="s">
@@ -8377,10 +8454,10 @@
       </c>
     </row>
     <row r="43" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B43" s="47" t="s">
+      <c r="B43" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="C43" s="45" t="s">
+      <c r="C43" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F43" s="14" t="s">
@@ -8416,8 +8493,8 @@
       <c r="AA43" s="38"/>
     </row>
     <row r="44" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B44" s="47"/>
-      <c r="C44" s="45"/>
+      <c r="B44" s="43"/>
+      <c r="C44" s="42"/>
       <c r="F44" s="14" t="s">
         <v>196</v>
       </c>
@@ -8448,11 +8525,13 @@
         <f>IF(W39=0, 0, W97*Y39/W39)</f>
         <v>0</v>
       </c>
-      <c r="AA44" s="38"/>
+      <c r="AA44" s="38" t="s">
+        <v>316</v>
+      </c>
     </row>
     <row r="45" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B45" s="47"/>
-      <c r="C45" s="45"/>
+      <c r="B45" s="43"/>
+      <c r="C45" s="42"/>
       <c r="F45" s="14" t="s">
         <v>197</v>
       </c>
@@ -8486,8 +8565,8 @@
       <c r="AA45" s="38"/>
     </row>
     <row r="46" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B46" s="47"/>
-      <c r="C46" s="45"/>
+      <c r="B46" s="43"/>
+      <c r="C46" s="42"/>
       <c r="F46" s="14" t="s">
         <v>198</v>
       </c>
@@ -8556,7 +8635,9 @@
         <f>SUM(Z43:Z46)</f>
         <v>0</v>
       </c>
-      <c r="AA47" s="38"/>
+      <c r="AA47" s="38" t="s">
+        <v>317</v>
+      </c>
     </row>
     <row r="48" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="F48" s="14" t="s">
@@ -8567,13 +8648,13 @@
       </c>
     </row>
     <row r="49" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B49" s="47" t="s">
+      <c r="B49" s="43" t="s">
         <v>263</v>
       </c>
-      <c r="C49" s="45" t="s">
+      <c r="C49" s="42" t="s">
         <v>174</v>
       </c>
-      <c r="E49" s="41" t="s">
+      <c r="E49" s="44" t="s">
         <v>251</v>
       </c>
       <c r="F49" s="14" t="s">
@@ -8607,12 +8688,14 @@
         <f>MIN(Z43,Z$15*Y38)</f>
         <v>0</v>
       </c>
-      <c r="AA49" s="38"/>
+      <c r="AA49" s="38" t="s">
+        <v>318</v>
+      </c>
     </row>
     <row r="50" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B50" s="47"/>
-      <c r="C50" s="45"/>
-      <c r="E50" s="41"/>
+      <c r="B50" s="43"/>
+      <c r="C50" s="42"/>
+      <c r="E50" s="44"/>
       <c r="F50" s="14" t="s">
         <v>252</v>
       </c>
@@ -8647,9 +8730,9 @@
       <c r="AA50" s="38"/>
     </row>
     <row r="51" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B51" s="47"/>
-      <c r="C51" s="45"/>
-      <c r="E51" s="41"/>
+      <c r="B51" s="43"/>
+      <c r="C51" s="42"/>
+      <c r="E51" s="44"/>
       <c r="F51" s="14" t="s">
         <v>253</v>
       </c>
@@ -8684,9 +8767,9 @@
       <c r="AA51" s="38"/>
     </row>
     <row r="52" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B52" s="47"/>
-      <c r="C52" s="45"/>
-      <c r="E52" s="41"/>
+      <c r="B52" s="43"/>
+      <c r="C52" s="42"/>
+      <c r="E52" s="44"/>
       <c r="F52" s="14" t="s">
         <v>254</v>
       </c>
@@ -8756,7 +8839,9 @@
         <f>SUM(Z49:Z52)</f>
         <v>0</v>
       </c>
-      <c r="AA53" s="38"/>
+      <c r="AA53" s="38" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="54" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B54" s="38" t="s">
@@ -8792,16 +8877,18 @@
         <f>Z47-Z53</f>
         <v>0</v>
       </c>
-      <c r="AA54" s="38"/>
+      <c r="AA54" s="38" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="55" spans="2:27" x14ac:dyDescent="0.2">
       <c r="F55" s="14"/>
     </row>
     <row r="56" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B56" s="47" t="s">
+      <c r="B56" s="43" t="s">
         <v>193</v>
       </c>
-      <c r="C56" s="45" t="s">
+      <c r="C56" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F56" s="14" t="s">
@@ -8835,11 +8922,13 @@
         <f>Z43*$H$21</f>
         <v>0</v>
       </c>
-      <c r="AA56" s="38"/>
+      <c r="AA56" s="38" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="57" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B57" s="47"/>
-      <c r="C57" s="45"/>
+      <c r="B57" s="43"/>
+      <c r="C57" s="42"/>
       <c r="F57" s="14" t="s">
         <v>200</v>
       </c>
@@ -8874,8 +8963,8 @@
       <c r="AA57" s="38"/>
     </row>
     <row r="58" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B58" s="47"/>
-      <c r="C58" s="45"/>
+      <c r="B58" s="43"/>
+      <c r="C58" s="42"/>
       <c r="F58" s="14" t="s">
         <v>201</v>
       </c>
@@ -8910,8 +8999,8 @@
       <c r="AA58" s="38"/>
     </row>
     <row r="59" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B59" s="47"/>
-      <c r="C59" s="45"/>
+      <c r="B59" s="43"/>
+      <c r="C59" s="42"/>
       <c r="F59" s="14" t="s">
         <v>202</v>
       </c>
@@ -8981,16 +9070,18 @@
         <f>SUM(Z56:Z59)</f>
         <v>0</v>
       </c>
-      <c r="AA60" s="38"/>
+      <c r="AA60" s="38" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="61" spans="2:27" x14ac:dyDescent="0.2">
       <c r="F61" s="14"/>
     </row>
     <row r="62" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B62" s="47" t="s">
+      <c r="B62" s="43" t="s">
         <v>178</v>
       </c>
-      <c r="C62" s="45" t="s">
+      <c r="C62" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F62" s="14" t="s">
@@ -9024,11 +9115,13 @@
         <f>AE14</f>
         <v>0.6</v>
       </c>
-      <c r="AA62" s="38"/>
+      <c r="AA62" s="38" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="63" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B63" s="47"/>
-      <c r="C63" s="45"/>
+      <c r="B63" s="43"/>
+      <c r="C63" s="42"/>
       <c r="F63" s="14" t="s">
         <v>91</v>
       </c>
@@ -9061,8 +9154,8 @@
       <c r="AA63" s="38"/>
     </row>
     <row r="64" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B64" s="47"/>
-      <c r="C64" s="45"/>
+      <c r="B64" s="43"/>
+      <c r="C64" s="42"/>
       <c r="F64" s="14" t="s">
         <v>92</v>
       </c>
@@ -9094,8 +9187,8 @@
       <c r="AA64" s="38"/>
     </row>
     <row r="65" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B65" s="47"/>
-      <c r="C65" s="45"/>
+      <c r="B65" s="43"/>
+      <c r="C65" s="42"/>
       <c r="F65" s="14" t="s">
         <v>93</v>
       </c>
@@ -9134,10 +9227,10 @@
       <c r="F67" s="14"/>
     </row>
     <row r="68" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B68" s="47" t="s">
+      <c r="B68" s="43" t="s">
         <v>238</v>
       </c>
-      <c r="C68" s="45" t="s">
+      <c r="C68" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F68" s="14" t="s">
@@ -9171,11 +9264,13 @@
         <f>W68*(1- $G$30)+Z38*Z62</f>
         <v>113.71737449773644</v>
       </c>
-      <c r="AA68" s="38"/>
+      <c r="AA68" s="38" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="69" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B69" s="47"/>
-      <c r="C69" s="45"/>
+      <c r="B69" s="43"/>
+      <c r="C69" s="42"/>
       <c r="F69" s="14" t="s">
         <v>110</v>
       </c>
@@ -9206,9 +9301,9 @@
       <c r="AA69" s="38"/>
     </row>
     <row r="70" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B70" s="47"/>
-      <c r="C70" s="45"/>
-      <c r="E70" s="41"/>
+      <c r="B70" s="43"/>
+      <c r="C70" s="42"/>
+      <c r="E70" s="44"/>
       <c r="F70" s="14" t="s">
         <v>111</v>
       </c>
@@ -9235,9 +9330,9 @@
       <c r="AA70" s="38"/>
     </row>
     <row r="71" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B71" s="47"/>
-      <c r="C71" s="45"/>
-      <c r="E71" s="41"/>
+      <c r="B71" s="43"/>
+      <c r="C71" s="42"/>
+      <c r="E71" s="44"/>
       <c r="F71" s="14" t="s">
         <v>112</v>
       </c>
@@ -9264,14 +9359,14 @@
       <c r="AA71" s="38"/>
     </row>
     <row r="72" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="E72" s="41"/>
+      <c r="E72" s="44"/>
       <c r="F72" s="14"/>
     </row>
     <row r="73" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B73" s="47" t="s">
+      <c r="B73" s="43" t="s">
         <v>235</v>
       </c>
-      <c r="C73" s="45" t="s">
+      <c r="C73" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F73" s="14" t="s">
@@ -9307,8 +9402,8 @@
       <c r="AA73" s="38"/>
     </row>
     <row r="74" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B74" s="47"/>
-      <c r="C74" s="45"/>
+      <c r="B74" s="43"/>
+      <c r="C74" s="42"/>
       <c r="F74" s="14" t="s">
         <v>128</v>
       </c>
@@ -9342,9 +9437,9 @@
       <c r="AA74" s="38"/>
     </row>
     <row r="75" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B75" s="47"/>
-      <c r="C75" s="45"/>
-      <c r="E75" s="41" t="s">
+      <c r="B75" s="43"/>
+      <c r="C75" s="42"/>
+      <c r="E75" s="44" t="s">
         <v>152</v>
       </c>
       <c r="F75" s="14" t="s">
@@ -9380,9 +9475,9 @@
       <c r="AA75" s="38"/>
     </row>
     <row r="76" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B76" s="47"/>
-      <c r="C76" s="45"/>
-      <c r="E76" s="41"/>
+      <c r="B76" s="43"/>
+      <c r="C76" s="42"/>
+      <c r="E76" s="44"/>
       <c r="F76" s="14" t="s">
         <v>130</v>
       </c>
@@ -9422,7 +9517,7 @@
       <c r="C77" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="E77" s="41"/>
+      <c r="E77" s="44"/>
       <c r="F77" s="14" t="s">
         <v>147</v>
       </c>
@@ -9459,7 +9554,7 @@
       </c>
     </row>
     <row r="78" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="E78" s="41"/>
+      <c r="E78" s="44"/>
       <c r="F78" s="14"/>
       <c r="AD78" t="s">
         <v>85</v>
@@ -9469,10 +9564,10 @@
       </c>
     </row>
     <row r="79" spans="2:32" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B79" s="48" t="s">
+      <c r="B79" s="45" t="s">
         <v>237</v>
       </c>
-      <c r="C79" s="45" t="s">
+      <c r="C79" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F79" s="14" t="s">
@@ -9505,8 +9600,8 @@
       </c>
     </row>
     <row r="80" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B80" s="48"/>
-      <c r="C80" s="45"/>
+      <c r="B80" s="45"/>
+      <c r="C80" s="42"/>
       <c r="F80" s="14" t="s">
         <v>148</v>
       </c>
@@ -9569,8 +9664,8 @@
       <c r="AA80" s="39"/>
     </row>
     <row r="81" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B81" s="48"/>
-      <c r="C81" s="45"/>
+      <c r="B81" s="45"/>
+      <c r="C81" s="42"/>
       <c r="E81" s="22">
         <v>0</v>
       </c>
@@ -9636,8 +9731,8 @@
       <c r="AA81" s="39"/>
     </row>
     <row r="82" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B82" s="48"/>
-      <c r="C82" s="45"/>
+      <c r="B82" s="45"/>
+      <c r="C82" s="42"/>
       <c r="E82" s="22">
         <v>1</v>
       </c>
@@ -9703,8 +9798,8 @@
       <c r="AA82" s="39"/>
     </row>
     <row r="83" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B83" s="48"/>
-      <c r="C83" s="45"/>
+      <c r="B83" s="45"/>
+      <c r="C83" s="42"/>
       <c r="E83" s="22">
         <v>2</v>
       </c>
@@ -9797,10 +9892,10 @@
       </c>
     </row>
     <row r="86" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B86" s="46" t="s">
+      <c r="B86" s="41" t="s">
         <v>181</v>
       </c>
-      <c r="C86" s="45" t="s">
+      <c r="C86" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F86" s="14" t="s">
@@ -9861,8 +9956,8 @@
       <c r="AA86" s="37"/>
     </row>
     <row r="87" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B87" s="46"/>
-      <c r="C87" s="45"/>
+      <c r="B87" s="41"/>
+      <c r="C87" s="42"/>
       <c r="F87" s="14" t="s">
         <v>132</v>
       </c>
@@ -9921,8 +10016,8 @@
       <c r="AA87" s="37"/>
     </row>
     <row r="88" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B88" s="46"/>
-      <c r="C88" s="45"/>
+      <c r="B88" s="41"/>
+      <c r="C88" s="42"/>
       <c r="F88" s="14" t="s">
         <v>133</v>
       </c>
@@ -9981,8 +10076,8 @@
       <c r="AA88" s="37"/>
     </row>
     <row r="89" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B89" s="46"/>
-      <c r="C89" s="45"/>
+      <c r="B89" s="41"/>
+      <c r="C89" s="42"/>
       <c r="F89" s="14" t="s">
         <v>134</v>
       </c>
@@ -10044,10 +10139,10 @@
       <c r="F90" s="14"/>
     </row>
     <row r="91" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B91" s="46" t="s">
+      <c r="B91" s="41" t="s">
         <v>204</v>
       </c>
-      <c r="C91" s="45" t="s">
+      <c r="C91" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F91" s="14" t="s">
@@ -10084,8 +10179,8 @@
       <c r="AA91" s="37"/>
     </row>
     <row r="92" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B92" s="46"/>
-      <c r="C92" s="45"/>
+      <c r="B92" s="41"/>
+      <c r="C92" s="42"/>
       <c r="F92" s="14" t="s">
         <v>206</v>
       </c>
@@ -10120,8 +10215,8 @@
       <c r="AA92" s="37"/>
     </row>
     <row r="93" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B93" s="46"/>
-      <c r="C93" s="45"/>
+      <c r="B93" s="41"/>
+      <c r="C93" s="42"/>
       <c r="F93" s="14" t="s">
         <v>207</v>
       </c>
@@ -10156,8 +10251,8 @@
       <c r="AA93" s="37"/>
     </row>
     <row r="94" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B94" s="46"/>
-      <c r="C94" s="45"/>
+      <c r="B94" s="41"/>
+      <c r="C94" s="42"/>
       <c r="F94" s="14" t="s">
         <v>208</v>
       </c>
@@ -10195,10 +10290,10 @@
       <c r="F95" s="14"/>
     </row>
     <row r="96" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B96" s="46" t="s">
+      <c r="B96" s="41" t="s">
         <v>209</v>
       </c>
-      <c r="C96" s="45" t="s">
+      <c r="C96" s="42" t="s">
         <v>174</v>
       </c>
       <c r="F96" s="14" t="s">
@@ -10235,8 +10330,8 @@
       <c r="AA96" s="37"/>
     </row>
     <row r="97" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B97" s="46"/>
-      <c r="C97" s="45"/>
+      <c r="B97" s="41"/>
+      <c r="C97" s="42"/>
       <c r="F97" s="14" t="s">
         <v>71</v>
       </c>
@@ -10271,8 +10366,8 @@
       <c r="AA97" s="37"/>
     </row>
     <row r="98" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B98" s="46"/>
-      <c r="C98" s="45"/>
+      <c r="B98" s="41"/>
+      <c r="C98" s="42"/>
       <c r="F98" s="14" t="s">
         <v>72</v>
       </c>
@@ -10307,8 +10402,8 @@
       <c r="AA98" s="37"/>
     </row>
     <row r="99" spans="2:27" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="46"/>
-      <c r="C99" s="45"/>
+      <c r="B99" s="41"/>
+      <c r="C99" s="42"/>
       <c r="F99" s="14" t="s">
         <v>81</v>
       </c>
@@ -10347,10 +10442,10 @@
       <c r="F100" s="14"/>
     </row>
     <row r="101" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B101" s="46" t="s">
+      <c r="B101" s="41" t="s">
         <v>210</v>
       </c>
-      <c r="C101" s="45" t="s">
+      <c r="C101" s="42" t="s">
         <v>174</v>
       </c>
       <c r="E101" s="26"/>
@@ -10388,8 +10483,8 @@
       <c r="AA101" s="37"/>
     </row>
     <row r="102" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B102" s="46"/>
-      <c r="C102" s="45"/>
+      <c r="B102" s="41"/>
+      <c r="C102" s="42"/>
       <c r="E102" s="26"/>
       <c r="F102" s="14" t="s">
         <v>212</v>
@@ -10425,8 +10520,8 @@
       <c r="AA102" s="37"/>
     </row>
     <row r="103" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B103" s="46"/>
-      <c r="C103" s="45"/>
+      <c r="B103" s="41"/>
+      <c r="C103" s="42"/>
       <c r="E103" s="26"/>
       <c r="F103" s="14" t="s">
         <v>213</v>
@@ -10462,8 +10557,8 @@
       <c r="AA103" s="37"/>
     </row>
     <row r="104" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B104" s="46"/>
-      <c r="C104" s="45"/>
+      <c r="B104" s="41"/>
+      <c r="C104" s="42"/>
       <c r="E104" s="26"/>
       <c r="F104" s="14" t="s">
         <v>214</v>
@@ -10724,7 +10819,7 @@
         <v>0.86560925711218095</v>
       </c>
       <c r="AA110" s="38" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="111" spans="2:27" ht="17" x14ac:dyDescent="0.2">
@@ -12059,7 +12154,7 @@
     </row>
     <row r="137" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B137" s="38" t="s">
         <v>186</v>
@@ -12455,7 +12550,7 @@
     </row>
     <row r="145" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B145" s="38" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="C145" s="33" t="s">
         <v>163</v>
@@ -12724,7 +12819,7 @@
     </row>
     <row r="149" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B149" s="38" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="C149" s="33" t="s">
         <v>163</v>
@@ -12953,6 +13048,30 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="E70:E72"/>
+    <mergeCell ref="E75:E78"/>
+    <mergeCell ref="Y5:Z5"/>
+    <mergeCell ref="P5:Q5"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="V5:W5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="AE4:AG4"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="B68:B71"/>
+    <mergeCell ref="C68:C71"/>
+    <mergeCell ref="C43:C46"/>
+    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="C56:C59"/>
     <mergeCell ref="B101:B104"/>
     <mergeCell ref="C101:C104"/>
     <mergeCell ref="B49:B52"/>
@@ -12968,30 +13087,6 @@
     <mergeCell ref="B73:B76"/>
     <mergeCell ref="C73:C76"/>
     <mergeCell ref="B86:B89"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="B68:B71"/>
-    <mergeCell ref="C68:C71"/>
-    <mergeCell ref="C43:C46"/>
-    <mergeCell ref="B43:B46"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="B56:B59"/>
-    <mergeCell ref="C56:C59"/>
-    <mergeCell ref="AE4:AG4"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="E70:E72"/>
-    <mergeCell ref="E75:E78"/>
-    <mergeCell ref="Y5:Z5"/>
-    <mergeCell ref="P5:Q5"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="V5:W5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E29:E30"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
continued work updating descriptions of variables and variable mathematical notations in carbon ledger workbook
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADD75E4-B89C-564A-AF5D-2C1999A2946F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3412FEB-9A56-694D-B6C0-0872A89E70D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-320" yWindow="760" windowWidth="34560" windowHeight="20040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="2060" yWindow="500" windowWidth="34560" windowHeight="19560" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="432">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -583,10 +583,6 @@
     <t>T = number of time periods</t>
   </si>
   <si>
-    <t>arr_young_sf_adjusted_by_tp_planted (T x T)   [e.g., col J]
-arr_young_sf_adjustment_factor (T x T)   [e.g., col I]</t>
-  </si>
-  <si>
     <t>(ref to above)</t>
   </si>
   <si>
@@ -752,10 +748,6 @@
     <t>vec_young_biomass_c_available_for_removals_total</t>
   </si>
   <si>
-    <t>arr_young_biomass_c_stock_removal_allocation (T x T)   [e.g., col G]
-arr_young_biomass_c_stock_removal_allocation_aux (T x T)   [e.g., col F]</t>
-  </si>
-  <si>
     <t>arr_young_biomass_c_ag_stock_if_untouched (T x T)</t>
   </si>
   <si>
@@ -909,9 +901,6 @@
     <t>a^{(y)}_{out}(t)</t>
   </si>
   <si>
-    <t>\chi_(t)</t>
-  </si>
-  <si>
     <t>\check{\alpha}(t)</t>
   </si>
   <si>
@@ -927,9 +916,6 @@
     <t>k_{heav}</t>
   </si>
   <si>
-    <t>rrr</t>
-  </si>
-  <si>
     <t>arr_biomass_c_average_bg_stock_in_conversion_targets</t>
   </si>
   <si>
@@ -945,18 +931,9 @@
     <t>this has been modified to use a logistic ramp rather than alinear</t>
   </si>
   <si>
-    <t>\overline{B}_{targ}(t)</t>
-  </si>
-  <si>
-    <t>\underline{B}_{targ}(t)</t>
-  </si>
-  <si>
     <t>\overline{B}_0</t>
   </si>
   <si>
-    <t>\Delta B_0</t>
-  </si>
-  <si>
     <t>\delta(t)</t>
   </si>
   <si>
@@ -975,54 +952,24 @@
     <t>\overline{y}_{conv}(t)</t>
   </si>
   <si>
-    <t>\overline{Y}_{preserved\_in\_conv}(t, u)</t>
-  </si>
-  <si>
-    <t>\overline{y}_{preserved\_in\_conv}(t)</t>
-  </si>
-  <si>
-    <t>\overline{y}_{availble\_from\_conv}(t)</t>
-  </si>
-  <si>
     <t>\underline{Y}_{conv}(t, u)</t>
   </si>
   <si>
     <t>\underline{y}_{conv}(t)</t>
   </si>
   <si>
-    <t>Q_0(t, u)</t>
-  </si>
-  <si>
     <t>\overline{Y}^*(t, u)</t>
   </si>
   <si>
-    <t>A^{young}(t, u)</t>
-  </si>
-  <si>
-    <t>\hat{A}^{young}(t, u)</t>
-  </si>
-  <si>
-    <t>L^{young}(t, u)</t>
-  </si>
-  <si>
     <t>A^{(protected)}(t)</t>
   </si>
   <si>
     <t>a^{(protected)}(t)</t>
   </si>
   <si>
-    <t>A^{(*protected)}(t)</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
-    <t>Average below ground stock contained In land use classes that forests transition into; used to estimate below-ground conversion losses of stock.</t>
-  </si>
-  <si>
-    <t>Average above ground stock contained In land use classes that forests transition into; used to estimate above-ground conversion losses of stock.</t>
-  </si>
-  <si>
     <t>Fraction of biomass that represents dead storage. Is set in SISEPUEDE to be max of exogenous specification and amount implied by average stock in conversion targets (cannot have biomass below transition targets and remain forest).</t>
   </si>
   <si>
@@ -1074,9 +1021,6 @@
     <t>Area of remaining (from simulation initialization) forest that is protected.</t>
   </si>
   <si>
-    <t>Nominal sequestration factor (mass of biomass growth per time period) associated with forests. Used in NPP fit from integration target.</t>
-  </si>
-  <si>
     <t>Fraction of biomass per time period lost to decomposition. This is estimated from the NPP fit funtion under the assumption that primary forests exist in steady state (i.e., that there is no net growth of biomass if left undistributed).</t>
   </si>
   <si>
@@ -1098,9 +1042,6 @@
     <t>arr_young_area_by_tp_planted_drops (T x T)   [e.g., col J]</t>
   </si>
   <si>
-    <t>Matrix ($T \times T$) storing how much area of young forest planted in time $t$ remains in time $u$</t>
-  </si>
-  <si>
     <t>Matrix ($T \times T$) storing how much forest area in each time period (column $u$) has to be dropped due to conversion into young forests. Only applicable if all other secondary forest has been elimnated.</t>
   </si>
   <si>
@@ -1117,6 +1058,285 @@
   </si>
   <si>
     <t>Vector ($T$) storing total above-ground mass of biomass preserved in each time period.</t>
+  </si>
+  <si>
+    <t>Vector ($T$) storing total biomass from conversion that is available to satisfy harvested wood product (HWP) and fuelwood (FW) demands.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix ($T \times T$) storing total young biomass that is converted to other (non-forest) land use types by time period planted. </t>
+  </si>
+  <si>
+    <t>Vector ($T$)  storing total young biomass that is converted to other (non-forest) land use types at time $t$.</t>
+  </si>
+  <si>
+    <t>K_{avail}(t, u)</t>
+  </si>
+  <si>
+    <t>k_{avail}(T)</t>
+  </si>
+  <si>
+    <t>Vector ($T$) storing how much biomass is available at time $t$ from young forests.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) used to determine whether young biomass is available for harvest. Determined based on number of years of growth required to make biomass available.</t>
+  </si>
+  <si>
+    <t>arr_young_biomass_c_stock_removal_allocation_aux (T x T)   [e.g., col F]</t>
+  </si>
+  <si>
+    <t>arr_young_biomass_c_stock_removal_allocation (T x T)   [e.g., col G]</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) storing counterfactual for young biomass above-ground stock if untouched at time $t$ for biomass planted at time $u$.</t>
+  </si>
+  <si>
+    <t>\overline{Y}_{alloc}(t, u)</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) storing total above-ground mass of biomas allocated for removal in time $t$ from biomass planted at time $u$.</t>
+  </si>
+  <si>
+    <t>\overline{Y}_{alloc\_aux}(t, u)</t>
+  </si>
+  <si>
+    <t>arr_young_sf_adjusted_by_tp_planted (T x T)   [e.g., col J]</t>
+  </si>
+  <si>
+    <t>arr_young_sf_adjustment_factor (T x T)   [e.g., col I]</t>
+  </si>
+  <si>
+    <t>\Psi^{(y)}(t, u)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix ($T \times T$) storing the adjustment factor for young forest factors; applied to unadjusted yuong forest sequestration factor $R^{(y)}_0(t, u)$ based on depletion leevels. </t>
+  </si>
+  <si>
+    <t>\overline{Y}(t, u)</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) storing total above-ground biomass stock at time $t$ for young forests planted at time $u$.</t>
+  </si>
+  <si>
+    <t>\Delta_0\overline{Y}(t, u)</t>
+  </si>
+  <si>
+    <t>\Delta\overline{Y}(t, u)</t>
+  </si>
+  <si>
+    <t>\underline{Y}(t, u)</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) storing total below-ground biomass stock at time $t$ for young forests planted at time $u$.</t>
+  </si>
+  <si>
+    <t>D^{(y)}(t, u)</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) storing the loss of biomass in young forests due to decomposition. Decomposition rates are determined as a function of the NPP curve and an assumption that primary forests are in steady state.</t>
+  </si>
+  <si>
+    <t>A^{(y)}(t, u)</t>
+  </si>
+  <si>
+    <t>\hat{A}^{(y)}(t, u)</t>
+  </si>
+  <si>
+    <t>L^{(y)}(t, u)</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) used in auxialiary calculations for total above-ground mass of biomas allocated for removal in time $t$ from biomass planted at time $u$.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) storing the sequestration factors (which come from AFOLU NPP curve estimates) for unperturbed young forests by time period planted.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) storing the adjusted sequestration factors (which come from AFOLU NPP curve estimates) for forests by time period planted. Adjustments are based off of the level of average stock depletion.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times T$) storing how much area of young forest planted in time $t$ remains in time $u$.</t>
+  </si>
+  <si>
+    <t>\chi(t)</t>
+  </si>
+  <si>
+    <t>\overline{M}_0^*</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing initial (start of simulation) above ground biomass stock.</t>
+  </si>
+  <si>
+    <t>\Delta B</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing sequestration factor in original forests (as adjusted due to degradation).</t>
+  </si>
+  <si>
+    <t>\overline{M}_0</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing above ground biomass stock left from start of simulation if untouched (without degradation).</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing biomass stock remaining from forests present at the start of the simulation.</t>
+  </si>
+  <si>
+    <t>\overline{\overline{B}}</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing average (mass per unit area) biomass stock remaining from forests present at the start of the simulation.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing average (mass per unit area) biomass stock remaining from forests present at the start of the simulation \emph{excluding} dead storage.</t>
+  </si>
+  <si>
+    <t>\overline{y}(t)</t>
+  </si>
+  <si>
+    <t>\overline{m}(t)</t>
+  </si>
+  <si>
+    <t>\underline{m}(t)</t>
+  </si>
+  <si>
+    <t>Vector ($T$) storing total above-ground biomass stock in young forests at the start of time period $t$.</t>
+  </si>
+  <si>
+    <t>Vector ($T$) storing total above-ground biomass stock in all forests at the start of time period $t$.</t>
+  </si>
+  <si>
+    <t>Vector ($T$) storing total below-ground biomass stock in all forests at the start of time period $t$.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing total mass of biomass from original forests converted away in each time period.</t>
+  </si>
+  <si>
+    <t>\Delta_0\overline{b}</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing average above ground stock contained In land use classes that forests transition into; used to estimate above-ground conversion losses of stock.</t>
+  </si>
+  <si>
+    <t>\overline{G}</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) soring average below ground stock contained In land use classes that forests transition into; used to estimate below-ground conversion losses of stock.</t>
+  </si>
+  <si>
+    <t>\underline{G}</t>
+  </si>
+  <si>
+    <t>Vector (length 2) storing nominal sequestration factor (mass of biomass growth per time period) associated with forests. Used in NPP fit from integration target.</t>
+  </si>
+  <si>
+    <t>\overline{b}_{conv}(t)</t>
+  </si>
+  <si>
+    <t>\overline{y}_{availconv}(t)</t>
+  </si>
+  <si>
+    <t>\overline{y}_{presconv}(t)</t>
+  </si>
+  <si>
+    <t>\overline{Y}_{presconv}(t, u)</t>
+  </si>
+  <si>
+    <t>\overline{b}_{presconv}(t)</t>
+  </si>
+  <si>
+    <t>\overline{b}_{availconv}(t)</t>
+  </si>
+  <si>
+    <t>r_{conv}(t)</t>
+  </si>
+  <si>
+    <t>Mass of biomass removals from converted land at time $t$.</t>
+  </si>
+  <si>
+    <t>Row-stochastic matrix ($T \times 2$) storing allocation of removals by forest type (column) at time $t$ (row).</t>
+  </si>
+  <si>
+    <t>\Phi_{conv}</t>
+  </si>
+  <si>
+    <t>A^{(0)}_{avail}</t>
+  </si>
+  <si>
+    <t>Matrix storing total biomass available (i.e., excluding dead storage) in original forests by type (column) excluding land converted out at time period $t$. Excludes young forests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vector ($T$) storing demand for removals from all forests, excluding those from conversions. </t>
+  </si>
+  <si>
+    <t>d_{rmv}</t>
+  </si>
+  <si>
+    <t>u^{(0)}_{rmv}</t>
+  </si>
+  <si>
+    <t>Vector ($T$) storing unmet demand for removals from original forests.</t>
+  </si>
+  <si>
+    <t>r^{(0)}_{rmv}</t>
+  </si>
+  <si>
+    <t>r^{(y)}_{rmv}</t>
+  </si>
+  <si>
+    <t>R^{(0)}_{rmv}</t>
+  </si>
+  <si>
+    <t>R_{rmv}</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing removals from original forests by type (columns), excluding conversions.</t>
+  </si>
+  <si>
+    <t>Vector ($T$) storing removals from young forests, excluding conversions.  Always $\leq d_{rmv}$.</t>
+  </si>
+  <si>
+    <t>Vector ($T$) storing removals from original forests, excluding conversions.  Always $\leq d_{rmv}$.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) storing removals from all forests byt ype (columns), excluding conversions. Removals from young secondary forests are added to those removals from original secondary forests.</t>
+  </si>
+  <si>
+    <t>\overline{\overline{B}}'</t>
+  </si>
+  <si>
+    <t>A^{(protected)*}(t)</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) giving fraction of original forest stock available when compared to healthy (unperturbed) baseline.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) giving fraction of removals satisfiable at time $t$ for forest type $v$.</t>
+  </si>
+  <si>
+    <t>\tilde{A}^{(0)}_{avail}</t>
+  </si>
+  <si>
+    <t>\tilde{a}^{(0)}</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) giving adjusted--based on availability in buffer zone--quantity of biomass available for removals by forest type.</t>
+  </si>
+  <si>
+    <t>Vector ($T $) giving adjusted--based on availability in buffer zone--total quantity of biomass available for removals.</t>
+  </si>
+  <si>
+    <t>Matrix ($T \times 2$) giving allocation of adjusted--based on availability in buffer zone--quantity of biomass available for removals by forest type.</t>
+  </si>
+  <si>
+    <t>\Phi_{avail}</t>
+  </si>
+  <si>
+    <t>\Psi^{(0)}_{seq}</t>
+  </si>
+  <si>
+    <t>\Psi^{(0)}_{rmvsat}</t>
+  </si>
+  <si>
+    <t>S^{(0)}(t, v)</t>
   </si>
 </sst>
 </file>
@@ -1270,7 +1490,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1378,9 +1598,6 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1405,9 +1622,6 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1425,6 +1639,15 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1961,60 +2184,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="50" t="s">
+      <c r="B1" s="47"/>
+      <c r="C1" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="49" t="s">
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="50" t="s">
+      <c r="G1" s="47"/>
+      <c r="H1" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="50"/>
-      <c r="J1" s="49" t="s">
+      <c r="I1" s="48"/>
+      <c r="J1" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="49"/>
-      <c r="L1" s="51" t="s">
+      <c r="K1" s="47"/>
+      <c r="L1" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="M1" s="51"/>
-      <c r="N1" s="44" t="s">
+      <c r="M1" s="49"/>
+      <c r="N1" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="51" t="s">
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="S1" s="51"/>
-      <c r="T1" s="51"/>
-      <c r="U1" s="52" t="s">
+      <c r="S1" s="49"/>
+      <c r="T1" s="49"/>
+      <c r="U1" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="V1" s="52"/>
+      <c r="V1" s="50"/>
       <c r="W1" s="4" t="s">
         <v>46</v>
       </c>
       <c r="X1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AC1" s="49" t="s">
+      <c r="AC1" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="AD1" s="49"/>
-      <c r="AE1" s="49"/>
-      <c r="AF1" s="49"/>
-      <c r="AG1" s="49"/>
-      <c r="AH1" s="49"/>
+      <c r="AD1" s="47"/>
+      <c r="AE1" s="47"/>
+      <c r="AF1" s="47"/>
+      <c r="AG1" s="47"/>
+      <c r="AH1" s="47"/>
       <c r="AI1" s="7" t="s">
         <v>37</v>
       </c>
@@ -6593,7 +6816,7 @@
     <col min="24" max="24" width="9.1640625" style="5" hidden="1" customWidth="1"/>
     <col min="25" max="26" width="13.33203125" style="4" hidden="1" customWidth="1"/>
     <col min="27" max="27" width="62.1640625" style="24" customWidth="1"/>
-    <col min="28" max="28" width="48.33203125" style="53" customWidth="1"/>
+    <col min="28" max="28" width="64.5" style="51" customWidth="1"/>
     <col min="29" max="30" width="14.6640625" customWidth="1"/>
     <col min="31" max="33" width="14.1640625" customWidth="1"/>
     <col min="34" max="34" width="4.1640625" customWidth="1"/>
@@ -6633,7 +6856,7 @@
       <c r="Y1" s="5"/>
       <c r="Z1" s="5"/>
       <c r="AA1" s="24"/>
-      <c r="AB1" s="55"/>
+      <c r="AB1" s="53"/>
     </row>
     <row r="2" spans="1:41" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B2" s="24"/>
@@ -6647,10 +6870,10 @@
       <c r="H2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="I2" s="44">
+      <c r="I2" s="43">
         <v>150</v>
       </c>
-      <c r="J2" s="44"/>
+      <c r="J2" s="43"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
@@ -6670,7 +6893,7 @@
       <c r="Y2" s="5"/>
       <c r="Z2" s="5"/>
       <c r="AA2" s="24"/>
-      <c r="AB2" s="55"/>
+      <c r="AB2" s="53"/>
     </row>
     <row r="3" spans="1:41" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B3" s="24"/>
@@ -6682,10 +6905,10 @@
       <c r="H3" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="I3" s="44">
+      <c r="I3" s="43">
         <v>30</v>
       </c>
-      <c r="J3" s="44"/>
+      <c r="J3" s="43"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
@@ -6703,7 +6926,7 @@
       <c r="Y3" s="5"/>
       <c r="Z3" s="5"/>
       <c r="AA3" s="24"/>
-      <c r="AB3" s="55"/>
+      <c r="AB3" s="53"/>
     </row>
     <row r="4" spans="1:41" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G4" s="8">
@@ -6740,12 +6963,12 @@
         <v>6</v>
       </c>
       <c r="Z4" s="20"/>
-      <c r="AB4" s="55"/>
-      <c r="AE4" s="43" t="s">
+      <c r="AB4" s="53"/>
+      <c r="AE4" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="AF4" s="43"/>
-      <c r="AG4" s="43"/>
+      <c r="AF4" s="42"/>
+      <c r="AG4" s="42"/>
       <c r="AL4" t="s">
         <v>94</v>
       </c>
@@ -6761,7 +6984,7 @@
     </row>
     <row r="5" spans="1:41" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>155</v>
@@ -6775,43 +6998,43 @@
       <c r="F5" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="G5" s="42" t="s">
+      <c r="G5" s="41" t="s">
         <v>51</v>
       </c>
-      <c r="H5" s="42"/>
+      <c r="H5" s="41"/>
       <c r="I5" s="17"/>
-      <c r="J5" s="42" t="s">
+      <c r="J5" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="K5" s="42"/>
-      <c r="M5" s="42" t="s">
+      <c r="K5" s="41"/>
+      <c r="M5" s="41" t="s">
         <v>65</v>
       </c>
-      <c r="N5" s="42"/>
-      <c r="P5" s="42" t="s">
+      <c r="N5" s="41"/>
+      <c r="P5" s="41" t="s">
         <v>78</v>
       </c>
-      <c r="Q5" s="42"/>
-      <c r="S5" s="42" t="s">
+      <c r="Q5" s="41"/>
+      <c r="S5" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="T5" s="42"/>
-      <c r="V5" s="42" t="s">
+      <c r="T5" s="41"/>
+      <c r="V5" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="W5" s="42"/>
-      <c r="Y5" s="42" t="s">
+      <c r="W5" s="41"/>
+      <c r="Y5" s="41" t="s">
         <v>135</v>
       </c>
-      <c r="Z5" s="42"/>
+      <c r="Z5" s="41"/>
       <c r="AA5" s="24" t="s">
-        <v>346</v>
-      </c>
-      <c r="AB5" s="56" t="s">
-        <v>347</v>
+        <v>328</v>
+      </c>
+      <c r="AB5" s="54" t="s">
+        <v>329</v>
       </c>
       <c r="AD5" s="36" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AE5" s="21" t="s">
         <v>33</v>
@@ -6879,7 +7102,7 @@
       <c r="Z6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="AB6" s="55"/>
+      <c r="AB6" s="53"/>
       <c r="AE6" s="19">
         <v>0</v>
       </c>
@@ -6968,10 +7191,10 @@
         <v>249360</v>
       </c>
       <c r="AA7" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="AB7" s="54" t="s">
-        <v>331</v>
+        <v>298</v>
+      </c>
+      <c r="AB7" s="52" t="s">
+        <v>314</v>
       </c>
       <c r="AE7" s="19">
         <v>0.01</v>
@@ -7063,10 +7286,10 @@
         <v>249801</v>
       </c>
       <c r="AA8" s="38" t="s">
-        <v>283</v>
-      </c>
-      <c r="AB8" s="54" t="s">
-        <v>332</v>
+        <v>281</v>
+      </c>
+      <c r="AB8" s="52" t="s">
+        <v>315</v>
       </c>
       <c r="AE8" s="19">
         <v>0.05</v>
@@ -7093,7 +7316,7 @@
     </row>
     <row r="9" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="B9" s="38" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>162</v>
@@ -7144,10 +7367,10 @@
         <v>116</v>
       </c>
       <c r="AA9" s="38" t="s">
-        <v>285</v>
-      </c>
-      <c r="AB9" s="54" t="s">
-        <v>333</v>
+        <v>283</v>
+      </c>
+      <c r="AB9" s="52" t="s">
+        <v>316</v>
       </c>
       <c r="AE9" s="19">
         <v>0.12</v>
@@ -7174,7 +7397,7 @@
     </row>
     <row r="10" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="B10" s="38" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C10" s="28" t="s">
         <v>174</v>
@@ -7211,10 +7434,10 @@
         <v>0</v>
       </c>
       <c r="AA10" s="38" t="s">
-        <v>286</v>
-      </c>
-      <c r="AB10" s="54" t="s">
-        <v>334</v>
+        <v>284</v>
+      </c>
+      <c r="AB10" s="52" t="s">
+        <v>317</v>
       </c>
       <c r="AE10" s="19">
         <v>0.2</v>
@@ -7229,7 +7452,7 @@
     </row>
     <row r="11" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="B11" s="38" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C11" s="28" t="s">
         <v>174</v>
@@ -7266,10 +7489,10 @@
         <v>0</v>
       </c>
       <c r="AA11" s="38" t="s">
-        <v>287</v>
-      </c>
-      <c r="AB11" s="54" t="s">
-        <v>335</v>
+        <v>285</v>
+      </c>
+      <c r="AB11" s="52" t="s">
+        <v>318</v>
       </c>
       <c r="AE11" s="19">
         <v>0.2</v>
@@ -7284,7 +7507,7 @@
     </row>
     <row r="12" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="B12" s="38" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C12" s="31" t="s">
         <v>162</v>
@@ -7314,10 +7537,10 @@
         <v>110</v>
       </c>
       <c r="AA12" s="38" t="s">
-        <v>284</v>
-      </c>
-      <c r="AB12" s="54" t="s">
-        <v>336</v>
+        <v>282</v>
+      </c>
+      <c r="AB12" s="52" t="s">
+        <v>319</v>
       </c>
       <c r="AE12" s="19">
         <v>0.36</v>
@@ -7397,10 +7620,10 @@
         <v>249244</v>
       </c>
       <c r="AA13" s="38" t="s">
-        <v>307</v>
-      </c>
-      <c r="AB13" s="54" t="s">
-        <v>323</v>
+        <v>300</v>
+      </c>
+      <c r="AB13" s="52" t="s">
+        <v>308</v>
       </c>
       <c r="AE13" s="19"/>
       <c r="AF13" s="19"/>
@@ -7408,7 +7631,7 @@
     </row>
     <row r="14" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="38" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C14" s="31" t="s">
         <v>162</v>
@@ -7438,10 +7661,10 @@
         <v>0.7</v>
       </c>
       <c r="AA14" s="38" t="s">
-        <v>288</v>
-      </c>
-      <c r="AB14" s="54" t="s">
-        <v>337</v>
+        <v>371</v>
+      </c>
+      <c r="AB14" s="52" t="s">
+        <v>320</v>
       </c>
       <c r="AE14" s="19">
         <v>0.6</v>
@@ -7456,16 +7679,16 @@
     </row>
     <row r="15" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="38" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C15" s="31" t="s">
         <v>162</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="G15" s="4">
         <v>5</v>
@@ -7510,10 +7733,10 @@
         <v>9</v>
       </c>
       <c r="AA15" s="38" t="s">
-        <v>300</v>
-      </c>
-      <c r="AB15" s="54" t="s">
-        <v>325</v>
+        <v>391</v>
+      </c>
+      <c r="AB15" s="52" t="s">
+        <v>390</v>
       </c>
       <c r="AE15" s="19"/>
       <c r="AF15" s="19"/>
@@ -7521,7 +7744,7 @@
     </row>
     <row r="16" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="38" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="C16" s="31"/>
       <c r="G16" s="4">
@@ -7581,10 +7804,10 @@
         <v>1.728</v>
       </c>
       <c r="AA16" s="38" t="s">
-        <v>301</v>
-      </c>
-      <c r="AB16" s="54" t="s">
-        <v>324</v>
+        <v>393</v>
+      </c>
+      <c r="AB16" s="52" t="s">
+        <v>392</v>
       </c>
       <c r="AE16" s="19"/>
       <c r="AF16" s="19"/>
@@ -7592,13 +7815,13 @@
     </row>
     <row r="17" spans="2:33" ht="51" x14ac:dyDescent="0.2">
       <c r="B17" s="38" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C17" s="31" t="s">
         <v>162</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G17" s="4">
         <v>0.33057704999999998</v>
@@ -7607,10 +7830,10 @@
         <v>0.37800893000000002</v>
       </c>
       <c r="AA17" s="38" t="s">
-        <v>289</v>
-      </c>
-      <c r="AB17" s="54" t="s">
-        <v>326</v>
+        <v>286</v>
+      </c>
+      <c r="AB17" s="52" t="s">
+        <v>309</v>
       </c>
       <c r="AE17" s="19">
         <v>1.8</v>
@@ -7625,12 +7848,12 @@
     </row>
     <row r="18" spans="2:33" ht="34" x14ac:dyDescent="0.2">
       <c r="B18" s="38" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C18" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E18" s="41" t="s">
+      <c r="E18" s="40" t="s">
         <v>118</v>
       </c>
       <c r="F18" s="10" t="s">
@@ -7643,10 +7866,10 @@
         <v>0.47800893</v>
       </c>
       <c r="AA18" s="38" t="s">
-        <v>290</v>
-      </c>
-      <c r="AB18" s="54" t="s">
-        <v>327</v>
+        <v>287</v>
+      </c>
+      <c r="AB18" s="52" t="s">
+        <v>310</v>
       </c>
       <c r="AE18" s="19">
         <v>3</v>
@@ -7661,23 +7884,23 @@
     </row>
     <row r="19" spans="2:33" ht="51" x14ac:dyDescent="0.2">
       <c r="B19" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C19" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E19" s="41"/>
+      <c r="E19" s="40"/>
       <c r="F19" s="10" t="s">
         <v>138</v>
       </c>
       <c r="G19" s="4">
         <v>0.67</v>
       </c>
-      <c r="AA19" s="40" t="s">
-        <v>291</v>
-      </c>
-      <c r="AB19" s="54" t="s">
-        <v>328</v>
+      <c r="AA19" s="39" t="s">
+        <v>288</v>
+      </c>
+      <c r="AB19" s="52" t="s">
+        <v>311</v>
       </c>
       <c r="AE19" s="19">
         <v>6</v>
@@ -7692,7 +7915,7 @@
     </row>
     <row r="20" spans="2:33" ht="17" x14ac:dyDescent="0.2">
       <c r="B20" s="38" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C20" s="31" t="s">
         <v>162</v>
@@ -7707,10 +7930,10 @@
         <v>100</v>
       </c>
       <c r="AA20" s="38" t="s">
-        <v>302</v>
-      </c>
-      <c r="AB20" s="54" t="s">
-        <v>329</v>
+        <v>296</v>
+      </c>
+      <c r="AB20" s="52" t="s">
+        <v>312</v>
       </c>
       <c r="AE20" s="19">
         <v>10</v>
@@ -7725,7 +7948,7 @@
     </row>
     <row r="21" spans="2:33" ht="17" x14ac:dyDescent="0.2">
       <c r="B21" s="38" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C21" s="31" t="s">
         <v>162</v>
@@ -7740,10 +7963,10 @@
         <v>0.25</v>
       </c>
       <c r="AA21" s="38" t="s">
-        <v>292</v>
-      </c>
-      <c r="AB21" s="54" t="s">
-        <v>330</v>
+        <v>289</v>
+      </c>
+      <c r="AB21" s="52" t="s">
+        <v>313</v>
       </c>
       <c r="AE21" s="19"/>
       <c r="AF21" s="19"/>
@@ -7751,7 +7974,7 @@
     </row>
     <row r="22" spans="2:33" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="38" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C22" s="32" t="s">
         <v>174</v>
@@ -7768,9 +7991,9 @@
         <v>37.800893000000002</v>
       </c>
       <c r="AA22" s="38" t="s">
-        <v>338</v>
-      </c>
-      <c r="AB22" s="54"/>
+        <v>321</v>
+      </c>
+      <c r="AB22" s="52"/>
       <c r="AE22" s="19">
         <v>12</v>
       </c>
@@ -7784,7 +8007,7 @@
     </row>
     <row r="23" spans="2:33" ht="17" x14ac:dyDescent="0.2">
       <c r="B23" s="38" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C23" s="32" t="s">
         <v>174</v>
@@ -7801,10 +8024,10 @@
         <v>62.199106999999998</v>
       </c>
       <c r="AA23" s="38" t="s">
-        <v>293</v>
-      </c>
-      <c r="AB23" s="54" t="s">
-        <v>339</v>
+        <v>290</v>
+      </c>
+      <c r="AB23" s="52" t="s">
+        <v>322</v>
       </c>
       <c r="AE23" s="19">
         <v>13.5</v>
@@ -7818,7 +8041,7 @@
       </c>
     </row>
     <row r="24" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="AB24" s="55"/>
+      <c r="AB24" s="53"/>
       <c r="AE24" s="19">
         <v>12</v>
       </c>
@@ -7883,10 +8106,10 @@
         <v>49500</v>
       </c>
       <c r="AA25" s="38" t="s">
-        <v>320</v>
-      </c>
-      <c r="AB25" s="54" t="s">
-        <v>340</v>
+        <v>306</v>
+      </c>
+      <c r="AB25" s="52" t="s">
+        <v>323</v>
       </c>
       <c r="AE25" s="19">
         <v>10</v>
@@ -7901,7 +8124,7 @@
     </row>
     <row r="26" spans="2:33" ht="17" x14ac:dyDescent="0.2">
       <c r="B26" s="38" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C26" s="33" t="s">
         <v>163</v>
@@ -7938,10 +8161,10 @@
         <v>0</v>
       </c>
       <c r="AA26" s="38" t="s">
-        <v>321</v>
-      </c>
-      <c r="AB26" s="54" t="s">
-        <v>341</v>
+        <v>307</v>
+      </c>
+      <c r="AB26" s="52" t="s">
+        <v>324</v>
       </c>
       <c r="AE26" s="19">
         <v>6</v>
@@ -8021,10 +8244,10 @@
         <v>49500</v>
       </c>
       <c r="AA27" s="38" t="s">
-        <v>322</v>
-      </c>
-      <c r="AB27" s="54" t="s">
-        <v>342</v>
+        <v>420</v>
+      </c>
+      <c r="AB27" s="52" t="s">
+        <v>325</v>
       </c>
       <c r="AE27" s="19">
         <v>3</v>
@@ -8055,7 +8278,7 @@
       <c r="W28" s="8"/>
       <c r="Y28" s="8"/>
       <c r="Z28" s="8"/>
-      <c r="AB28" s="55"/>
+      <c r="AB28" s="53"/>
       <c r="AE28" s="19">
         <v>1.8</v>
       </c>
@@ -8069,12 +8292,12 @@
     </row>
     <row r="29" spans="2:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="38" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C29" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="E29" s="41" t="s">
+      <c r="E29" s="40" t="s">
         <v>170</v>
       </c>
       <c r="F29" s="25" t="s">
@@ -8087,20 +8310,20 @@
         <v>0.92</v>
       </c>
       <c r="AA29" s="38" t="s">
-        <v>303</v>
-      </c>
-      <c r="AB29" s="54" t="s">
-        <v>343</v>
+        <v>389</v>
+      </c>
+      <c r="AB29" s="52" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="30" spans="2:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="38" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C30" s="32" t="s">
         <v>174</v>
       </c>
-      <c r="E30" s="41"/>
+      <c r="E30" s="40"/>
       <c r="F30" s="25" t="s">
         <v>171</v>
       </c>
@@ -8117,15 +8340,15 @@
         <v>2E-3</v>
       </c>
       <c r="AA30" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="AB30" s="54" t="s">
-        <v>344</v>
+        <v>297</v>
+      </c>
+      <c r="AB30" s="52" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="31" spans="2:33" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E31" s="26"/>
-      <c r="AB31" s="55"/>
+      <c r="AB31" s="53"/>
     </row>
     <row r="32" spans="2:33" ht="17" x14ac:dyDescent="0.2">
       <c r="F32" s="15" t="s">
@@ -8145,7 +8368,7 @@
       <c r="W32" s="8"/>
       <c r="Y32" s="8"/>
       <c r="Z32" s="8"/>
-      <c r="AB32" s="55"/>
+      <c r="AB32" s="53"/>
     </row>
     <row r="33" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B33" s="38" t="s">
@@ -8179,14 +8402,14 @@
         <v>2520000</v>
       </c>
       <c r="AA33" s="38" t="s">
-        <v>306</v>
-      </c>
-      <c r="AB33" s="54" t="s">
-        <v>345</v>
+        <v>299</v>
+      </c>
+      <c r="AB33" s="52" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="34" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="AB34" s="55"/>
+      <c r="AB34" s="53"/>
     </row>
     <row r="35" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="F35" s="11" t="s">
@@ -8206,7 +8429,7 @@
       <c r="W35" s="12"/>
       <c r="Y35" s="12"/>
       <c r="Z35" s="12"/>
-      <c r="AB35" s="55"/>
+      <c r="AB35" s="53"/>
     </row>
     <row r="36" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="F36" s="15" t="s">
@@ -8228,7 +8451,7 @@
       <c r="P36" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="AB36" s="55"/>
+      <c r="AB36" s="53"/>
       <c r="AD36" t="s">
         <v>77</v>
       </c>
@@ -8285,13 +8508,13 @@
       <c r="Z37" s="4">
         <v>0</v>
       </c>
-      <c r="AB37" s="55"/>
+      <c r="AB37" s="53"/>
     </row>
     <row r="38" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B38" s="37" t="s">
-        <v>348</v>
-      </c>
-      <c r="C38" s="45" t="s">
+        <v>330</v>
+      </c>
+      <c r="C38" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F38" s="14" t="s">
@@ -8377,17 +8600,17 @@
         <v>85</v>
       </c>
       <c r="AA38" s="38" t="s">
-        <v>317</v>
-      </c>
-      <c r="AB38" s="54" t="s">
-        <v>353</v>
+        <v>364</v>
+      </c>
+      <c r="AB38" s="52" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="39" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B39" s="38" t="s">
-        <v>349</v>
-      </c>
-      <c r="C39" s="45"/>
+        <v>331</v>
+      </c>
+      <c r="C39" s="44"/>
       <c r="F39" s="14" t="s">
         <v>69</v>
       </c>
@@ -8470,17 +8693,17 @@
         <v>80</v>
       </c>
       <c r="AA39" s="38" t="s">
-        <v>318</v>
-      </c>
-      <c r="AB39" s="54" t="s">
-        <v>351</v>
+        <v>365</v>
+      </c>
+      <c r="AB39" s="52" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="40" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B40" s="38" t="s">
-        <v>350</v>
-      </c>
-      <c r="C40" s="45"/>
+        <v>332</v>
+      </c>
+      <c r="C40" s="44"/>
       <c r="F40" s="14" t="s">
         <v>79</v>
       </c>
@@ -8562,15 +8785,15 @@
         <v>92</v>
       </c>
       <c r="AA40" s="38" t="s">
-        <v>319</v>
-      </c>
-      <c r="AB40" s="54" t="s">
-        <v>352</v>
+        <v>366</v>
+      </c>
+      <c r="AB40" s="52" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="41" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B41" s="38"/>
-      <c r="C41" s="45"/>
+      <c r="C41" s="44"/>
       <c r="F41" s="14" t="s">
         <v>80</v>
       </c>
@@ -8651,23 +8874,23 @@
         <v>43</v>
       </c>
       <c r="AA41" s="38"/>
-      <c r="AB41" s="54"/>
+      <c r="AB41" s="52"/>
     </row>
     <row r="42" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="F42" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="AB42" s="55"/>
+      <c r="AB42" s="53"/>
     </row>
     <row r="43" spans="2:30" ht="17" x14ac:dyDescent="0.2">
-      <c r="B43" s="47" t="s">
-        <v>190</v>
-      </c>
-      <c r="C43" s="45" t="s">
+      <c r="B43" s="46" t="s">
+        <v>189</v>
+      </c>
+      <c r="C43" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H43" s="4">
         <v>0</v>
@@ -8697,17 +8920,17 @@
         <v>0</v>
       </c>
       <c r="AA43" s="38" t="s">
-        <v>308</v>
-      </c>
-      <c r="AB43" s="54" t="s">
-        <v>355</v>
+        <v>301</v>
+      </c>
+      <c r="AB43" s="52" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="44" spans="2:30" ht="17" x14ac:dyDescent="0.2">
-      <c r="B44" s="47"/>
-      <c r="C44" s="45"/>
+      <c r="B44" s="46"/>
+      <c r="C44" s="44"/>
       <c r="F44" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H44" s="4">
         <v>0</v>
@@ -8737,13 +8960,13 @@
         <v>0</v>
       </c>
       <c r="AA44" s="38"/>
-      <c r="AB44" s="54"/>
+      <c r="AB44" s="52"/>
     </row>
     <row r="45" spans="2:30" ht="17" x14ac:dyDescent="0.2">
-      <c r="B45" s="47"/>
-      <c r="C45" s="45"/>
+      <c r="B45" s="46"/>
+      <c r="C45" s="44"/>
       <c r="F45" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H45" s="4">
         <v>0</v>
@@ -8773,13 +8996,13 @@
         <v>0</v>
       </c>
       <c r="AA45" s="38"/>
-      <c r="AB45" s="54"/>
+      <c r="AB45" s="52"/>
     </row>
     <row r="46" spans="2:30" ht="17" x14ac:dyDescent="0.2">
-      <c r="B46" s="47"/>
-      <c r="C46" s="45"/>
+      <c r="B46" s="46"/>
+      <c r="C46" s="44"/>
       <c r="F46" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H46" s="4">
         <v>0</v>
@@ -8809,11 +9032,11 @@
         <v>0</v>
       </c>
       <c r="AA46" s="38"/>
-      <c r="AB46" s="54"/>
+      <c r="AB46" s="52"/>
     </row>
     <row r="47" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B47" s="38" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C47" s="28" t="s">
         <v>174</v>
@@ -8848,30 +9071,30 @@
         <v>0</v>
       </c>
       <c r="AA47" s="38" t="s">
-        <v>309</v>
-      </c>
-      <c r="AB47" s="54" t="s">
-        <v>354</v>
+        <v>302</v>
+      </c>
+      <c r="AB47" s="52" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="48" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="F48" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="AB48" s="55"/>
+      <c r="AB48" s="53"/>
     </row>
     <row r="49" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B49" s="47" t="s">
-        <v>262</v>
-      </c>
-      <c r="C49" s="45" t="s">
+      <c r="B49" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="C49" s="44" t="s">
         <v>174</v>
       </c>
-      <c r="E49" s="41" t="s">
-        <v>250</v>
+      <c r="E49" s="40" t="s">
+        <v>248</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H49" s="4">
         <f>MIN(H43,H$15*G38)</f>
@@ -8902,18 +9125,18 @@
         <v>0</v>
       </c>
       <c r="AA49" s="38" t="s">
-        <v>310</v>
-      </c>
-      <c r="AB49" s="54" t="s">
-        <v>356</v>
+        <v>398</v>
+      </c>
+      <c r="AB49" s="52" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="50" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B50" s="47"/>
-      <c r="C50" s="45"/>
-      <c r="E50" s="41"/>
+      <c r="B50" s="46"/>
+      <c r="C50" s="44"/>
+      <c r="E50" s="40"/>
       <c r="F50" s="14" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H50" s="4">
         <f>MIN(H44,H$15*G39)</f>
@@ -8944,14 +9167,14 @@
         <v>0</v>
       </c>
       <c r="AA50" s="38"/>
-      <c r="AB50" s="54"/>
+      <c r="AB50" s="52"/>
     </row>
     <row r="51" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B51" s="47"/>
-      <c r="C51" s="45"/>
-      <c r="E51" s="41"/>
+      <c r="B51" s="46"/>
+      <c r="C51" s="44"/>
+      <c r="E51" s="40"/>
       <c r="F51" s="14" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H51" s="4">
         <f>MIN(H45,H$15*G40)</f>
@@ -8982,14 +9205,14 @@
         <v>0</v>
       </c>
       <c r="AA51" s="38"/>
-      <c r="AB51" s="54"/>
+      <c r="AB51" s="52"/>
     </row>
     <row r="52" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B52" s="47"/>
-      <c r="C52" s="45"/>
-      <c r="E52" s="41"/>
+      <c r="B52" s="46"/>
+      <c r="C52" s="44"/>
+      <c r="E52" s="40"/>
       <c r="F52" s="14" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H52" s="4">
         <f>MIN(H46,H$15*G41)</f>
@@ -9020,11 +9243,11 @@
         <v>0</v>
       </c>
       <c r="AA52" s="38"/>
-      <c r="AB52" s="54"/>
+      <c r="AB52" s="52"/>
     </row>
     <row r="53" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B53" s="38" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C53" s="28" t="s">
         <v>174</v>
@@ -9059,15 +9282,15 @@
         <v>0</v>
       </c>
       <c r="AA53" s="38" t="s">
-        <v>311</v>
-      </c>
-      <c r="AB53" s="54" t="s">
-        <v>357</v>
+        <v>397</v>
+      </c>
+      <c r="AB53" s="52" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="54" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B54" s="38" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C54" s="28"/>
       <c r="F54" s="14"/>
@@ -9100,23 +9323,25 @@
         <v>0</v>
       </c>
       <c r="AA54" s="38" t="s">
-        <v>312</v>
-      </c>
-      <c r="AB54" s="54"/>
+        <v>396</v>
+      </c>
+      <c r="AB54" s="52" t="s">
+        <v>339</v>
+      </c>
     </row>
     <row r="55" spans="2:28" x14ac:dyDescent="0.2">
       <c r="F55" s="14"/>
-      <c r="AB55" s="54"/>
+      <c r="AB55" s="52"/>
     </row>
     <row r="56" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B56" s="47" t="s">
-        <v>192</v>
-      </c>
-      <c r="C56" s="45" t="s">
+      <c r="B56" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="C56" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F56" s="14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H56" s="4">
         <f>H43*$H$21</f>
@@ -9147,15 +9372,17 @@
         <v>0</v>
       </c>
       <c r="AA56" s="38" t="s">
-        <v>313</v>
-      </c>
-      <c r="AB56" s="54"/>
+        <v>303</v>
+      </c>
+      <c r="AB56" s="52" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="57" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B57" s="47"/>
-      <c r="C57" s="45"/>
+      <c r="B57" s="46"/>
+      <c r="C57" s="44"/>
       <c r="F57" s="14" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H57" s="4">
         <f>H44*$H$21</f>
@@ -9186,13 +9413,13 @@
         <v>0</v>
       </c>
       <c r="AA57" s="38"/>
-      <c r="AB57" s="54"/>
+      <c r="AB57" s="52"/>
     </row>
     <row r="58" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B58" s="47"/>
-      <c r="C58" s="45"/>
+      <c r="B58" s="46"/>
+      <c r="C58" s="44"/>
       <c r="F58" s="14" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H58" s="4">
         <f>H45*$H$21</f>
@@ -9223,13 +9450,13 @@
         <v>0</v>
       </c>
       <c r="AA58" s="38"/>
-      <c r="AB58" s="54"/>
+      <c r="AB58" s="52"/>
     </row>
     <row r="59" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B59" s="47"/>
-      <c r="C59" s="45"/>
+      <c r="B59" s="46"/>
+      <c r="C59" s="44"/>
       <c r="F59" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H59" s="4">
         <f>H46*$H$21</f>
@@ -9260,11 +9487,11 @@
         <v>0</v>
       </c>
       <c r="AA59" s="38"/>
-      <c r="AB59" s="54"/>
+      <c r="AB59" s="52"/>
     </row>
     <row r="60" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B60" s="38" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C60" s="28" t="s">
         <v>174</v>
@@ -9299,19 +9526,21 @@
         <v>0</v>
       </c>
       <c r="AA60" s="38" t="s">
-        <v>314</v>
-      </c>
-      <c r="AB60" s="54"/>
+        <v>304</v>
+      </c>
+      <c r="AB60" s="52" t="s">
+        <v>341</v>
+      </c>
     </row>
     <row r="61" spans="2:28" x14ac:dyDescent="0.2">
       <c r="F61" s="14"/>
-      <c r="AB61" s="54"/>
+      <c r="AB61" s="52"/>
     </row>
     <row r="62" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B62" s="47" t="s">
+      <c r="B62" s="46" t="s">
         <v>178</v>
       </c>
-      <c r="C62" s="45" t="s">
+      <c r="C62" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F62" s="14" t="s">
@@ -9346,13 +9575,15 @@
         <v>0.6</v>
       </c>
       <c r="AA62" s="38" t="s">
-        <v>315</v>
-      </c>
-      <c r="AB62" s="54"/>
+        <v>358</v>
+      </c>
+      <c r="AB62" s="52" t="s">
+        <v>368</v>
+      </c>
     </row>
     <row r="63" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B63" s="47"/>
-      <c r="C63" s="45"/>
+      <c r="B63" s="46"/>
+      <c r="C63" s="44"/>
       <c r="F63" s="14" t="s">
         <v>91</v>
       </c>
@@ -9383,11 +9614,11 @@
         <v>0.36</v>
       </c>
       <c r="AA63" s="38"/>
-      <c r="AB63" s="54"/>
+      <c r="AB63" s="52"/>
     </row>
     <row r="64" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B64" s="47"/>
-      <c r="C64" s="45"/>
+      <c r="B64" s="46"/>
+      <c r="C64" s="44"/>
       <c r="F64" s="14" t="s">
         <v>92</v>
       </c>
@@ -9417,11 +9648,11 @@
         <v>0.2</v>
       </c>
       <c r="AA64" s="38"/>
-      <c r="AB64" s="54"/>
+      <c r="AB64" s="52"/>
     </row>
     <row r="65" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B65" s="47"/>
-      <c r="C65" s="45"/>
+      <c r="B65" s="46"/>
+      <c r="C65" s="44"/>
       <c r="F65" s="14" t="s">
         <v>93</v>
       </c>
@@ -9450,23 +9681,23 @@
         <v>0.12</v>
       </c>
       <c r="AA65" s="38"/>
-      <c r="AB65" s="54"/>
+      <c r="AB65" s="52"/>
     </row>
     <row r="66" spans="2:32" ht="17" x14ac:dyDescent="0.2">
       <c r="F66" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="AB66" s="54"/>
+      <c r="AB66" s="52"/>
     </row>
     <row r="67" spans="2:32" x14ac:dyDescent="0.2">
       <c r="F67" s="14"/>
-      <c r="AB67" s="54"/>
+      <c r="AB67" s="52"/>
     </row>
     <row r="68" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B68" s="47" t="s">
-        <v>237</v>
-      </c>
-      <c r="C68" s="45" t="s">
+      <c r="B68" s="46" t="s">
+        <v>235</v>
+      </c>
+      <c r="C68" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F68" s="14" t="s">
@@ -9501,13 +9732,15 @@
         <v>113.71737449773644</v>
       </c>
       <c r="AA68" s="38" t="s">
-        <v>316</v>
-      </c>
-      <c r="AB68" s="54"/>
+        <v>305</v>
+      </c>
+      <c r="AB68" s="52" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="69" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B69" s="47"/>
-      <c r="C69" s="45"/>
+      <c r="B69" s="46"/>
+      <c r="C69" s="44"/>
       <c r="F69" s="14" t="s">
         <v>110</v>
       </c>
@@ -9536,12 +9769,12 @@
         <v>59.120937045501634</v>
       </c>
       <c r="AA69" s="38"/>
-      <c r="AB69" s="54"/>
+      <c r="AB69" s="52"/>
     </row>
     <row r="70" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B70" s="47"/>
-      <c r="C70" s="45"/>
-      <c r="E70" s="41"/>
+      <c r="B70" s="46"/>
+      <c r="C70" s="44"/>
+      <c r="E70" s="40"/>
       <c r="F70" s="14" t="s">
         <v>111</v>
       </c>
@@ -9566,12 +9799,12 @@
         <v>34.923908138103698</v>
       </c>
       <c r="AA70" s="38"/>
-      <c r="AB70" s="54"/>
+      <c r="AB70" s="52"/>
     </row>
     <row r="71" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B71" s="47"/>
-      <c r="C71" s="45"/>
-      <c r="E71" s="41"/>
+      <c r="B71" s="46"/>
+      <c r="C71" s="44"/>
+      <c r="E71" s="40"/>
       <c r="F71" s="14" t="s">
         <v>112</v>
       </c>
@@ -9596,18 +9829,18 @@
         <v>7.7352753599069999</v>
       </c>
       <c r="AA71" s="38"/>
-      <c r="AB71" s="54"/>
+      <c r="AB71" s="52"/>
     </row>
     <row r="72" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="E72" s="41"/>
+      <c r="E72" s="40"/>
       <c r="F72" s="14"/>
-      <c r="AB72" s="54"/>
+      <c r="AB72" s="52"/>
     </row>
     <row r="73" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B73" s="47" t="s">
-        <v>234</v>
-      </c>
-      <c r="C73" s="45" t="s">
+      <c r="B73" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="C73" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F73" s="14" t="s">
@@ -9640,12 +9873,16 @@
         <f>INT(Y$4-$AG$6 &gt; $E81)*MAX(W96-$H$22*W38-Z43,0)</f>
         <v>0</v>
       </c>
-      <c r="AA73" s="38"/>
-      <c r="AB73" s="54"/>
+      <c r="AA73" s="38" t="s">
+        <v>342</v>
+      </c>
+      <c r="AB73" s="52" t="s">
+        <v>345</v>
+      </c>
     </row>
     <row r="74" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B74" s="47"/>
-      <c r="C74" s="45"/>
+      <c r="B74" s="46"/>
+      <c r="C74" s="44"/>
       <c r="F74" s="14" t="s">
         <v>128</v>
       </c>
@@ -9677,12 +9914,12 @@
         <v>0</v>
       </c>
       <c r="AA74" s="38"/>
-      <c r="AB74" s="54"/>
+      <c r="AB74" s="52"/>
     </row>
     <row r="75" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B75" s="47"/>
-      <c r="C75" s="45"/>
-      <c r="E75" s="41" t="s">
+      <c r="B75" s="46"/>
+      <c r="C75" s="44"/>
+      <c r="E75" s="40" t="s">
         <v>152</v>
       </c>
       <c r="F75" s="14" t="s">
@@ -9716,12 +9953,12 @@
         <v>0</v>
       </c>
       <c r="AA75" s="38"/>
-      <c r="AB75" s="54"/>
+      <c r="AB75" s="52"/>
     </row>
     <row r="76" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B76" s="47"/>
-      <c r="C76" s="45"/>
-      <c r="E76" s="41"/>
+      <c r="B76" s="46"/>
+      <c r="C76" s="44"/>
+      <c r="E76" s="40"/>
       <c r="F76" s="14" t="s">
         <v>130</v>
       </c>
@@ -9753,16 +9990,16 @@
         <v>0</v>
       </c>
       <c r="AA76" s="38"/>
-      <c r="AB76" s="54"/>
+      <c r="AB76" s="52"/>
     </row>
     <row r="77" spans="2:32" ht="17" x14ac:dyDescent="0.2">
       <c r="B77" s="38" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C77" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="E77" s="41"/>
+      <c r="E77" s="40"/>
       <c r="F77" s="14" t="s">
         <v>147</v>
       </c>
@@ -9793,16 +10030,20 @@
         <f>SUM(Z73:Z76)</f>
         <v>0</v>
       </c>
-      <c r="AA77" s="38"/>
-      <c r="AB77" s="54"/>
+      <c r="AA77" s="56" t="s">
+        <v>343</v>
+      </c>
+      <c r="AB77" s="52" t="s">
+        <v>344</v>
+      </c>
       <c r="AF77" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="78" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="E78" s="41"/>
+      <c r="E78" s="40"/>
       <c r="F78" s="14"/>
-      <c r="AB78" s="54"/>
+      <c r="AB78" s="52"/>
       <c r="AD78" t="s">
         <v>85</v>
       </c>
@@ -9811,10 +10052,10 @@
       </c>
     </row>
     <row r="79" spans="2:32" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B79" s="48" t="s">
-        <v>236</v>
-      </c>
-      <c r="C79" s="45" t="s">
+      <c r="B79" s="37" t="s">
+        <v>347</v>
+      </c>
+      <c r="C79" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F79" s="14" t="s">
@@ -9841,15 +10082,21 @@
       <c r="Y79" s="4">
         <v>0</v>
       </c>
-      <c r="AA79" s="39"/>
-      <c r="AB79" s="54"/>
+      <c r="AA79" s="38" t="s">
+        <v>349</v>
+      </c>
+      <c r="AB79" s="52" t="s">
+        <v>350</v>
+      </c>
       <c r="AD79" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="80" spans="2:32" ht="17" x14ac:dyDescent="0.2">
-      <c r="B80" s="48"/>
-      <c r="C80" s="45"/>
+      <c r="B80" s="37" t="s">
+        <v>346</v>
+      </c>
+      <c r="C80" s="44"/>
       <c r="F80" s="14" t="s">
         <v>148</v>
       </c>
@@ -9909,12 +10156,16 @@
         <f>IF(Y80&gt;=Y$132, IF(Y79&lt;Y$132, Y$132-Y79, 0),Z73)</f>
         <v>0</v>
       </c>
-      <c r="AA80" s="39"/>
-      <c r="AB80" s="54"/>
+      <c r="AA80" s="38" t="s">
+        <v>351</v>
+      </c>
+      <c r="AB80" s="52" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="81" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B81" s="48"/>
-      <c r="C81" s="45"/>
+      <c r="B81" s="55"/>
+      <c r="C81" s="44"/>
       <c r="E81" s="22">
         <v>0</v>
       </c>
@@ -9977,12 +10228,12 @@
         <f>IF(Y81&gt;=Y$132, IF(Y80&lt;Y$132, Y$132-Y80, 0),Z74)</f>
         <v>0</v>
       </c>
-      <c r="AA81" s="39"/>
-      <c r="AB81" s="54"/>
+      <c r="AA81" s="37"/>
+      <c r="AB81" s="52"/>
     </row>
     <row r="82" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B82" s="48"/>
-      <c r="C82" s="45"/>
+      <c r="B82" s="55"/>
+      <c r="C82" s="44"/>
       <c r="E82" s="22">
         <v>1</v>
       </c>
@@ -10045,12 +10296,12 @@
         <f>IF(Y82&gt;=Y$132, IF(Y81&lt;Y$132, Y$132-Y81, 0),Z75)</f>
         <v>0</v>
       </c>
-      <c r="AA82" s="39"/>
-      <c r="AB82" s="54"/>
+      <c r="AA82" s="37"/>
+      <c r="AB82" s="52"/>
     </row>
     <row r="83" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B83" s="48"/>
-      <c r="C83" s="45"/>
+      <c r="B83" s="55"/>
+      <c r="C83" s="44"/>
       <c r="E83" s="22">
         <v>2</v>
       </c>
@@ -10113,15 +10364,15 @@
         <f>IF(Y83&gt;=Y$132, IF(Y82&lt;Y$132, Y$132-Y82, 0),Z76)</f>
         <v>0</v>
       </c>
-      <c r="AA83" s="39"/>
-      <c r="AB83" s="54"/>
+      <c r="AA83" s="37"/>
+      <c r="AB83" s="52"/>
     </row>
     <row r="84" spans="2:28" x14ac:dyDescent="0.2">
       <c r="E84" s="22">
         <v>3</v>
       </c>
       <c r="F84" s="14"/>
-      <c r="AB84" s="54"/>
+      <c r="AB84" s="52"/>
     </row>
     <row r="85" spans="2:28" x14ac:dyDescent="0.2">
       <c r="F85" s="14"/>
@@ -10143,13 +10394,13 @@
       <c r="Y85" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="AB85" s="54"/>
+      <c r="AB85" s="52"/>
     </row>
     <row r="86" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B86" s="46" t="s">
-        <v>180</v>
-      </c>
-      <c r="C86" s="45" t="s">
+      <c r="B86" s="37" t="s">
+        <v>352</v>
+      </c>
+      <c r="C86" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F86" s="14" t="s">
@@ -10207,12 +10458,18 @@
         <f>Z62*Y86</f>
         <v>0.6</v>
       </c>
-      <c r="AA86" s="37"/>
-      <c r="AB86" s="54"/>
+      <c r="AA86" s="37" t="s">
+        <v>359</v>
+      </c>
+      <c r="AB86" s="52" t="s">
+        <v>369</v>
+      </c>
     </row>
     <row r="87" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B87" s="46"/>
-      <c r="C87" s="45"/>
+      <c r="B87" s="37" t="s">
+        <v>353</v>
+      </c>
+      <c r="C87" s="44"/>
       <c r="F87" s="14" t="s">
         <v>132</v>
       </c>
@@ -10268,12 +10525,16 @@
         <f>Z63</f>
         <v>0.36</v>
       </c>
-      <c r="AA87" s="37"/>
-      <c r="AB87" s="54"/>
+      <c r="AA87" s="37" t="s">
+        <v>354</v>
+      </c>
+      <c r="AB87" s="52" t="s">
+        <v>355</v>
+      </c>
     </row>
     <row r="88" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B88" s="46"/>
-      <c r="C88" s="45"/>
+      <c r="B88" s="37"/>
+      <c r="C88" s="44"/>
       <c r="F88" s="14" t="s">
         <v>133</v>
       </c>
@@ -10330,11 +10591,11 @@
         <v>0.2</v>
       </c>
       <c r="AA88" s="37"/>
-      <c r="AB88" s="54"/>
+      <c r="AB88" s="52"/>
     </row>
     <row r="89" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B89" s="46"/>
-      <c r="C89" s="45"/>
+      <c r="B89" s="55"/>
+      <c r="C89" s="44"/>
       <c r="F89" s="14" t="s">
         <v>134</v>
       </c>
@@ -10391,21 +10652,21 @@
         <v>0.12</v>
       </c>
       <c r="AA89" s="37"/>
-      <c r="AB89" s="54"/>
+      <c r="AB89" s="52"/>
     </row>
     <row r="90" spans="2:28" x14ac:dyDescent="0.2">
       <c r="F90" s="14"/>
-      <c r="AB90" s="54"/>
+      <c r="AB90" s="52"/>
     </row>
     <row r="91" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B91" s="46" t="s">
+      <c r="B91" s="45" t="s">
+        <v>202</v>
+      </c>
+      <c r="C91" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="F91" s="14" t="s">
         <v>203</v>
-      </c>
-      <c r="C91" s="45" t="s">
-        <v>174</v>
-      </c>
-      <c r="F91" s="14" t="s">
-        <v>204</v>
       </c>
       <c r="H91" s="4">
         <f>H57*H33</f>
@@ -10435,14 +10696,18 @@
         <f>(W96-Z80-Z43)*$G$30</f>
         <v>9.8621113109027395E-2</v>
       </c>
-      <c r="AA91" s="37"/>
-      <c r="AB91" s="54"/>
+      <c r="AA91" s="37" t="s">
+        <v>362</v>
+      </c>
+      <c r="AB91" s="52" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="92" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B92" s="46"/>
-      <c r="C92" s="45"/>
+      <c r="B92" s="45"/>
+      <c r="C92" s="44"/>
       <c r="F92" s="14" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H92" s="4">
         <f>H58*H34</f>
@@ -10473,13 +10738,13 @@
         <v>4.7678726762454618E-2</v>
       </c>
       <c r="AA92" s="37"/>
-      <c r="AB92" s="54"/>
+      <c r="AB92" s="52"/>
     </row>
     <row r="93" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B93" s="46"/>
-      <c r="C93" s="45"/>
+      <c r="B93" s="45"/>
+      <c r="C93" s="44"/>
       <c r="F93" s="14" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H93" s="4">
         <f>H59*H35</f>
@@ -10510,13 +10775,13 @@
         <v>2.5983329604301563E-2</v>
       </c>
       <c r="AA93" s="37"/>
-      <c r="AB93" s="54"/>
+      <c r="AB93" s="52"/>
     </row>
     <row r="94" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B94" s="46"/>
-      <c r="C94" s="45"/>
+      <c r="B94" s="45"/>
+      <c r="C94" s="44"/>
       <c r="F94" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H94" s="4">
         <f>H60*H36</f>
@@ -10547,17 +10812,17 @@
         <v>4.049540093E-3</v>
       </c>
       <c r="AA94" s="37"/>
-      <c r="AB94" s="54"/>
+      <c r="AB94" s="52"/>
     </row>
     <row r="95" spans="2:28" x14ac:dyDescent="0.2">
       <c r="F95" s="14"/>
-      <c r="AB95" s="54"/>
+      <c r="AB95" s="52"/>
     </row>
     <row r="96" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B96" s="46" t="s">
-        <v>208</v>
-      </c>
-      <c r="C96" s="45" t="s">
+      <c r="B96" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="C96" s="44" t="s">
         <v>174</v>
       </c>
       <c r="F96" s="14" t="s">
@@ -10591,12 +10856,16 @@
         <f>W96 - Z80 - Z91 - Z43 + Z38*Z86</f>
         <v>113.71737449773644</v>
       </c>
-      <c r="AA96" s="37"/>
-      <c r="AB96" s="54"/>
+      <c r="AA96" s="38" t="s">
+        <v>356</v>
+      </c>
+      <c r="AB96" s="52" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="97" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B97" s="46"/>
-      <c r="C97" s="45"/>
+      <c r="B97" s="45"/>
+      <c r="C97" s="44"/>
       <c r="F97" s="14" t="s">
         <v>71</v>
       </c>
@@ -10629,11 +10898,11 @@
         <v>59.120937045501627</v>
       </c>
       <c r="AA97" s="37"/>
-      <c r="AB97" s="54"/>
+      <c r="AB97" s="52"/>
     </row>
     <row r="98" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B98" s="46"/>
-      <c r="C98" s="45"/>
+      <c r="B98" s="45"/>
+      <c r="C98" s="44"/>
       <c r="F98" s="14" t="s">
         <v>72</v>
       </c>
@@ -10666,11 +10935,11 @@
         <v>34.923908138103698</v>
       </c>
       <c r="AA98" s="37"/>
-      <c r="AB98" s="54"/>
+      <c r="AB98" s="52"/>
     </row>
     <row r="99" spans="2:28" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="46"/>
-      <c r="C99" s="45"/>
+      <c r="B99" s="45"/>
+      <c r="C99" s="44"/>
       <c r="F99" s="14" t="s">
         <v>81</v>
       </c>
@@ -10703,23 +10972,23 @@
         <v>7.7352753599069999</v>
       </c>
       <c r="AA99" s="37"/>
-      <c r="AB99" s="54"/>
+      <c r="AB99" s="52"/>
     </row>
     <row r="100" spans="2:28" x14ac:dyDescent="0.2">
       <c r="E100" s="26"/>
       <c r="F100" s="14"/>
-      <c r="AB100" s="54"/>
+      <c r="AB100" s="52"/>
     </row>
     <row r="101" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B101" s="46" t="s">
-        <v>209</v>
-      </c>
-      <c r="C101" s="45" t="s">
+      <c r="B101" s="45" t="s">
+        <v>208</v>
+      </c>
+      <c r="C101" s="44" t="s">
         <v>174</v>
       </c>
       <c r="E101" s="26"/>
       <c r="F101" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H101" s="4">
         <f>H96*$H$21</f>
@@ -10749,15 +11018,19 @@
         <f>Z96*$H$21</f>
         <v>28.429343624434111</v>
       </c>
-      <c r="AA101" s="37"/>
-      <c r="AB101" s="54"/>
+      <c r="AA101" s="38" t="s">
+        <v>360</v>
+      </c>
+      <c r="AB101" s="52" t="s">
+        <v>361</v>
+      </c>
     </row>
     <row r="102" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B102" s="46"/>
-      <c r="C102" s="45"/>
+      <c r="B102" s="45"/>
+      <c r="C102" s="44"/>
       <c r="E102" s="26"/>
       <c r="F102" s="14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H102" s="4">
         <f t="shared" ref="H102:H104" si="9">H97*$H$21</f>
@@ -10788,14 +11061,14 @@
         <v>14.780234261375407</v>
       </c>
       <c r="AA102" s="37"/>
-      <c r="AB102" s="54"/>
+      <c r="AB102" s="52"/>
     </row>
     <row r="103" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B103" s="46"/>
-      <c r="C103" s="45"/>
+      <c r="B103" s="45"/>
+      <c r="C103" s="44"/>
       <c r="E103" s="26"/>
       <c r="F103" s="14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H103" s="4">
         <f>H98*$H$21</f>
@@ -10826,14 +11099,14 @@
         <v>8.7309770345259246</v>
       </c>
       <c r="AA103" s="37"/>
-      <c r="AB103" s="54"/>
+      <c r="AB103" s="52"/>
     </row>
     <row r="104" spans="2:28" ht="17" x14ac:dyDescent="0.2">
-      <c r="B104" s="46"/>
-      <c r="C104" s="45"/>
+      <c r="B104" s="45"/>
+      <c r="C104" s="44"/>
       <c r="E104" s="26"/>
       <c r="F104" s="14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H104" s="4">
         <f t="shared" si="9"/>
@@ -10864,7 +11137,7 @@
         <v>1.93381883997675</v>
       </c>
       <c r="AA104" s="37"/>
-      <c r="AB104" s="54"/>
+      <c r="AB104" s="52"/>
     </row>
     <row r="105" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B105" s="29"/>
@@ -10872,7 +11145,7 @@
       <c r="E105" s="26"/>
       <c r="F105" s="14"/>
       <c r="AA105" s="29"/>
-      <c r="AB105" s="54"/>
+      <c r="AB105" s="52"/>
     </row>
     <row r="106" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B106" s="29"/>
@@ -10880,7 +11153,7 @@
       <c r="E106" s="26"/>
       <c r="F106" s="14"/>
       <c r="AA106" s="29"/>
-      <c r="AB106" s="54"/>
+      <c r="AB106" s="52"/>
     </row>
     <row r="107" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="E107" s="26"/>
@@ -10891,14 +11164,14 @@
         <v>124</v>
       </c>
       <c r="H107" s="8"/>
-      <c r="AB107" s="54"/>
+      <c r="AB107" s="52"/>
     </row>
     <row r="108" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B108" s="38" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C108" s="34" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E108" s="26"/>
       <c r="F108" s="14" t="s">
@@ -10961,11 +11234,11 @@
         <v>0.92</v>
       </c>
       <c r="AA108" s="38"/>
-      <c r="AB108" s="54"/>
+      <c r="AB108" s="52"/>
     </row>
     <row r="109" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B109" s="38" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C109" s="28" t="s">
         <v>174</v>
@@ -11029,12 +11302,16 @@
         <f>Z7*$H$20</f>
         <v>24936000</v>
       </c>
-      <c r="AA109" s="38"/>
-      <c r="AB109" s="54"/>
+      <c r="AA109" s="38" t="s">
+        <v>372</v>
+      </c>
+      <c r="AB109" s="52" t="s">
+        <v>377</v>
+      </c>
     </row>
     <row r="110" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B110" s="38" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C110" s="28" t="s">
         <v>174</v>
@@ -11097,13 +11374,15 @@
         <v>0.86560925711218095</v>
       </c>
       <c r="AA110" s="38" t="s">
-        <v>294</v>
-      </c>
-      <c r="AB110" s="54"/>
+        <v>429</v>
+      </c>
+      <c r="AB110" s="52" t="s">
+        <v>373</v>
+      </c>
     </row>
     <row r="111" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B111" s="38" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C111" s="33" t="s">
         <v>163</v>
@@ -11167,12 +11446,16 @@
         <f>Z108*Z110</f>
         <v>0.7963605165432065</v>
       </c>
-      <c r="AA111" s="38"/>
-      <c r="AB111" s="54"/>
+      <c r="AA111" s="38" t="s">
+        <v>374</v>
+      </c>
+      <c r="AB111" s="52" t="s">
+        <v>375</v>
+      </c>
     </row>
     <row r="112" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B112" s="38" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C112" s="33" t="s">
         <v>163</v>
@@ -11236,12 +11519,16 @@
         <f>W112 - W133 - W121 - W144 + Z111*Z7</f>
         <v>15603395.572368858</v>
       </c>
-      <c r="AA112" s="38"/>
-      <c r="AB112" s="54"/>
+      <c r="AA112" s="38" t="s">
+        <v>376</v>
+      </c>
+      <c r="AB112" s="52" t="s">
+        <v>378</v>
+      </c>
     </row>
     <row r="113" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B113" s="38" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C113" s="33" t="s">
         <v>163</v>
@@ -11305,12 +11592,16 @@
         <f>Z112/Z7</f>
         <v>62.573771143603061</v>
       </c>
-      <c r="AA113" s="38"/>
-      <c r="AB113" s="54"/>
+      <c r="AA113" s="38" t="s">
+        <v>379</v>
+      </c>
+      <c r="AB113" s="52" t="s">
+        <v>380</v>
+      </c>
     </row>
     <row r="114" spans="2:28" ht="34" x14ac:dyDescent="0.2">
       <c r="B114" s="38" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C114" s="28" t="s">
         <v>174</v>
@@ -11374,12 +11665,16 @@
         <f>MAX(Z113-$H22,0)</f>
         <v>24.772878143603059</v>
       </c>
-      <c r="AA114" s="38"/>
-      <c r="AB114" s="54"/>
+      <c r="AA114" s="38" t="s">
+        <v>419</v>
+      </c>
+      <c r="AB114" s="57" t="s">
+        <v>381</v>
+      </c>
     </row>
     <row r="115" spans="2:28" x14ac:dyDescent="0.2">
       <c r="F115" s="13"/>
-      <c r="AB115" s="54"/>
+      <c r="AB115" s="52"/>
     </row>
     <row r="116" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="F116" s="11" t="s">
@@ -11399,17 +11694,17 @@
       <c r="W116" s="12"/>
       <c r="Y116" s="12"/>
       <c r="Z116" s="12"/>
-      <c r="AB116" s="54"/>
+      <c r="AB116" s="52"/>
     </row>
     <row r="117" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B117" s="38" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C117" s="34" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F117" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G117" s="4">
         <f>G113*G7</f>
@@ -11468,17 +11763,17 @@
         <v>15603395.572368858</v>
       </c>
       <c r="AA117" s="38"/>
-      <c r="AB117" s="54"/>
+      <c r="AB117" s="52"/>
     </row>
     <row r="118" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B118" s="38" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C118" s="33" t="s">
         <v>163</v>
       </c>
       <c r="F118" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H118" s="4">
         <f>SUM(H96:H99)</f>
@@ -11508,18 +11803,22 @@
         <f>SUM(Z96:Z99)</f>
         <v>215.49749504124878</v>
       </c>
-      <c r="AA118" s="38"/>
-      <c r="AB118" s="54"/>
+      <c r="AA118" s="38" t="s">
+        <v>382</v>
+      </c>
+      <c r="AB118" s="52" t="s">
+        <v>385</v>
+      </c>
     </row>
     <row r="119" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B119" s="38" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C119" s="33" t="s">
         <v>163</v>
       </c>
       <c r="F119" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G119" s="4">
         <f>G117+G118</f>
@@ -11577,18 +11876,22 @@
         <f>Z117+Z118</f>
         <v>15603611.069863901</v>
       </c>
-      <c r="AA119" s="38"/>
-      <c r="AB119" s="54"/>
+      <c r="AA119" s="38" t="s">
+        <v>383</v>
+      </c>
+      <c r="AB119" s="52" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="120" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B120" s="38" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C120" s="33" t="s">
         <v>163</v>
       </c>
       <c r="F120" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G120" s="4">
         <f>G119*$G$21</f>
@@ -11646,18 +11949,22 @@
         <f>Z119*$H$21</f>
         <v>3900902.7674659751</v>
       </c>
-      <c r="AA120" s="38"/>
-      <c r="AB120" s="54"/>
+      <c r="AA120" s="38" t="s">
+        <v>384</v>
+      </c>
+      <c r="AB120" s="52" t="s">
+        <v>387</v>
+      </c>
     </row>
     <row r="121" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B121" s="38" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C121" s="28" t="s">
         <v>174</v>
       </c>
       <c r="F121" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="G121" s="4">
         <f>G9*G113</f>
@@ -11715,18 +12022,22 @@
         <f>Z9*Z113</f>
         <v>7258.5574526579549</v>
       </c>
-      <c r="AA121" s="38"/>
-      <c r="AB121" s="54"/>
+      <c r="AA121" s="38" t="s">
+        <v>395</v>
+      </c>
+      <c r="AB121" s="52" t="s">
+        <v>388</v>
+      </c>
     </row>
     <row r="122" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B122" s="38" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C122" s="28" t="s">
         <v>174</v>
       </c>
       <c r="F122" s="10" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="G122" s="4">
         <f>MIN(G121,G9*G15)</f>
@@ -11784,18 +12095,22 @@
         <f>MIN(Z121,Z9*Z15)</f>
         <v>1044</v>
       </c>
-      <c r="AA122" s="38"/>
-      <c r="AB122" s="54"/>
+      <c r="AA122" s="38" t="s">
+        <v>399</v>
+      </c>
+      <c r="AB122" s="52" t="s">
+        <v>388</v>
+      </c>
     </row>
     <row r="123" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B123" s="38" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C123" s="28" t="s">
         <v>174</v>
       </c>
       <c r="F123" s="10" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G123" s="4">
         <f>(G121-G122)*$G$14</f>
@@ -11853,18 +12168,22 @@
         <f>(Z121-Z122+Z54)*$G$14</f>
         <v>4350.1902168605684</v>
       </c>
-      <c r="AA123" s="38"/>
-      <c r="AB123" s="54"/>
+      <c r="AA123" s="38" t="s">
+        <v>400</v>
+      </c>
+      <c r="AB123" s="52" t="s">
+        <v>388</v>
+      </c>
     </row>
     <row r="124" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B124" s="38" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C124" s="33" t="s">
         <v>163</v>
       </c>
       <c r="F124" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="G124" s="4">
         <f>MIN(G123+H123, G33)</f>
@@ -11894,18 +12213,22 @@
         <f>MIN(Y123+Z123, Y33)</f>
         <v>10471.887293585241</v>
       </c>
-      <c r="AA124" s="38"/>
-      <c r="AB124" s="54"/>
+      <c r="AA124" s="38" t="s">
+        <v>401</v>
+      </c>
+      <c r="AB124" s="52" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="125" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="B125" s="38" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C125" s="28" t="s">
         <v>174</v>
       </c>
       <c r="F125" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="G125" s="4">
         <f>G123/(G123+H123)</f>
@@ -11963,12 +12286,16 @@
         <f>Z123/(Y123+Z123)</f>
         <v>0.41541606540450088</v>
       </c>
-      <c r="AA125" s="38"/>
-      <c r="AB125" s="54"/>
+      <c r="AA125" s="38" t="s">
+        <v>404</v>
+      </c>
+      <c r="AB125" s="52" t="s">
+        <v>403</v>
+      </c>
     </row>
     <row r="126" spans="2:28" ht="34" x14ac:dyDescent="0.2">
       <c r="B126" s="38" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C126" s="28" t="s">
         <v>174</v>
@@ -12032,11 +12359,15 @@
         <f>MAX(Z13-Z27, 0)*Z114</f>
         <v>4948233.7719158493</v>
       </c>
-      <c r="AA126" s="38"/>
-      <c r="AB126" s="54"/>
+      <c r="AA126" s="38" t="s">
+        <v>405</v>
+      </c>
+      <c r="AB126" s="52" t="s">
+        <v>406</v>
+      </c>
     </row>
     <row r="127" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="AB127" s="54"/>
+      <c r="AB127" s="52"/>
     </row>
     <row r="128" spans="2:28" ht="17" x14ac:dyDescent="0.2">
       <c r="F128" s="15" t="s">
@@ -12056,17 +12387,17 @@
       <c r="W128" s="8"/>
       <c r="Y128" s="8"/>
       <c r="Z128" s="8"/>
-      <c r="AB128" s="54"/>
+      <c r="AB128" s="52"/>
     </row>
     <row r="129" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B129" s="38" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C129" s="28" t="s">
         <v>174</v>
       </c>
       <c r="F129" s="14" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G129" s="4">
         <f>MAX(G33-G124,0)</f>
@@ -12096,12 +12427,16 @@
         <f>MAX(Y33-Y124,0)</f>
         <v>2509528.1127064149</v>
       </c>
-      <c r="AA129" s="38"/>
-      <c r="AB129" s="54"/>
+      <c r="AA129" s="38" t="s">
+        <v>408</v>
+      </c>
+      <c r="AB129" s="52" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="130" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B130" s="38" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C130" s="28" t="s">
         <v>174</v>
@@ -12137,12 +12472,16 @@
         <f>MIN(Y140,Y129)</f>
         <v>236958.69160889552</v>
       </c>
-      <c r="AA130" s="38"/>
-      <c r="AB130" s="54"/>
+      <c r="AA130" s="38" t="s">
+        <v>411</v>
+      </c>
+      <c r="AB130" s="52" t="s">
+        <v>417</v>
+      </c>
     </row>
     <row r="131" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B131" s="38" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C131" s="28" t="s">
         <v>174</v>
@@ -12178,12 +12517,16 @@
         <f>Y129-Y130</f>
         <v>2272569.4210975193</v>
       </c>
-      <c r="AA131" s="38"/>
-      <c r="AB131" s="54"/>
+      <c r="AA131" s="38" t="s">
+        <v>409</v>
+      </c>
+      <c r="AB131" s="52" t="s">
+        <v>410</v>
+      </c>
     </row>
     <row r="132" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B132" s="38" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C132" s="28" t="s">
         <v>174</v>
@@ -12219,12 +12562,16 @@
         <f>MIN(Y131,Z77)</f>
         <v>0</v>
       </c>
-      <c r="AA132" s="38"/>
-      <c r="AB132" s="54"/>
+      <c r="AA132" s="38" t="s">
+        <v>412</v>
+      </c>
+      <c r="AB132" s="52" t="s">
+        <v>416</v>
+      </c>
     </row>
     <row r="133" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B133" s="38" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C133" s="28" t="s">
         <v>174</v>
@@ -12288,12 +12635,16 @@
         <f>Z141*Y130</f>
         <v>209877.50332872596</v>
       </c>
-      <c r="AA133" s="38"/>
-      <c r="AB133" s="54"/>
+      <c r="AA133" s="38" t="s">
+        <v>413</v>
+      </c>
+      <c r="AB133" s="52" t="s">
+        <v>415</v>
+      </c>
     </row>
     <row r="134" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B134" s="38" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C134" s="33" t="s">
         <v>163</v>
@@ -12357,8 +12708,12 @@
         <f>Z133+Y132</f>
         <v>209877.50332872596</v>
       </c>
-      <c r="AA134" s="38"/>
-      <c r="AB134" s="54"/>
+      <c r="AA134" s="38" t="s">
+        <v>414</v>
+      </c>
+      <c r="AB134" s="52" t="s">
+        <v>418</v>
+      </c>
     </row>
     <row r="135" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="F135" s="15" t="s">
@@ -12378,11 +12733,11 @@
       <c r="W135" s="8"/>
       <c r="Y135" s="8"/>
       <c r="Z135" s="8"/>
-      <c r="AB135" s="54"/>
+      <c r="AB135" s="52"/>
     </row>
     <row r="136" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="B136" s="38" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C136" s="28" t="s">
         <v>174</v>
@@ -12446,13 +12801,15 @@
         <f>Z114/$H$23</f>
         <v>0.39828350178087057</v>
       </c>
-      <c r="AA136" s="38"/>
-      <c r="AB136" s="54">
-        <v>0.5</v>
+      <c r="AA136" s="38" t="s">
+        <v>431</v>
+      </c>
+      <c r="AB136" s="52" t="s">
+        <v>421</v>
       </c>
       <c r="AC136">
         <f>SUM(AB$6:AB136)</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AD136">
         <v>20</v>
@@ -12460,16 +12817,16 @@
     </row>
     <row r="137" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B137" s="38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C137" s="28" t="s">
         <v>174</v>
       </c>
       <c r="F137" s="10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G137" s="4">
         <f>MAX(MIN((G136-$G$17)/$G$18, 1), 0)</f>
@@ -12527,13 +12884,15 @@
         <f>MAX(MIN((Z136-$H$17)/$H$18, 1), 0)</f>
         <v>4.2414629745244618E-2</v>
       </c>
-      <c r="AA137" s="38"/>
-      <c r="AB137" s="54">
-        <v>0.3</v>
+      <c r="AA137" s="39" t="s">
+        <v>430</v>
+      </c>
+      <c r="AB137" s="52" t="s">
+        <v>422</v>
       </c>
       <c r="AC137">
         <f>SUM(AB$6:AB137)</f>
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="AD137">
         <v>20</v>
@@ -12542,12 +12901,10 @@
     <row r="138" spans="1:30" x14ac:dyDescent="0.2">
       <c r="B138" s="38"/>
       <c r="AA138" s="38"/>
-      <c r="AB138" s="54">
-        <v>0.2</v>
-      </c>
+      <c r="AB138" s="52"/>
       <c r="AC138">
         <f>SUM(AB$6:AB138)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD138">
         <v>20</v>
@@ -12555,7 +12912,7 @@
     </row>
     <row r="139" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B139" s="38" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C139" s="28" t="s">
         <v>174</v>
@@ -12619,13 +12976,15 @@
         <f>Z126*Z137</f>
         <v>209877.50332872596</v>
       </c>
-      <c r="AA139" s="38"/>
-      <c r="AB139" s="54">
-        <v>0.125</v>
+      <c r="AA139" s="38" t="s">
+        <v>423</v>
+      </c>
+      <c r="AB139" s="52" t="s">
+        <v>425</v>
       </c>
       <c r="AC139">
         <f>SUM(AB$6:AB159)</f>
-        <v>1.125</v>
+        <v>0</v>
       </c>
       <c r="AD139">
         <v>20</v>
@@ -12633,7 +12992,7 @@
     </row>
     <row r="140" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B140" s="38" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C140" s="28" t="s">
         <v>174</v>
@@ -12697,12 +13056,16 @@
         <f>Y140</f>
         <v>236958.69160889552</v>
       </c>
-      <c r="AA140" s="38"/>
-      <c r="AB140" s="54"/>
+      <c r="AA140" s="38" t="s">
+        <v>424</v>
+      </c>
+      <c r="AB140" s="52" t="s">
+        <v>426</v>
+      </c>
     </row>
     <row r="141" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B141" s="38" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C141" s="28" t="s">
         <v>174</v>
@@ -12766,15 +13129,19 @@
         <f>Z139/Z140</f>
         <v>0.88571346298253728</v>
       </c>
-      <c r="AA141" s="38"/>
-      <c r="AB141" s="54"/>
+      <c r="AA141" s="38" t="s">
+        <v>428</v>
+      </c>
+      <c r="AB141" s="52" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="142" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="AB142" s="54"/>
+      <c r="AB142" s="52"/>
     </row>
     <row r="143" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="F143" s="15" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G143" s="8"/>
       <c r="H143" s="8"/>
@@ -12790,17 +13157,17 @@
       <c r="W143" s="8"/>
       <c r="Y143" s="8"/>
       <c r="Z143" s="8"/>
-      <c r="AB143" s="54"/>
+      <c r="AB143" s="52"/>
     </row>
     <row r="144" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B144" s="38" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C144" s="33" t="s">
         <v>163</v>
       </c>
       <c r="F144" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G144" s="4">
         <f>(G112 - G133 - G121)*$G$30</f>
@@ -12859,11 +13226,11 @@
         <v>24156.603765901902</v>
       </c>
       <c r="AA144" s="38"/>
-      <c r="AB144" s="54"/>
+      <c r="AB144" s="52"/>
     </row>
     <row r="145" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B145" s="38" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C145" s="33" t="s">
         <v>163</v>
@@ -12925,17 +13292,17 @@
         <v>6039.1509414754755</v>
       </c>
       <c r="AA145" s="38"/>
-      <c r="AB145" s="54"/>
+      <c r="AB145" s="52"/>
     </row>
     <row r="146" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B146" s="38" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C146" s="33" t="s">
         <v>163</v>
       </c>
       <c r="F146" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G146" s="4">
         <f>G133*$G21</f>
@@ -12994,7 +13361,7 @@
         <v>52469.375832181489</v>
       </c>
       <c r="AA146" s="38"/>
-      <c r="AB146" s="54"/>
+      <c r="AB146" s="52"/>
     </row>
     <row r="147" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B147" s="38" t="s">
@@ -13063,7 +13430,7 @@
         <v>1864.3672357973865</v>
       </c>
       <c r="AA147" s="38"/>
-      <c r="AB147" s="54"/>
+      <c r="AB147" s="52"/>
     </row>
     <row r="148" spans="2:30" ht="17" x14ac:dyDescent="0.2">
       <c r="B148" s="38" t="s">
@@ -13132,11 +13499,11 @@
         <v>1353.1913631644886</v>
       </c>
       <c r="AA148" s="38"/>
-      <c r="AB148" s="54"/>
+      <c r="AB148" s="52"/>
     </row>
     <row r="149" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B149" s="38" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="C149" s="33" t="s">
         <v>163</v>
@@ -13198,17 +13565,17 @@
         <v>129.19999999999999</v>
       </c>
       <c r="AA149" s="38"/>
-      <c r="AB149" s="54"/>
+      <c r="AB149" s="52"/>
     </row>
     <row r="150" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="AB150" s="54"/>
+      <c r="AB150" s="52"/>
     </row>
     <row r="151" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="AB151" s="54"/>
+      <c r="AB151" s="52"/>
     </row>
     <row r="152" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B152" s="24" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="G152" s="4">
         <f>G147+G122</f>
@@ -13266,14 +13633,14 @@
         <f>Z147+Z122</f>
         <v>2908.3672357973865</v>
       </c>
-      <c r="AB152" s="54"/>
+      <c r="AB152" s="52"/>
     </row>
     <row r="153" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="AB153" s="54"/>
+      <c r="AB153" s="52"/>
     </row>
     <row r="154" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B154" s="38" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C154" s="33" t="s">
         <v>163</v>
@@ -13307,7 +13674,7 @@
         <v>247430.57890248077</v>
       </c>
       <c r="AA154" s="38"/>
-      <c r="AB154" s="54"/>
+      <c r="AB154" s="52"/>
     </row>
     <row r="155" spans="2:30" x14ac:dyDescent="0.2">
       <c r="G155" s="4">
@@ -13340,49 +13707,48 @@
       </c>
     </row>
     <row r="160" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="AB160" s="53">
+      <c r="AB160" s="51">
         <v>0.1225</v>
       </c>
       <c r="AC160">
         <f>SUM(AB$6:AB160)</f>
-        <v>1.2475000000000001</v>
+        <v>0.1225</v>
       </c>
       <c r="AD160">
         <v>20</v>
       </c>
     </row>
     <row r="161" spans="28:30" x14ac:dyDescent="0.2">
-      <c r="AB161" s="53">
+      <c r="AB161" s="51">
         <v>0.12239999999999999</v>
       </c>
       <c r="AC161">
         <f>SUM(AB$6:AB161)</f>
-        <v>1.3699000000000001</v>
+        <v>0.24490000000000001</v>
       </c>
       <c r="AD161">
         <v>20</v>
       </c>
     </row>
     <row r="162" spans="28:30" x14ac:dyDescent="0.2">
-      <c r="AB162" s="53">
+      <c r="AB162" s="51">
         <v>0.12230000000000001</v>
       </c>
       <c r="AC162">
         <f>SUM(AB$6:AB162)</f>
-        <v>1.4922000000000002</v>
+        <v>0.36720000000000003</v>
       </c>
       <c r="AD162">
         <v>20</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="36">
     <mergeCell ref="B101:B104"/>
     <mergeCell ref="C101:C104"/>
     <mergeCell ref="B49:B52"/>
     <mergeCell ref="C49:C52"/>
     <mergeCell ref="E49:E52"/>
-    <mergeCell ref="B79:B83"/>
     <mergeCell ref="C79:C83"/>
     <mergeCell ref="C86:C89"/>
     <mergeCell ref="B96:B99"/>
@@ -13391,7 +13757,6 @@
     <mergeCell ref="C91:C94"/>
     <mergeCell ref="B73:B76"/>
     <mergeCell ref="C73:C76"/>
-    <mergeCell ref="B86:B89"/>
     <mergeCell ref="C38:C41"/>
     <mergeCell ref="C62:C65"/>
     <mergeCell ref="B68:B71"/>

</xml_diff>

<commit_message>
some minor updates to variable indexing in the carbon ledger workbook
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07306AE-55B5-2F40-9E05-17D9F0059831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DF1C0F-5C91-4848-9A35-540414953B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8240" yWindow="760" windowWidth="34560" windowHeight="20060" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="-3860" yWindow="760" windowWidth="34560" windowHeight="20040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="480">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -997,9 +997,6 @@
     <t>\overline{Y}_{alloc}(t, u)</t>
   </si>
   <si>
-    <t>\overline{Y}_{alloc\_aux}(t, u)</t>
-  </si>
-  <si>
     <t>\Psi^{(y)}(t, u)</t>
   </si>
   <si>
@@ -1279,9 +1276,6 @@
     <t>Matrix ($n_T \times 2$) storing removals from original forests by type (columns), excluding conversions.</t>
   </si>
   <si>
-    <t>Matrix ($n_T \times 2$) storing removals from all forests byt ype (columns), excluding conversions. Removals from young secondary forests are added to those removals from original secondary forests.</t>
-  </si>
-  <si>
     <t>Matrix ($n_T \times 2$) giving fraction of original forest stock available when compared to healthy (unperturbed) baseline.</t>
   </si>
   <si>
@@ -1481,6 +1475,12 @@
   </si>
   <si>
     <t>d_{rmv}(t)</t>
+  </si>
+  <si>
+    <t>\overline{Y}_{aux}(t, u)</t>
+  </si>
+  <si>
+    <t>Matrix ($n_T \times 2$) storing removals from all forests by type (columns), excluding conversions. Removals from young secondary forests are added to those removals from original secondary forests.</t>
   </si>
 </sst>
 </file>
@@ -6961,16 +6961,16 @@
     <col min="10" max="11" width="13.33203125" style="4" customWidth="1"/>
     <col min="12" max="12" width="11.83203125" style="5" customWidth="1"/>
     <col min="13" max="14" width="13.33203125" style="4" customWidth="1"/>
-    <col min="15" max="15" width="21.1640625" style="5" customWidth="1"/>
-    <col min="16" max="16" width="21.1640625" style="4" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" style="5" customWidth="1"/>
-    <col min="19" max="20" width="13.33203125" style="4" customWidth="1"/>
-    <col min="21" max="21" width="9.1640625" style="5" customWidth="1"/>
-    <col min="22" max="22" width="13.33203125" style="4" customWidth="1"/>
-    <col min="23" max="23" width="12.5" style="4" customWidth="1"/>
-    <col min="24" max="24" width="9.1640625" style="5" customWidth="1"/>
-    <col min="25" max="26" width="13.33203125" style="4" customWidth="1"/>
+    <col min="15" max="15" width="21.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="21.1640625" style="4" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" style="5" hidden="1" customWidth="1"/>
+    <col min="19" max="20" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="9.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="12.5" style="4" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="9.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="25" max="26" width="13.33203125" style="4" hidden="1" customWidth="1"/>
     <col min="27" max="27" width="62.1640625" style="24" customWidth="1"/>
     <col min="28" max="28" width="64.5" style="58" customWidth="1"/>
     <col min="29" max="29" width="14.6640625" style="59" customWidth="1"/>
@@ -7145,7 +7145,7 @@
     </row>
     <row r="5" spans="1:41" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>155</v>
@@ -7195,7 +7195,7 @@
         <v>313</v>
       </c>
       <c r="AC5" s="27" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AD5" s="36" t="s">
         <v>230</v>
@@ -7293,7 +7293,7 @@
     </row>
     <row r="7" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B7" s="38" t="s">
         <v>156</v>
@@ -7362,10 +7362,10 @@
         <v>290</v>
       </c>
       <c r="AB7" s="53" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AC7" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AE7" s="19">
         <v>0.01</v>
@@ -7392,7 +7392,7 @@
     </row>
     <row r="8" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B8" s="38" t="s">
         <v>157</v>
@@ -7463,10 +7463,10 @@
         <v>279</v>
       </c>
       <c r="AB8" s="53" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AC8" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AE8" s="19">
         <v>0.05</v>
@@ -7493,7 +7493,7 @@
     </row>
     <row r="9" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B9" s="38" t="s">
         <v>222</v>
@@ -7550,10 +7550,10 @@
         <v>281</v>
       </c>
       <c r="AB9" s="53" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AC9" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AE9" s="19">
         <v>0.12</v>
@@ -7580,7 +7580,7 @@
     </row>
     <row r="10" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B10" s="38" t="s">
         <v>221</v>
@@ -7626,7 +7626,7 @@
         <v>302</v>
       </c>
       <c r="AC10" s="54" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AE10" s="19">
         <v>0.2</v>
@@ -7641,7 +7641,7 @@
     </row>
     <row r="11" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B11" s="38" t="s">
         <v>219</v>
@@ -7687,7 +7687,7 @@
         <v>303</v>
       </c>
       <c r="AC11" s="54" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AE11" s="19">
         <v>0.2</v>
@@ -7702,7 +7702,7 @@
     </row>
     <row r="12" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B12" s="38" t="s">
         <v>220</v>
@@ -7741,7 +7741,7 @@
         <v>304</v>
       </c>
       <c r="AC12" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AE12" s="19">
         <v>0.36</v>
@@ -7756,7 +7756,7 @@
     </row>
     <row r="13" spans="1:41" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B13" s="38" t="s">
         <v>158</v>
@@ -7830,7 +7830,7 @@
         <v>298</v>
       </c>
       <c r="AC13" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AE13" s="19"/>
       <c r="AF13" s="19"/>
@@ -7838,7 +7838,7 @@
     </row>
     <row r="14" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B14" s="38" t="s">
         <v>223</v>
@@ -7871,13 +7871,13 @@
         <v>0.7</v>
       </c>
       <c r="AA14" s="38" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="AB14" s="53" t="s">
         <v>305</v>
       </c>
       <c r="AC14" s="54" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AE14" s="19">
         <v>0.6</v>
@@ -7892,7 +7892,7 @@
     </row>
     <row r="15" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B15" s="38" t="s">
         <v>244</v>
@@ -7949,13 +7949,13 @@
         <v>9</v>
       </c>
       <c r="AA15" s="38" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AB15" s="53" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="AC15" s="54" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="AE15" s="19"/>
       <c r="AF15" s="19"/>
@@ -7963,7 +7963,7 @@
     </row>
     <row r="16" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B16" s="38" t="s">
         <v>286</v>
@@ -8028,13 +8028,13 @@
         <v>1.728</v>
       </c>
       <c r="AA16" s="38" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AB16" s="53" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="AC16" s="54" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="AE16" s="19"/>
       <c r="AF16" s="19"/>
@@ -8042,10 +8042,10 @@
     </row>
     <row r="17" spans="1:33" ht="51" x14ac:dyDescent="0.2">
       <c r="A17" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C17" s="31" t="s">
         <v>162</v>
@@ -8060,13 +8060,13 @@
         <v>0.37800893000000002</v>
       </c>
       <c r="AA17" s="38" t="s">
+        <v>451</v>
+      </c>
+      <c r="AB17" s="53" t="s">
         <v>453</v>
       </c>
-      <c r="AB17" s="53" t="s">
-        <v>455</v>
-      </c>
       <c r="AC17" s="54" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="AE17" s="19">
         <v>1.8</v>
@@ -8081,10 +8081,10 @@
     </row>
     <row r="18" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C18" s="31" t="s">
         <v>162</v>
@@ -8102,13 +8102,13 @@
         <v>0.47800893</v>
       </c>
       <c r="AA18" s="38" t="s">
+        <v>452</v>
+      </c>
+      <c r="AB18" s="53" t="s">
         <v>454</v>
       </c>
-      <c r="AB18" s="53" t="s">
-        <v>456</v>
-      </c>
       <c r="AC18" s="54" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="AE18" s="19">
         <v>3</v>
@@ -8123,7 +8123,7 @@
     </row>
     <row r="19" spans="1:33" ht="51" x14ac:dyDescent="0.2">
       <c r="A19" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B19" s="38" t="s">
         <v>224</v>
@@ -8145,7 +8145,7 @@
         <v>299</v>
       </c>
       <c r="AC19" s="54" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="AE19" s="19">
         <v>6</v>
@@ -8160,7 +8160,7 @@
     </row>
     <row r="20" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B20" s="38" t="s">
         <v>226</v>
@@ -8178,13 +8178,13 @@
         <v>100</v>
       </c>
       <c r="AA20" s="38" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="AB20" s="53" t="s">
         <v>300</v>
       </c>
       <c r="AC20" s="54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AE20" s="19">
         <v>10</v>
@@ -8199,7 +8199,7 @@
     </row>
     <row r="21" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B21" s="38" t="s">
         <v>228</v>
@@ -8223,7 +8223,7 @@
         <v>301</v>
       </c>
       <c r="AC21" s="55" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="AE21" s="19"/>
       <c r="AF21" s="19"/>
@@ -8231,7 +8231,7 @@
     </row>
     <row r="22" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B22" s="38" t="s">
         <v>275</v>
@@ -8251,13 +8251,13 @@
         <v>37.800893000000002</v>
       </c>
       <c r="AA22" s="38" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="AB22" s="53" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="AC22" s="54" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="AE22" s="19">
         <v>12</v>
@@ -8272,7 +8272,7 @@
     </row>
     <row r="23" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B23" s="38" t="s">
         <v>227</v>
@@ -8292,13 +8292,13 @@
         <v>62.199106999999998</v>
       </c>
       <c r="AA23" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AB23" s="53" t="s">
         <v>306</v>
       </c>
       <c r="AC23" s="54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AE23" s="19">
         <v>13.5</v>
@@ -8327,7 +8327,7 @@
     </row>
     <row r="25" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B25" s="38" t="s">
         <v>159</v>
@@ -8381,13 +8381,13 @@
         <v>49500</v>
       </c>
       <c r="AA25" s="38" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="AB25" s="53" t="s">
         <v>307</v>
       </c>
       <c r="AC25" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AE25" s="19">
         <v>10</v>
@@ -8402,7 +8402,7 @@
     </row>
     <row r="26" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B26" s="38" t="s">
         <v>274</v>
@@ -8442,13 +8442,13 @@
         <v>0</v>
       </c>
       <c r="AA26" s="38" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="AB26" s="53" t="s">
         <v>308</v>
       </c>
       <c r="AC26" s="54" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AE26" s="19">
         <v>6</v>
@@ -8463,7 +8463,7 @@
     </row>
     <row r="27" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B27" s="38" t="s">
         <v>160</v>
@@ -8531,13 +8531,13 @@
         <v>49500</v>
       </c>
       <c r="AA27" s="38" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="AB27" s="53" t="s">
         <v>309</v>
       </c>
       <c r="AC27" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AE27" s="19">
         <v>3</v>
@@ -8583,7 +8583,7 @@
     </row>
     <row r="29" spans="1:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B29" s="38" t="s">
         <v>273</v>
@@ -8604,18 +8604,18 @@
         <v>0.92</v>
       </c>
       <c r="AA29" s="38" t="s">
+        <v>337</v>
+      </c>
+      <c r="AB29" s="53" t="s">
         <v>338</v>
       </c>
-      <c r="AB29" s="53" t="s">
-        <v>339</v>
-      </c>
       <c r="AC29" s="54" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="30" spans="1:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B30" s="38" t="s">
         <v>229</v>
@@ -8640,13 +8640,13 @@
         <v>2E-3</v>
       </c>
       <c r="AA30" s="38" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="AB30" s="53" t="s">
         <v>310</v>
       </c>
       <c r="AC30" s="54" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="31" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -8677,7 +8677,7 @@
     </row>
     <row r="33" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B33" s="38" t="s">
         <v>168</v>
@@ -8716,7 +8716,7 @@
         <v>311</v>
       </c>
       <c r="AC33" s="54" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="34" spans="1:30" x14ac:dyDescent="0.2">
@@ -8827,7 +8827,7 @@
     </row>
     <row r="38" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B38" s="37" t="s">
         <v>314</v>
@@ -8918,18 +8918,18 @@
         <v>85</v>
       </c>
       <c r="AA38" s="38" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="AB38" s="53" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="AC38" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="39" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B39" s="38" t="s">
         <v>315</v>
@@ -9017,18 +9017,18 @@
         <v>80</v>
       </c>
       <c r="AA39" s="38" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="AB39" s="53" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AC39" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="40" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B40" s="38" t="s">
         <v>316</v>
@@ -9115,13 +9115,13 @@
         <v>92</v>
       </c>
       <c r="AA40" s="38" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="AB40" s="53" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AC40" s="54" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="41" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -9219,7 +9219,7 @@
     </row>
     <row r="43" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B43" s="46" t="s">
         <v>189</v>
@@ -9261,10 +9261,10 @@
         <v>293</v>
       </c>
       <c r="AB43" s="53" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="AC43" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="44" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -9379,6 +9379,9 @@
       <c r="AC46" s="54"/>
     </row>
     <row r="47" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A47" s="19" t="s">
+        <v>456</v>
+      </c>
       <c r="B47" s="38" t="s">
         <v>190</v>
       </c>
@@ -9418,10 +9421,10 @@
         <v>294</v>
       </c>
       <c r="AB47" s="53" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="AC47" s="54" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -9473,13 +9476,13 @@
         <v>0</v>
       </c>
       <c r="AA49" s="38" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="AB49" s="53" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="AC49" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="50" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -9636,13 +9639,13 @@
         <v>0</v>
       </c>
       <c r="AA53" s="38" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AB53" s="53" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="AC53" s="54" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="54" spans="1:29" x14ac:dyDescent="0.2">
@@ -9680,13 +9683,13 @@
         <v>0</v>
       </c>
       <c r="AA54" s="38" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="AB54" s="53" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="AC54" s="54" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="55" spans="1:29" x14ac:dyDescent="0.2">
@@ -9736,10 +9739,10 @@
         <v>295</v>
       </c>
       <c r="AB56" s="53" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="AC56" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="57" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -9896,10 +9899,10 @@
         <v>296</v>
       </c>
       <c r="AB60" s="53" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="AC60" s="54" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="61" spans="1:29" x14ac:dyDescent="0.2">
@@ -9909,7 +9912,7 @@
     </row>
     <row r="62" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B62" s="46" t="s">
         <v>178</v>
@@ -9949,13 +9952,13 @@
         <v>0.6</v>
       </c>
       <c r="AA62" s="38" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AB62" s="53" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AC62" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="63" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -10065,10 +10068,10 @@
     </row>
     <row r="66" spans="1:32" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B66" s="38" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="C66" s="31" t="s">
         <v>162</v>
@@ -10077,13 +10080,13 @@
         <v>49</v>
       </c>
       <c r="AA66" s="38" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="AB66" s="53" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="AC66" s="54" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="67" spans="1:32" x14ac:dyDescent="0.2">
@@ -10133,10 +10136,10 @@
         <v>297</v>
       </c>
       <c r="AB68" s="53" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="AC68" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="69" spans="1:32" ht="17" x14ac:dyDescent="0.2">
@@ -10243,7 +10246,7 @@
     </row>
     <row r="73" spans="1:32" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B73" s="46" t="s">
         <v>231</v>
@@ -10282,13 +10285,13 @@
         <v>0</v>
       </c>
       <c r="AA73" s="38" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="AB73" s="53" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="AC73" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="74" spans="1:32" ht="17" x14ac:dyDescent="0.2">
@@ -10408,7 +10411,7 @@
     </row>
     <row r="77" spans="1:32" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B77" s="38" t="s">
         <v>232</v>
@@ -10448,13 +10451,13 @@
         <v>0</v>
       </c>
       <c r="AA77" s="56" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="AB77" s="53" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="AC77" s="54" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="AF77" t="s">
         <v>106</v>
@@ -10474,10 +10477,10 @@
     </row>
     <row r="79" spans="1:32" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B79" s="37" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="C79" s="44" t="s">
         <v>174</v>
@@ -10510,10 +10513,10 @@
         <v>317</v>
       </c>
       <c r="AB79" s="53" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="AC79" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="AD79" t="s">
         <v>86</v>
@@ -10521,10 +10524,10 @@
     </row>
     <row r="80" spans="1:32" ht="17" x14ac:dyDescent="0.2">
       <c r="A80" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B80" s="37" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C80" s="44"/>
       <c r="F80" s="14" t="s">
@@ -10587,13 +10590,13 @@
         <v>0</v>
       </c>
       <c r="AA80" s="38" t="s">
-        <v>318</v>
+        <v>478</v>
       </c>
       <c r="AB80" s="53" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="AC80" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="81" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -10836,10 +10839,10 @@
     </row>
     <row r="86" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A86" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B86" s="37" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C86" s="44" t="s">
         <v>174</v>
@@ -10900,21 +10903,21 @@
         <v>0.6</v>
       </c>
       <c r="AA86" s="37" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AB86" s="53" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="AC86" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="87" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B87" s="37" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="C87" s="44"/>
       <c r="F87" s="14" t="s">
@@ -10973,13 +10976,13 @@
         <v>0.36</v>
       </c>
       <c r="AA87" s="37" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="AB87" s="53" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="AC87" s="54" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="88" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -11150,13 +11153,13 @@
         <v>9.8621113109027395E-2</v>
       </c>
       <c r="AA91" s="37" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="AB91" s="53" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="AC91" s="54" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="92" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -11280,7 +11283,7 @@
     </row>
     <row r="96" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A96" s="19" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B96" s="45" t="s">
         <v>207</v>
@@ -11320,13 +11323,13 @@
         <v>113.71737449773644</v>
       </c>
       <c r="AA96" s="38" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AB96" s="53" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="AC96" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="97" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -11489,13 +11492,13 @@
         <v>28.429343624434111</v>
       </c>
       <c r="AA101" s="38" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="AB101" s="53" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="AC101" s="54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="102" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -11783,13 +11786,13 @@
         <v>24936000</v>
       </c>
       <c r="AA109" s="38" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="AB109" s="53" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="AC109" s="54" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="110" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -11857,13 +11860,13 @@
         <v>0.87277215440147748</v>
       </c>
       <c r="AA110" s="38" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="AB110" s="53" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="AC110" s="54" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="111" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -11933,13 +11936,13 @@
         <v>0.80295038204935931</v>
       </c>
       <c r="AA111" s="38" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AB111" s="53" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="AC111" s="54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="112" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12009,13 +12012,13 @@
         <v>15618862.859584641</v>
       </c>
       <c r="AA112" s="38" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AB112" s="53" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="AC112" s="54" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="113" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12085,13 +12088,13 @@
         <v>62.635799083993589</v>
       </c>
       <c r="AA113" s="38" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="AB113" s="53" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="AC113" s="54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="114" spans="2:29" ht="34" x14ac:dyDescent="0.2">
@@ -12161,13 +12164,13 @@
         <v>24.834906083993587</v>
       </c>
       <c r="AA114" s="38" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="AB114" s="57" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="AC114" s="54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="115" spans="2:29" x14ac:dyDescent="0.2">
@@ -12305,13 +12308,13 @@
         <v>215.49749504124878</v>
       </c>
       <c r="AA118" s="38" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="AB118" s="53" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="AC118" s="54" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="119" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12381,13 +12384,13 @@
         <v>15619078.357079683</v>
       </c>
       <c r="AA119" s="38" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="AB119" s="53" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="AC119" s="54" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="120" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12457,13 +12460,13 @@
         <v>3904769.5892699207</v>
       </c>
       <c r="AA120" s="38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="AB120" s="53" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="AC120" s="54" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="121" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12533,13 +12536,13 @@
         <v>7265.7526937432567</v>
       </c>
       <c r="AA121" s="38" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="AB121" s="53" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AC121" s="54" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="122" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12609,13 +12612,13 @@
         <v>1044</v>
       </c>
       <c r="AA122" s="38" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AB122" s="53" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AC122" s="54" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="123" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12685,13 +12688,13 @@
         <v>4355.2268856202791</v>
       </c>
       <c r="AA123" s="38" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="AB123" s="53" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AC123" s="54" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="124" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12733,13 +12736,13 @@
         <v>4355.2268856202791</v>
       </c>
       <c r="AA124" s="38" t="s">
+        <v>346</v>
+      </c>
+      <c r="AB124" s="53" t="s">
         <v>347</v>
       </c>
-      <c r="AB124" s="53" t="s">
-        <v>348</v>
-      </c>
       <c r="AC124" s="54" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="125" spans="2:29" ht="17" x14ac:dyDescent="0.2">
@@ -12809,13 +12812,13 @@
         <v>1</v>
       </c>
       <c r="AA125" s="38" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="AB125" s="53" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="AC125" s="54" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="126" spans="2:29" ht="34" x14ac:dyDescent="0.2">
@@ -12885,13 +12888,13 @@
         <v>4960623.4808412148</v>
       </c>
       <c r="AA126" s="38" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="AB126" s="53" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AC126" s="54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="127" spans="2:29" x14ac:dyDescent="0.2">
@@ -12958,13 +12961,13 @@
         <v>2515644.7731143795</v>
       </c>
       <c r="AA129" s="38" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="AB129" s="53" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="AC129" s="54" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="130" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13006,13 +13009,13 @@
         <v>220752.12927619604</v>
       </c>
       <c r="AA130" s="38" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="AB130" s="53" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="AC130" s="54" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="131" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13054,13 +13057,13 @@
         <v>2294892.6438381835</v>
       </c>
       <c r="AA131" s="38" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="AB131" s="53" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="AC131" s="54" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="132" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13102,13 +13105,13 @@
         <v>0</v>
       </c>
       <c r="AA132" s="38" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="AB132" s="53" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="AC132" s="54" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="133" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13178,13 +13181,13 @@
         <v>220752.12927619604</v>
       </c>
       <c r="AA133" s="38" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="AB133" s="53" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="AC133" s="54" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="134" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13254,13 +13257,13 @@
         <v>220752.12927619604</v>
       </c>
       <c r="AA134" s="38" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="AB134" s="53" t="s">
-        <v>412</v>
+        <v>479</v>
       </c>
       <c r="AC134" s="54" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="135" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13351,13 +13354,13 @@
         <v>0.39928074986661122</v>
       </c>
       <c r="AA136" s="38" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="AB136" s="53" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="AC136" s="54" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AD136">
         <v>20</v>
@@ -13433,13 +13436,13 @@
         <v>4.4500883836231256E-2</v>
       </c>
       <c r="AA137" s="39" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="AB137" s="53" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="AC137" s="54" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AD137">
         <v>20</v>
@@ -13521,13 +13524,13 @@
         <v>220752.12927619604</v>
       </c>
       <c r="AA139" s="38" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="AB139" s="53" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="AC139" s="54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AD139">
         <v>20</v>
@@ -13600,13 +13603,13 @@
         <v>220752.12927619604</v>
       </c>
       <c r="AA140" s="38" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="AB140" s="53" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="AC140" s="54" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="141" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13676,13 +13679,13 @@
         <v>1</v>
       </c>
       <c r="AA141" s="38" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="AB141" s="53" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="AC141" s="54" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="142" spans="1:30" x14ac:dyDescent="0.2">
@@ -13777,13 +13780,13 @@
         <v>24163.802947564651</v>
       </c>
       <c r="AA144" s="38" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AB144" s="53" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="AC144" s="54" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="145" spans="2:30" x14ac:dyDescent="0.2">
@@ -13850,13 +13853,13 @@
         <v>6040.9507368911627</v>
       </c>
       <c r="AA145" s="38" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="AB145" s="53" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="AC145" s="54" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="146" spans="2:30" ht="17" x14ac:dyDescent="0.2">
@@ -13926,13 +13929,13 @@
         <v>55188.032319049009</v>
       </c>
       <c r="AA146" s="38" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="AB146" s="53" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="AC146" s="54" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="147" spans="2:30" ht="17" x14ac:dyDescent="0.2">
@@ -14002,13 +14005,13 @@
         <v>1866.5258081229777</v>
       </c>
       <c r="AA147" s="38" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="AB147" s="53" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="AC147" s="54" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="148" spans="2:30" ht="17" x14ac:dyDescent="0.2">
@@ -14078,13 +14081,13 @@
         <v>1354.9901734358141</v>
       </c>
       <c r="AA148" s="38" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="AB148" s="53" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="AC148" s="54" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="149" spans="2:30" x14ac:dyDescent="0.2">
@@ -14151,13 +14154,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA149" s="38" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AB149" s="53" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="AC149" s="54" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="150" spans="2:30" x14ac:dyDescent="0.2">
@@ -14271,13 +14274,13 @@
         <v>225107.35616181631</v>
       </c>
       <c r="AA154" s="38" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AB154" s="53" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="AC154" s="54" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="155" spans="2:30" x14ac:dyDescent="0.2">
@@ -14315,19 +14318,19 @@
     </row>
     <row r="156" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B156" s="38" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C156" s="31" t="s">
         <v>162</v>
       </c>
       <c r="AA156" s="38" t="s">
+        <v>393</v>
+      </c>
+      <c r="AB156" s="53" t="s">
         <v>394</v>
       </c>
-      <c r="AB156" s="53" t="s">
+      <c r="AC156" s="54" t="s">
         <v>395</v>
-      </c>
-      <c r="AC156" s="54" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="157" spans="2:30" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
updated carbon ledger variables and descriptions
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A037414-49F1-A147-8E76-3E5546D626CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29F1DFB-7242-B94B-ADE9-ABFF08AE6623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14800" yWindow="760" windowWidth="34560" windowHeight="20040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="5380" yWindow="760" windowWidth="34560" windowHeight="20040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="482">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -892,9 +892,6 @@
     <t>\hat{\alpha}(t)</t>
   </si>
   <si>
-    <t>\gamma</t>
-  </si>
-  <si>
     <t>arr_biomass_c_average_bg_stock_in_conversion_targets</t>
   </si>
   <si>
@@ -931,12 +928,6 @@
     <t xml:space="preserve">Fractional threshold for stock loss (compared to undisturbed forest levels) below which sequestration declines. </t>
   </si>
   <si>
-    <t xml:space="preserve">Initial steady-state storage in each class. Used in integration targets for NPP curve and as initial carbon storage condition. </t>
-  </si>
-  <si>
-    <t>Ratio of below-ground carbon stock to above-ground carbon stock in each forest type.</t>
-  </si>
-  <si>
     <t>Area of young forest that would be converted away assuming no protection (counterfactual).</t>
   </si>
   <si>
@@ -949,9 +940,6 @@
     <t>Fraction of biomass in each forest type that's converted to another land use class that is available for use to satisfy fuelwood and harvested wood product demands.</t>
   </si>
   <si>
-    <t>In healthy forest, available stock factor per unit area. Used to determine when average stocks fall below thresholds.</t>
-  </si>
-  <si>
     <t>Total area of forest protected.</t>
   </si>
   <si>
@@ -1090,9 +1078,6 @@
     <t>B</t>
   </si>
   <si>
-    <t>\overline{B_{avail}}</t>
-  </si>
-  <si>
     <t>b</t>
   </si>
   <si>
@@ -1174,9 +1159,6 @@
     <t>Matrix ($n_T \times 2$) soring average below ground stock contained In land use classes that forests transition into; used to estimate below-ground conversion losses of stock.</t>
   </si>
   <si>
-    <t>Matrix ($n_T \times 2$) storing avrage biomass stock per unit area required to be considered forest.</t>
-  </si>
-  <si>
     <t>Matrix ($n_T \times 2$) storing above ground biomass stock left from start of simulation if untouched (without degradation).</t>
   </si>
   <si>
@@ -1354,9 +1336,6 @@
     <t>vec_young_sf_curve_specification (T)</t>
   </si>
   <si>
-    <t>\tau</t>
-  </si>
-  <si>
     <t>z:\tau</t>
   </si>
   <si>
@@ -1487,6 +1466,27 @@
   </si>
   <si>
     <t>\overline{M}_0(t, v)</t>
+  </si>
+  <si>
+    <t>\tau(v)</t>
+  </si>
+  <si>
+    <t>Vector (dim $2$) storing avrage biomass stock per unit area required to be considered forest.</t>
+  </si>
+  <si>
+    <t>\overline{B_{avail}}(v)</t>
+  </si>
+  <si>
+    <t>\gamma(v)</t>
+  </si>
+  <si>
+    <t>Vector (dim $2$) storing available stock factor per unit area in healthy forest. Used to determine when average stocks fall below thresholds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vector (dim $2$) storing initial steady-state storage in each class. Used in integration targets for NPP curve and as initial carbon storage condition. </t>
+  </si>
+  <si>
+    <t>Vector (dim $2$) storing ratio of below-ground carbon stock to above-ground carbon stock in each forest type.</t>
   </si>
 </sst>
 </file>
@@ -7167,7 +7167,7 @@
     </row>
     <row r="5" spans="1:41" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="61" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>155</v>
@@ -7211,13 +7211,13 @@
       </c>
       <c r="Z5" s="55"/>
       <c r="AA5" s="24" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="AB5" s="40" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="AC5" s="27" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="AD5" s="36" t="s">
         <v>230</v>
@@ -7315,7 +7315,7 @@
     </row>
     <row r="7" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B7" s="38" t="s">
         <v>156</v>
@@ -7381,13 +7381,13 @@
         <v>249360</v>
       </c>
       <c r="AA7" s="38" t="s">
-        <v>455</v>
+        <v>448</v>
       </c>
       <c r="AB7" s="42" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="AC7" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="AE7" s="19">
         <v>0.01</v>
@@ -7414,7 +7414,7 @@
     </row>
     <row r="8" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B8" s="38" t="s">
         <v>157</v>
@@ -7482,13 +7482,13 @@
         <v>249801</v>
       </c>
       <c r="AA8" s="38" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="AB8" s="42" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="AC8" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="AE8" s="19">
         <v>0.05</v>
@@ -7515,7 +7515,7 @@
     </row>
     <row r="9" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B9" s="38" t="s">
         <v>222</v>
@@ -7569,13 +7569,13 @@
         <v>116</v>
       </c>
       <c r="AA9" s="38" t="s">
-        <v>457</v>
+        <v>450</v>
       </c>
       <c r="AB9" s="42" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="AC9" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="AE9" s="19">
         <v>0.12</v>
@@ -7602,7 +7602,7 @@
     </row>
     <row r="10" spans="1:41" ht="85" x14ac:dyDescent="0.2">
       <c r="A10" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B10" s="38" t="s">
         <v>221</v>
@@ -7645,10 +7645,10 @@
         <v>280</v>
       </c>
       <c r="AB10" s="42" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="AC10" s="43" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="AE10" s="19">
         <v>0.2</v>
@@ -7663,7 +7663,7 @@
     </row>
     <row r="11" spans="1:41" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B11" s="38" t="s">
         <v>219</v>
@@ -7706,10 +7706,10 @@
         <v>281</v>
       </c>
       <c r="AB11" s="42" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="AC11" s="43" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="AE11" s="19">
         <v>0.2</v>
@@ -7724,7 +7724,7 @@
     </row>
     <row r="12" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B12" s="38" t="s">
         <v>220</v>
@@ -7760,10 +7760,10 @@
         <v>279</v>
       </c>
       <c r="AB12" s="42" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="AC12" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="AE12" s="19">
         <v>0.36</v>
@@ -7778,7 +7778,7 @@
     </row>
     <row r="13" spans="1:41" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B13" s="38" t="s">
         <v>158</v>
@@ -7846,13 +7846,13 @@
         <v>249244</v>
       </c>
       <c r="AA13" s="38" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="AB13" s="42" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AC13" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="AE13" s="19"/>
       <c r="AF13" s="19"/>
@@ -7860,7 +7860,7 @@
     </row>
     <row r="14" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B14" s="38" t="s">
         <v>223</v>
@@ -7893,13 +7893,13 @@
         <v>0.7</v>
       </c>
       <c r="AA14" s="38" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="AB14" s="42" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="AC14" s="43" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="AE14" s="19">
         <v>0.6</v>
@@ -7914,7 +7914,7 @@
     </row>
     <row r="15" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B15" s="38" t="s">
         <v>244</v>
@@ -7971,13 +7971,13 @@
         <v>9</v>
       </c>
       <c r="AA15" s="38" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
       <c r="AB15" s="42" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="AC15" s="43" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="AE15" s="19"/>
       <c r="AF15" s="19"/>
@@ -7985,10 +7985,10 @@
     </row>
     <row r="16" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C16" s="31" t="s">
         <v>162</v>
@@ -8050,13 +8050,13 @@
         <v>1.728</v>
       </c>
       <c r="AA16" s="38" t="s">
-        <v>460</v>
+        <v>453</v>
       </c>
       <c r="AB16" s="42" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="AC16" s="43" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="AE16" s="19"/>
       <c r="AF16" s="19"/>
@@ -8064,10 +8064,10 @@
     </row>
     <row r="17" spans="1:33" ht="136" x14ac:dyDescent="0.2">
       <c r="A17" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="C17" s="31" t="s">
         <v>162</v>
@@ -8082,13 +8082,13 @@
         <v>0.37800893000000002</v>
       </c>
       <c r="AA17" s="38" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="AB17" s="42" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="AC17" s="43" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="AE17" s="19">
         <v>1.8</v>
@@ -8103,10 +8103,10 @@
     </row>
     <row r="18" spans="1:33" ht="102" x14ac:dyDescent="0.2">
       <c r="A18" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="C18" s="31" t="s">
         <v>162</v>
@@ -8124,13 +8124,13 @@
         <v>0.47800893</v>
       </c>
       <c r="AA18" s="38" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="AB18" s="42" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="AC18" s="43" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="AE18" s="19">
         <v>3</v>
@@ -8145,7 +8145,7 @@
     </row>
     <row r="19" spans="1:33" ht="136" x14ac:dyDescent="0.2">
       <c r="A19" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B19" s="38" t="s">
         <v>224</v>
@@ -8164,10 +8164,10 @@
         <v>282</v>
       </c>
       <c r="AB19" s="42" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="AC19" s="43" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="AE19" s="19">
         <v>6</v>
@@ -8182,7 +8182,7 @@
     </row>
     <row r="20" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B20" s="38" t="s">
         <v>226</v>
@@ -8200,13 +8200,13 @@
         <v>100</v>
       </c>
       <c r="AA20" s="38" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
       <c r="AB20" s="42" t="s">
-        <v>296</v>
+        <v>480</v>
       </c>
       <c r="AC20" s="43" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="AE20" s="19">
         <v>10</v>
@@ -8221,7 +8221,7 @@
     </row>
     <row r="21" spans="1:33" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B21" s="38" t="s">
         <v>228</v>
@@ -8239,13 +8239,13 @@
         <v>0.25</v>
       </c>
       <c r="AA21" s="38" t="s">
-        <v>283</v>
+        <v>478</v>
       </c>
       <c r="AB21" s="42" t="s">
-        <v>297</v>
+        <v>481</v>
       </c>
       <c r="AC21" s="44" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="AE21" s="19"/>
       <c r="AF21" s="19"/>
@@ -8253,7 +8253,7 @@
     </row>
     <row r="22" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B22" s="38" t="s">
         <v>275</v>
@@ -8273,13 +8273,13 @@
         <v>37.800893000000002</v>
       </c>
       <c r="AA22" s="38" t="s">
-        <v>437</v>
+        <v>475</v>
       </c>
       <c r="AB22" s="42" t="s">
-        <v>377</v>
+        <v>476</v>
       </c>
       <c r="AC22" s="43" t="s">
-        <v>438</v>
+        <v>431</v>
       </c>
       <c r="AE22" s="19">
         <v>12</v>
@@ -8294,7 +8294,7 @@
     </row>
     <row r="23" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B23" s="38" t="s">
         <v>227</v>
@@ -8314,13 +8314,13 @@
         <v>62.199106999999998</v>
       </c>
       <c r="AA23" s="38" t="s">
-        <v>349</v>
+        <v>477</v>
       </c>
       <c r="AB23" s="42" t="s">
-        <v>302</v>
+        <v>479</v>
       </c>
       <c r="AC23" s="43" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="AE23" s="19">
         <v>13.5</v>
@@ -8349,7 +8349,7 @@
     </row>
     <row r="25" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B25" s="38" t="s">
         <v>159</v>
@@ -8403,13 +8403,13 @@
         <v>49500</v>
       </c>
       <c r="AA25" s="38" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="AB25" s="42" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="AC25" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="AE25" s="19">
         <v>10</v>
@@ -8424,7 +8424,7 @@
     </row>
     <row r="26" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B26" s="38" t="s">
         <v>274</v>
@@ -8464,13 +8464,13 @@
         <v>0</v>
       </c>
       <c r="AA26" s="38" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="AB26" s="42" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="AC26" s="43" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="AE26" s="19">
         <v>6</v>
@@ -8485,7 +8485,7 @@
     </row>
     <row r="27" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B27" s="38" t="s">
         <v>160</v>
@@ -8553,13 +8553,13 @@
         <v>49500</v>
       </c>
       <c r="AA27" s="38" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
       <c r="AB27" s="42" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="AC27" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="AE27" s="19">
         <v>3</v>
@@ -8605,7 +8605,7 @@
     </row>
     <row r="29" spans="1:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B29" s="38" t="s">
         <v>273</v>
@@ -8626,18 +8626,18 @@
         <v>0.92</v>
       </c>
       <c r="AA29" s="38" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="AB29" s="42" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="AC29" s="43" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
     </row>
     <row r="30" spans="1:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B30" s="38" t="s">
         <v>229</v>
@@ -8662,13 +8662,13 @@
         <v>2E-3</v>
       </c>
       <c r="AA30" s="38" t="s">
-        <v>439</v>
+        <v>432</v>
       </c>
       <c r="AB30" s="42" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="AC30" s="43" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="31" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -8699,7 +8699,7 @@
     </row>
     <row r="33" spans="1:30" ht="51" x14ac:dyDescent="0.2">
       <c r="A33" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B33" s="38" t="s">
         <v>168</v>
@@ -8732,13 +8732,13 @@
         <v>2520000</v>
       </c>
       <c r="AA33" s="38" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="AB33" s="42" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="AC33" s="43" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
     </row>
     <row r="34" spans="1:30" x14ac:dyDescent="0.2">
@@ -8849,10 +8849,10 @@
     </row>
     <row r="38" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B38" s="37" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="C38" s="50" t="s">
         <v>174</v>
@@ -8940,21 +8940,21 @@
         <v>85</v>
       </c>
       <c r="AA38" s="38" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="AB38" s="42" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="AC38" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="39" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C39" s="50"/>
       <c r="F39" s="14" t="s">
@@ -9039,21 +9039,21 @@
         <v>80</v>
       </c>
       <c r="AA39" s="38" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="AB39" s="42" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="AC39" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="40" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B40" s="38" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C40" s="50"/>
       <c r="F40" s="14" t="s">
@@ -9137,13 +9137,13 @@
         <v>92</v>
       </c>
       <c r="AA40" s="38" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="AB40" s="42" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="AC40" s="43" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="41" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -9241,7 +9241,7 @@
     </row>
     <row r="43" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B43" s="51" t="s">
         <v>189</v>
@@ -9280,13 +9280,13 @@
         <v>0</v>
       </c>
       <c r="AA43" s="38" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="AB43" s="42" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="AC43" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="44" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -9402,7 +9402,7 @@
     </row>
     <row r="47" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A47" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B47" s="38" t="s">
         <v>190</v>
@@ -9440,13 +9440,13 @@
         <v>0</v>
       </c>
       <c r="AA47" s="38" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="AB47" s="42" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="AC47" s="43" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="48" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -9458,7 +9458,7 @@
     </row>
     <row r="49" spans="1:29" ht="51" x14ac:dyDescent="0.2">
       <c r="A49" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B49" s="51" t="s">
         <v>258</v>
@@ -9501,13 +9501,13 @@
         <v>0</v>
       </c>
       <c r="AA49" s="38" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="AB49" s="42" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="AC49" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="50" spans="1:29" ht="51" x14ac:dyDescent="0.2">
@@ -9629,7 +9629,7 @@
     </row>
     <row r="53" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A53" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B53" s="38" t="s">
         <v>259</v>
@@ -9667,18 +9667,18 @@
         <v>0</v>
       </c>
       <c r="AA53" s="38" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="AB53" s="42" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="AC53" s="43" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="54" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A54" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B54" s="38" t="s">
         <v>261</v>
@@ -9714,13 +9714,13 @@
         <v>0</v>
       </c>
       <c r="AA54" s="38" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="AB54" s="42" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
       <c r="AC54" s="43" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="55" spans="1:29" x14ac:dyDescent="0.2">
@@ -9730,7 +9730,7 @@
     </row>
     <row r="56" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B56" s="51" t="s">
         <v>191</v>
@@ -9770,13 +9770,13 @@
         <v>0</v>
       </c>
       <c r="AA56" s="38" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="AB56" s="42" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="AC56" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="57" spans="1:29" ht="34" x14ac:dyDescent="0.2">
@@ -9895,7 +9895,7 @@
     </row>
     <row r="60" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A60" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B60" s="38" t="s">
         <v>192</v>
@@ -9933,13 +9933,13 @@
         <v>0</v>
       </c>
       <c r="AA60" s="38" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AB60" s="42" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="AC60" s="43" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="61" spans="1:29" x14ac:dyDescent="0.2">
@@ -9949,7 +9949,7 @@
     </row>
     <row r="62" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A62" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B62" s="51" t="s">
         <v>178</v>
@@ -9989,13 +9989,13 @@
         <v>0.6</v>
       </c>
       <c r="AA62" s="38" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="AB62" s="42" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="AC62" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="63" spans="1:29" ht="34" x14ac:dyDescent="0.2">
@@ -10105,10 +10105,10 @@
     </row>
     <row r="66" spans="1:32" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="61" t="s">
+        <v>424</v>
+      </c>
+      <c r="B66" s="38" t="s">
         <v>430</v>
-      </c>
-      <c r="B66" s="38" t="s">
-        <v>436</v>
       </c>
       <c r="C66" s="31" t="s">
         <v>162</v>
@@ -10117,13 +10117,13 @@
         <v>49</v>
       </c>
       <c r="AA66" s="38" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="AB66" s="42" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="AC66" s="43" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="67" spans="1:32" x14ac:dyDescent="0.2">
@@ -10133,7 +10133,7 @@
     </row>
     <row r="68" spans="1:32" ht="34" x14ac:dyDescent="0.2">
       <c r="A68" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B68" s="51" t="s">
         <v>233</v>
@@ -10173,13 +10173,13 @@
         <v>113.71737449773646</v>
       </c>
       <c r="AA68" s="38" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="AB68" s="42" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="AC68" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="69" spans="1:32" ht="34" x14ac:dyDescent="0.2">
@@ -10286,7 +10286,7 @@
     </row>
     <row r="73" spans="1:32" ht="34" x14ac:dyDescent="0.2">
       <c r="A73" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B73" s="51" t="s">
         <v>231</v>
@@ -10325,13 +10325,13 @@
         <v>0</v>
       </c>
       <c r="AA73" s="38" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="AB73" s="42" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="AC73" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="74" spans="1:32" ht="34" x14ac:dyDescent="0.2">
@@ -10451,7 +10451,7 @@
     </row>
     <row r="77" spans="1:32" ht="34" x14ac:dyDescent="0.2">
       <c r="A77" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B77" s="38" t="s">
         <v>232</v>
@@ -10491,13 +10491,13 @@
         <v>0</v>
       </c>
       <c r="AA77" s="45" t="s">
-        <v>445</v>
+        <v>438</v>
       </c>
       <c r="AB77" s="42" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
       <c r="AC77" s="43" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="AF77" t="s">
         <v>106</v>
@@ -10517,10 +10517,10 @@
     </row>
     <row r="79" spans="1:32" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B79" s="37" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="C79" s="50" t="s">
         <v>174</v>
@@ -10550,13 +10550,13 @@
         <v>0</v>
       </c>
       <c r="AA79" s="38" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="AB79" s="42" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="AC79" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="AD79" t="s">
         <v>86</v>
@@ -10564,10 +10564,10 @@
     </row>
     <row r="80" spans="1:32" ht="34" x14ac:dyDescent="0.2">
       <c r="A80" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B80" s="37" t="s">
-        <v>443</v>
+        <v>436</v>
       </c>
       <c r="C80" s="50"/>
       <c r="F80" s="14" t="s">
@@ -10630,13 +10630,13 @@
         <v>0</v>
       </c>
       <c r="AA80" s="38" t="s">
-        <v>452</v>
+        <v>445</v>
       </c>
       <c r="AB80" s="42" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="AC80" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="81" spans="1:29" ht="34" x14ac:dyDescent="0.2">
@@ -10879,10 +10879,10 @@
     </row>
     <row r="86" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A86" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B86" s="37" t="s">
-        <v>442</v>
+        <v>435</v>
       </c>
       <c r="C86" s="50" t="s">
         <v>174</v>
@@ -10943,21 +10943,21 @@
         <v>0.6</v>
       </c>
       <c r="AA86" s="37" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="AB86" s="42" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="AC86" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="87" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A87" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B87" s="37" t="s">
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="C87" s="50"/>
       <c r="F87" s="14" t="s">
@@ -11016,13 +11016,13 @@
         <v>0.36</v>
       </c>
       <c r="AA87" s="37" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="AB87" s="42" t="s">
-        <v>440</v>
+        <v>433</v>
       </c>
       <c r="AC87" s="43" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="88" spans="1:29" ht="34" x14ac:dyDescent="0.2">
@@ -11156,7 +11156,7 @@
     </row>
     <row r="91" spans="1:29" ht="51" x14ac:dyDescent="0.2">
       <c r="A91" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B91" s="49" t="s">
         <v>202</v>
@@ -11196,13 +11196,13 @@
         <v>9.8621113109027395E-2</v>
       </c>
       <c r="AA91" s="37" t="s">
-        <v>468</v>
+        <v>461</v>
       </c>
       <c r="AB91" s="42" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="AC91" s="43" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="92" spans="1:29" ht="51" x14ac:dyDescent="0.2">
@@ -11321,10 +11321,10 @@
     </row>
     <row r="95" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A95" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B95" s="37" t="s">
-        <v>464</v>
+        <v>457</v>
       </c>
       <c r="C95" s="28"/>
       <c r="F95" s="14"/>
@@ -11357,13 +11357,13 @@
         <v>0.17633270956878355</v>
       </c>
       <c r="AA95" s="37" t="s">
-        <v>467</v>
+        <v>460</v>
       </c>
       <c r="AB95" s="42" t="s">
-        <v>465</v>
+        <v>458</v>
       </c>
       <c r="AC95" s="43" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
     </row>
     <row r="96" spans="1:29" x14ac:dyDescent="0.2">
@@ -11373,7 +11373,7 @@
     </row>
     <row r="97" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A97" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B97" s="49" t="s">
         <v>207</v>
@@ -11413,13 +11413,13 @@
         <v>113.71737449773644</v>
       </c>
       <c r="AA97" s="38" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="AB97" s="42" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="AC97" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="98" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -11544,7 +11544,7 @@
     </row>
     <row r="102" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B102" s="49" t="s">
         <v>208</v>
@@ -11585,13 +11585,13 @@
         <v>28.429343624434111</v>
       </c>
       <c r="AA102" s="38" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="AB102" s="42" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="AC102" s="43" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="103" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -11814,7 +11814,7 @@
     </row>
     <row r="110" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A110" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B110" s="38" t="s">
         <v>235</v>
@@ -11882,18 +11882,18 @@
         <v>24936000</v>
       </c>
       <c r="AA110" s="38" t="s">
-        <v>480</v>
+        <v>473</v>
       </c>
       <c r="AB110" s="42" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="AC110" s="43" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="111" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A111" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B111" s="38" t="s">
         <v>181</v>
@@ -11959,18 +11959,18 @@
         <v>1</v>
       </c>
       <c r="AA111" s="38" t="s">
-        <v>454</v>
+        <v>447</v>
       </c>
       <c r="AB111" s="42" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="AC111" s="43" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="112" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A112" s="61" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B112" s="38" t="s">
         <v>182</v>
@@ -12038,16 +12038,19 @@
         <v>0.92</v>
       </c>
       <c r="AA112" s="38" t="s">
-        <v>479</v>
+        <v>472</v>
       </c>
       <c r="AB112" s="42" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="AC112" s="43" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="113" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="113" spans="1:29" ht="34" x14ac:dyDescent="0.2">
+      <c r="A113" s="61" t="s">
+        <v>424</v>
+      </c>
       <c r="B113" s="38" t="s">
         <v>236</v>
       </c>
@@ -12114,16 +12117,19 @@
         <v>15778712.754563004</v>
       </c>
       <c r="AA113" s="38" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
       <c r="AB113" s="42" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="AC113" s="43" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="114" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="114" spans="1:29" ht="34" x14ac:dyDescent="0.2">
+      <c r="A114" s="61" t="s">
+        <v>424</v>
+      </c>
       <c r="B114" s="38" t="s">
         <v>239</v>
       </c>
@@ -12190,16 +12196,19 @@
         <v>63.276839727955583</v>
       </c>
       <c r="AA114" s="38" t="s">
-        <v>477</v>
+        <v>470</v>
       </c>
       <c r="AB114" s="42" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="AC114" s="43" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="115" spans="2:29" ht="68" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="115" spans="1:29" ht="68" x14ac:dyDescent="0.2">
+      <c r="A115" s="61" t="s">
+        <v>424</v>
+      </c>
       <c r="B115" s="38" t="s">
         <v>277</v>
       </c>
@@ -12266,21 +12275,21 @@
         <v>25.475946727955581</v>
       </c>
       <c r="AA115" s="38" t="s">
-        <v>478</v>
+        <v>471</v>
       </c>
       <c r="AB115" s="46" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="AC115" s="43" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="116" spans="2:29" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="116" spans="1:29" x14ac:dyDescent="0.2">
       <c r="F116" s="13"/>
       <c r="AB116" s="42"/>
       <c r="AC116" s="43"/>
     </row>
-    <row r="117" spans="2:29" ht="17" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="F117" s="11" t="s">
         <v>58</v>
       </c>
@@ -12301,7 +12310,7 @@
       <c r="AB117" s="42"/>
       <c r="AC117" s="43"/>
     </row>
-    <row r="118" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="B118" s="38" t="s">
         <v>241</v>
       </c>
@@ -12371,7 +12380,7 @@
       <c r="AB118" s="42"/>
       <c r="AC118" s="43"/>
     </row>
-    <row r="119" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="B119" s="38" t="s">
         <v>240</v>
       </c>
@@ -12410,16 +12419,16 @@
         <v>215.49749504124878</v>
       </c>
       <c r="AA119" s="38" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="AB119" s="42" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="AC119" s="43" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="120" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="120" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="B120" s="38" t="s">
         <v>237</v>
       </c>
@@ -12486,16 +12495,16 @@
         <v>15778928.252058046</v>
       </c>
       <c r="AA120" s="38" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="AB120" s="42" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="AC120" s="43" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="121" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="121" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="B121" s="38" t="s">
         <v>238</v>
       </c>
@@ -12562,16 +12571,16 @@
         <v>3944732.0630145115</v>
       </c>
       <c r="AA121" s="38" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="AB121" s="42" t="s">
-        <v>470</v>
+        <v>463</v>
       </c>
       <c r="AC121" s="43" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="122" spans="2:29" ht="17" x14ac:dyDescent="0.2">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="122" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="B122" s="38" t="s">
         <v>276</v>
       </c>
@@ -12638,16 +12647,16 @@
         <v>7340.1134084428477</v>
       </c>
       <c r="AA122" s="38" t="s">
-        <v>471</v>
+        <v>464</v>
       </c>
       <c r="AB122" s="42" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="AC122" s="43" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="123" spans="2:29" ht="51" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="123" spans="1:29" ht="51" x14ac:dyDescent="0.2">
       <c r="B123" s="38" t="s">
         <v>260</v>
       </c>
@@ -12714,16 +12723,16 @@
         <v>1044</v>
       </c>
       <c r="AA123" s="38" t="s">
-        <v>474</v>
+        <v>467</v>
       </c>
       <c r="AB123" s="42" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="AC123" s="43" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="124" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="124" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="B124" s="38" t="s">
         <v>278</v>
       </c>
@@ -12790,16 +12799,16 @@
         <v>4407.2793859099929</v>
       </c>
       <c r="AA124" s="38" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="AB124" s="42" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="AC124" s="43" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="125" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="125" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="B125" s="38" t="s">
         <v>253</v>
       </c>
@@ -12838,16 +12847,16 @@
         <v>9842.1904497703563</v>
       </c>
       <c r="AA125" s="38" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="AB125" s="42" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="AC125" s="43" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="126" spans="2:29" ht="34" x14ac:dyDescent="0.2">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="126" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="B126" s="38" t="s">
         <v>254</v>
       </c>
@@ -12914,16 +12923,16 @@
         <v>0.44779456447246724</v>
       </c>
       <c r="AA126" s="38" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="AB126" s="42" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="AC126" s="43" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="127" spans="2:29" ht="68" x14ac:dyDescent="0.2">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="127" spans="1:29" ht="68" x14ac:dyDescent="0.2">
       <c r="B127" s="38" t="s">
         <v>183</v>
       </c>
@@ -12990,16 +12999,16 @@
         <v>5088667.5032287594</v>
       </c>
       <c r="AA127" s="38" t="s">
-        <v>476</v>
+        <v>469</v>
       </c>
       <c r="AB127" s="42" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="AC127" s="43" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="128" spans="2:29" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="128" spans="1:29" x14ac:dyDescent="0.2">
       <c r="AB128" s="42"/>
       <c r="AC128" s="43"/>
     </row>
@@ -13063,13 +13072,13 @@
         <v>2510157.8095502295</v>
       </c>
       <c r="AA130" s="38" t="s">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="AB130" s="42" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="AC130" s="43" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
     </row>
     <row r="131" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -13111,13 +13120,13 @@
         <v>388638.22348903998</v>
       </c>
       <c r="AA131" s="38" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="AB131" s="42" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
       <c r="AC131" s="43" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="132" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -13159,13 +13168,13 @@
         <v>2121519.5860611894</v>
       </c>
       <c r="AA132" s="38" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="AB132" s="42" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="AC132" s="43" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="133" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -13207,13 +13216,13 @@
         <v>0</v>
       </c>
       <c r="AA133" s="38" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="AB133" s="42" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="AC133" s="43" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="134" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -13283,13 +13292,13 @@
         <v>336166.07900932123</v>
       </c>
       <c r="AA134" s="38" t="s">
-        <v>447</v>
+        <v>440</v>
       </c>
       <c r="AB134" s="42" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="AC134" s="43" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
     </row>
     <row r="135" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -13359,13 +13368,13 @@
         <v>336166.07900932123</v>
       </c>
       <c r="AA135" s="38" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="AB135" s="42" t="s">
-        <v>453</v>
+        <v>446</v>
       </c>
       <c r="AC135" s="43" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
     </row>
     <row r="136" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13456,13 +13465,13 @@
         <v>0.40958701751064658</v>
       </c>
       <c r="AA137" s="38" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="AB137" s="42" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="AC137" s="43" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="AD137">
         <v>20</v>
@@ -13470,7 +13479,7 @@
     </row>
     <row r="138" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="A138" s="48" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B138" s="38" t="s">
         <v>184</v>
@@ -13538,13 +13547,13 @@
         <v>6.6061710417515754E-2</v>
       </c>
       <c r="AA138" s="39" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="AB138" s="42" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="AC138" s="43" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="AD138">
         <v>20</v>
@@ -13626,13 +13635,13 @@
         <v>336166.07900932123</v>
       </c>
       <c r="AA140" s="38" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="AB140" s="42" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="AC140" s="43" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="AD140">
         <v>20</v>
@@ -13705,13 +13714,13 @@
         <v>388638.22348903998</v>
       </c>
       <c r="AA141" s="38" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="AB141" s="42" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="AC141" s="43" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
     </row>
     <row r="142" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -13781,13 +13790,13 @@
         <v>0.86498460185247705</v>
       </c>
       <c r="AA142" s="38" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="AB142" s="42" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="AC142" s="43" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
     </row>
     <row r="143" spans="1:30" x14ac:dyDescent="0.2">
@@ -13882,18 +13891,18 @@
         <v>24233.450635277597</v>
       </c>
       <c r="AA145" s="38" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
       <c r="AB145" s="42" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="AC145" s="43" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B146" s="38" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C146" s="33" t="s">
         <v>163</v>
@@ -13955,13 +13964,13 @@
         <v>6058.3626588193993</v>
       </c>
       <c r="AA146" s="38" t="s">
-        <v>463</v>
+        <v>456</v>
       </c>
       <c r="AB146" s="42" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="AC146" s="43" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="147" spans="2:29" ht="51" x14ac:dyDescent="0.2">
@@ -14031,13 +14040,13 @@
         <v>84041.519752330307</v>
       </c>
       <c r="AA147" s="38" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="AB147" s="42" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="AC147" s="43" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="148" spans="2:29" ht="34" x14ac:dyDescent="0.2">
@@ -14107,13 +14116,13 @@
         <v>1888.8340225328548</v>
       </c>
       <c r="AA148" s="38" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="AB148" s="42" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="AC148" s="43" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="149" spans="2:29" ht="34" x14ac:dyDescent="0.2">
@@ -14183,18 +14192,18 @@
         <v>1373.5803521107118</v>
       </c>
       <c r="AA149" s="38" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="AB149" s="42" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="AC149" s="43" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B150" s="38" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C150" s="33" t="s">
         <v>163</v>
@@ -14256,13 +14265,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA150" s="38" t="s">
+        <v>339</v>
+      </c>
+      <c r="AB150" s="42" t="s">
+        <v>390</v>
+      </c>
+      <c r="AC150" s="43" t="s">
         <v>343</v>
-      </c>
-      <c r="AB150" s="42" t="s">
-        <v>396</v>
-      </c>
-      <c r="AC150" s="43" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -14376,13 +14385,13 @@
         <v>398480.41393881035</v>
       </c>
       <c r="AA155" s="38" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="AB155" s="42" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="AC155" s="43" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -14420,19 +14429,19 @@
     </row>
     <row r="157" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B157" s="38" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="C157" s="31" t="s">
         <v>162</v>
       </c>
       <c r="AA157" s="38" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="AB157" s="42" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="AC157" s="43" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
     </row>
     <row r="158" spans="2:29" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
some additional work on validation workbook
</commit_message>
<xml_diff>
--- a/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
+++ b/sisepuede/ref/validation_workbooks/carbon_ledger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/validation_workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B5603A1-8EBF-334C-9F4E-C5B2926DDFCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D111AA-CE75-364C-8638-1EC89673CD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="25580" windowHeight="20040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
+    <workbookView xWindow="3280" yWindow="760" windowWidth="34200" windowHeight="20040" activeTab="2" xr2:uid="{49B92464-5B50-C04B-B571-E5276F1DC1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="492">
   <si>
     <t>forest_primary_c_ha</t>
   </si>
@@ -916,9 +916,6 @@
     <t>\overline{Y}^*(t, u)</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fractional threshold for stock loss (compared to undisturbed forest levels) below which sequestration declines. </t>
   </si>
   <si>
@@ -1273,9 +1270,6 @@
     <t>Vector ($n_T$) storing unmet demand for removals from original forests.</t>
   </si>
   <si>
-    <t>Vector ($n_T$) storing removals from young forests, excluding conversions.  Always $\leq d_{rmv}$.</t>
-  </si>
-  <si>
     <t>Vector ($n_T$) giving total removals supplied.</t>
   </si>
   <si>
@@ -1345,9 +1339,6 @@
     <t>\overline{y}_{avail}(t)</t>
   </si>
   <si>
-    <t>r^{(y)}_{rmv}(t)</t>
-  </si>
-  <si>
     <t>R^{(0)}_{rmv}(t, v)</t>
   </si>
   <si>
@@ -1357,9 +1348,6 @@
     <t>u^{(0)}_{rmv}(t)</t>
   </si>
   <si>
-    <t>r^{(0)}_{rmv}(t)</t>
-  </si>
-  <si>
     <t>d_{rmv}(t)</t>
   </si>
   <si>
@@ -1381,9 +1369,6 @@
     <t>A_{out}(t, v)</t>
   </si>
   <si>
-    <t>A^*(t + 1, v)</t>
-  </si>
-  <si>
     <t>\overline{\eta}(t, v)</t>
   </si>
   <si>
@@ -1514,6 +1499,24 @@
   </si>
   <si>
     <t>vec_biomass_c_removals_young_priority_frac</t>
+  </si>
+  <si>
+    <t>Vector ($n_T$) storing removals from young forests, excluding conversions, after original forests.  Always $\leq d_{rmv}$.</t>
+  </si>
+  <si>
+    <t>r^{(y)}_{post}(t)</t>
+  </si>
+  <si>
+    <t>r^{(0)}(t)</t>
+  </si>
+  <si>
+    <t>r^{(y)}_{pre}(t)</t>
+  </si>
+  <si>
+    <t>Vector ($n_T$) storing removals from young forests, excluding conversions, before original forests.  Always $\leq d_{rmv}$.</t>
+  </si>
+  <si>
+    <t>- NOTE: is A^*(t + 1, v)</t>
   </si>
 </sst>
 </file>
@@ -1673,7 +1676,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1849,6 +1852,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7005,18 +7011,18 @@
     <col min="8" max="8" width="15.1640625" style="4" customWidth="1"/>
     <col min="9" max="9" width="11.5" style="5" customWidth="1"/>
     <col min="10" max="11" width="13.33203125" style="4" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" style="5" customWidth="1"/>
-    <col min="13" max="14" width="13.33203125" style="4" customWidth="1"/>
-    <col min="15" max="15" width="21.1640625" style="5" customWidth="1"/>
-    <col min="16" max="16" width="21.1640625" style="4" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" style="5" customWidth="1"/>
-    <col min="19" max="20" width="13.33203125" style="4" customWidth="1"/>
-    <col min="21" max="21" width="9.1640625" style="5" customWidth="1"/>
-    <col min="22" max="22" width="13.33203125" style="4" customWidth="1"/>
-    <col min="23" max="23" width="12.5" style="4" customWidth="1"/>
-    <col min="24" max="24" width="9.1640625" style="5" customWidth="1"/>
-    <col min="25" max="26" width="13.33203125" style="4" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" style="5" hidden="1" customWidth="1"/>
+    <col min="13" max="14" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="21.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="21.1640625" style="4" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" style="5" hidden="1" customWidth="1"/>
+    <col min="19" max="20" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="9.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="13.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="12.5" style="4" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="9.1640625" style="5" hidden="1" customWidth="1"/>
+    <col min="25" max="26" width="13.33203125" style="4" hidden="1" customWidth="1"/>
     <col min="27" max="27" width="24" style="24" customWidth="1"/>
     <col min="28" max="28" width="64.5" style="47" customWidth="1"/>
     <col min="29" max="29" width="14.6640625" style="48" customWidth="1"/>
@@ -7194,7 +7200,7 @@
     </row>
     <row r="5" spans="1:41" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="50" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B5" s="24" t="s">
         <v>155</v>
@@ -7238,13 +7244,13 @@
       </c>
       <c r="Z5" s="52"/>
       <c r="AA5" s="24" t="s">
+        <v>301</v>
+      </c>
+      <c r="AB5" s="40" t="s">
         <v>302</v>
       </c>
-      <c r="AB5" s="40" t="s">
-        <v>303</v>
-      </c>
       <c r="AC5" s="27" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AD5" s="36" t="s">
         <v>229</v>
@@ -7342,7 +7348,7 @@
     </row>
     <row r="7" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B7" s="38" t="s">
         <v>156</v>
@@ -7408,13 +7414,13 @@
         <v>249360</v>
       </c>
       <c r="AA7" s="38" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="AB7" s="42" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AC7" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AE7" s="19">
         <v>0.01</v>
@@ -7441,7 +7447,7 @@
     </row>
     <row r="8" spans="1:41" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B8" s="38" t="s">
         <v>157</v>
@@ -7509,13 +7515,13 @@
         <v>249801</v>
       </c>
       <c r="AA8" s="38" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="AB8" s="42" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AC8" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AE8" s="19">
         <v>0.05</v>
@@ -7542,7 +7548,7 @@
     </row>
     <row r="9" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B9" s="38" t="s">
         <v>221</v>
@@ -7596,13 +7602,13 @@
         <v>116</v>
       </c>
       <c r="AA9" s="38" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="AB9" s="42" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="AC9" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AE9" s="19">
         <v>0.12</v>
@@ -7629,7 +7635,7 @@
     </row>
     <row r="10" spans="1:41" ht="85" x14ac:dyDescent="0.2">
       <c r="A10" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B10" s="38" t="s">
         <v>220</v>
@@ -7672,10 +7678,10 @@
         <v>279</v>
       </c>
       <c r="AB10" s="42" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="AC10" s="43" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="AE10" s="19">
         <v>0.2</v>
@@ -7690,7 +7696,7 @@
     </row>
     <row r="11" spans="1:41" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B11" s="38" t="s">
         <v>218</v>
@@ -7733,10 +7739,10 @@
         <v>280</v>
       </c>
       <c r="AB11" s="42" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AC11" s="43" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="AE11" s="19">
         <v>0.2</v>
@@ -7751,10 +7757,10 @@
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A12" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="C12" s="28"/>
       <c r="G12" s="4">
@@ -7814,10 +7820,10 @@
         <v>116</v>
       </c>
       <c r="AA12" s="38" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="AB12" s="42" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="AC12" s="43"/>
       <c r="AE12" s="19"/>
@@ -7826,7 +7832,7 @@
     </row>
     <row r="13" spans="1:41" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B13" s="38" t="s">
         <v>219</v>
@@ -7862,10 +7868,10 @@
         <v>278</v>
       </c>
       <c r="AB13" s="42" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="AC13" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AE13" s="19">
         <v>0.36</v>
@@ -7880,7 +7886,7 @@
     </row>
     <row r="14" spans="1:41" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B14" s="38" t="s">
         <v>158</v>
@@ -7947,14 +7953,12 @@
         <f>MAX(Z7-Z9,0)</f>
         <v>249244</v>
       </c>
-      <c r="AA14" s="38" t="s">
-        <v>446</v>
-      </c>
-      <c r="AB14" s="42" t="s">
-        <v>291</v>
+      <c r="AA14" s="38"/>
+      <c r="AB14" s="62" t="s">
+        <v>491</v>
       </c>
       <c r="AC14" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AE14" s="19"/>
       <c r="AF14" s="19"/>
@@ -7962,7 +7966,7 @@
     </row>
     <row r="15" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B15" s="38" t="s">
         <v>222</v>
@@ -7995,13 +7999,13 @@
         <v>0.7</v>
       </c>
       <c r="AA15" s="38" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AB15" s="42" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="AC15" s="43" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="AE15" s="19">
         <v>0.6</v>
@@ -8016,7 +8020,7 @@
     </row>
     <row r="16" spans="1:41" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B16" s="38" t="s">
         <v>243</v>
@@ -8073,13 +8077,13 @@
         <v>9</v>
       </c>
       <c r="AA16" s="38" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="AB16" s="42" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AC16" s="43" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AE16" s="19"/>
       <c r="AF16" s="19"/>
@@ -8087,7 +8091,7 @@
     </row>
     <row r="17" spans="1:33" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B17" s="38" t="s">
         <v>282</v>
@@ -8152,13 +8156,13 @@
         <v>1.728</v>
       </c>
       <c r="AA17" s="38" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
       <c r="AB17" s="42" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AC17" s="43" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AE17" s="19"/>
       <c r="AF17" s="19"/>
@@ -8166,10 +8170,10 @@
     </row>
     <row r="18" spans="1:33" ht="136" x14ac:dyDescent="0.2">
       <c r="A18" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="C18" s="31" t="s">
         <v>162</v>
@@ -8184,13 +8188,13 @@
         <v>0.37800893000000002</v>
       </c>
       <c r="AA18" s="38" t="s">
+        <v>412</v>
+      </c>
+      <c r="AB18" s="42" t="s">
         <v>414</v>
       </c>
-      <c r="AB18" s="42" t="s">
-        <v>416</v>
-      </c>
       <c r="AC18" s="43" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="AE18" s="19">
         <v>1.8</v>
@@ -8205,10 +8209,10 @@
     </row>
     <row r="19" spans="1:33" ht="102" x14ac:dyDescent="0.2">
       <c r="A19" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B19" s="38" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C19" s="31" t="s">
         <v>162</v>
@@ -8226,13 +8230,13 @@
         <v>0.47800893</v>
       </c>
       <c r="AA19" s="38" t="s">
+        <v>413</v>
+      </c>
+      <c r="AB19" s="42" t="s">
         <v>415</v>
       </c>
-      <c r="AB19" s="42" t="s">
-        <v>417</v>
-      </c>
       <c r="AC19" s="43" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="AE19" s="19">
         <v>3</v>
@@ -8247,7 +8251,7 @@
     </row>
     <row r="20" spans="1:33" ht="136" x14ac:dyDescent="0.2">
       <c r="A20" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B20" s="38" t="s">
         <v>223</v>
@@ -8266,10 +8270,10 @@
         <v>281</v>
       </c>
       <c r="AB20" s="42" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AC20" s="43" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="AE20" s="19">
         <v>6</v>
@@ -8284,7 +8288,7 @@
     </row>
     <row r="21" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B21" s="38" t="s">
         <v>225</v>
@@ -8302,13 +8306,13 @@
         <v>100</v>
       </c>
       <c r="AA21" s="38" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="AB21" s="42" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="AC21" s="43" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="AE21" s="19">
         <v>10</v>
@@ -8323,7 +8327,7 @@
     </row>
     <row r="22" spans="1:33" ht="51" x14ac:dyDescent="0.2">
       <c r="A22" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B22" s="38" t="s">
         <v>227</v>
@@ -8341,13 +8345,13 @@
         <v>0.25</v>
       </c>
       <c r="AA22" s="38" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
       <c r="AB22" s="42" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="AC22" s="44" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="AE22" s="19"/>
       <c r="AF22" s="19"/>
@@ -8355,7 +8359,7 @@
     </row>
     <row r="23" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B23" s="38" t="s">
         <v>274</v>
@@ -8375,13 +8379,13 @@
         <v>37.800893000000002</v>
       </c>
       <c r="AA23" s="38" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
       <c r="AB23" s="42" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="AC23" s="43" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="AE23" s="19">
         <v>12</v>
@@ -8396,7 +8400,7 @@
     </row>
     <row r="24" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B24" s="38" t="s">
         <v>226</v>
@@ -8416,13 +8420,13 @@
         <v>62.199106999999998</v>
       </c>
       <c r="AA24" s="38" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="AB24" s="42" t="s">
-        <v>469</v>
+        <v>464</v>
       </c>
       <c r="AC24" s="43" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="AE24" s="19">
         <v>13.5</v>
@@ -8451,7 +8455,7 @@
     </row>
     <row r="26" spans="1:33" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B26" s="38" t="s">
         <v>159</v>
@@ -8505,13 +8509,13 @@
         <v>49500</v>
       </c>
       <c r="AA26" s="38" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="AB26" s="42" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="AC26" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AE26" s="19">
         <v>10</v>
@@ -8526,7 +8530,7 @@
     </row>
     <row r="27" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B27" s="38" t="s">
         <v>273</v>
@@ -8566,13 +8570,13 @@
         <v>0</v>
       </c>
       <c r="AA27" s="38" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="AB27" s="42" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="AC27" s="43" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="AE27" s="19">
         <v>6</v>
@@ -8587,7 +8591,7 @@
     </row>
     <row r="28" spans="1:33" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B28" s="38" t="s">
         <v>160</v>
@@ -8655,13 +8659,13 @@
         <v>49500</v>
       </c>
       <c r="AA28" s="38" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="AB28" s="42" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="AC28" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AE28" s="19">
         <v>3</v>
@@ -8707,7 +8711,7 @@
     </row>
     <row r="30" spans="1:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B30" s="38" t="s">
         <v>272</v>
@@ -8728,18 +8732,18 @@
         <v>0.92</v>
       </c>
       <c r="AA30" s="38" t="s">
+        <v>318</v>
+      </c>
+      <c r="AB30" s="42" t="s">
         <v>319</v>
       </c>
-      <c r="AB30" s="42" t="s">
-        <v>320</v>
-      </c>
       <c r="AC30" s="43" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="31" spans="1:33" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B31" s="38" t="s">
         <v>228</v>
@@ -8764,13 +8768,13 @@
         <v>2E-3</v>
       </c>
       <c r="AA31" s="38" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="AB31" s="42" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AC31" s="43" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="32" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -8801,7 +8805,7 @@
     </row>
     <row r="34" spans="1:30" ht="51" x14ac:dyDescent="0.2">
       <c r="A34" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B34" s="38" t="s">
         <v>168</v>
@@ -8837,15 +8841,18 @@
         <v>285</v>
       </c>
       <c r="AB34" s="42" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AC34" s="43" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="35" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A35" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B35" s="38" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="C35" s="31" t="s">
         <v>162</v>
@@ -8873,10 +8880,10 @@
         <v>0.5</v>
       </c>
       <c r="AA35" s="38" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="AB35" s="42" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="AC35" s="43"/>
     </row>
@@ -8988,10 +8995,10 @@
     </row>
     <row r="40" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B40" s="37" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C40" s="55" t="s">
         <v>174</v>
@@ -9079,21 +9086,21 @@
         <v>85</v>
       </c>
       <c r="AA40" s="38" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AB40" s="42" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AC40" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="41" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B41" s="38" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C41" s="55"/>
       <c r="F41" s="14" t="s">
@@ -9178,21 +9185,21 @@
         <v>80</v>
       </c>
       <c r="AA41" s="38" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="AB41" s="42" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AC41" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="42" spans="1:30" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B42" s="38" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C42" s="55"/>
       <c r="F42" s="14" t="s">
@@ -9276,13 +9283,13 @@
         <v>92</v>
       </c>
       <c r="AA42" s="38" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AB42" s="42" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="AC42" s="43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="43" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -9380,7 +9387,7 @@
     </row>
     <row r="45" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B45" s="56" t="s">
         <v>189</v>
@@ -9422,10 +9429,10 @@
         <v>286</v>
       </c>
       <c r="AB45" s="42" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="AC45" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="46" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -9541,7 +9548,7 @@
     </row>
     <row r="49" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A49" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B49" s="38" t="s">
         <v>190</v>
@@ -9582,10 +9589,10 @@
         <v>287</v>
       </c>
       <c r="AB49" s="42" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="AC49" s="43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="50" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -9597,7 +9604,7 @@
     </row>
     <row r="51" spans="1:29" ht="51" x14ac:dyDescent="0.2">
       <c r="A51" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B51" s="56" t="s">
         <v>257</v>
@@ -9640,13 +9647,13 @@
         <v>0</v>
       </c>
       <c r="AA51" s="38" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="AB51" s="42" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="AC51" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="52" spans="1:29" ht="51" x14ac:dyDescent="0.2">
@@ -9768,7 +9775,7 @@
     </row>
     <row r="55" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A55" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B55" s="38" t="s">
         <v>258</v>
@@ -9806,18 +9813,18 @@
         <v>0</v>
       </c>
       <c r="AA55" s="38" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AB55" s="42" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="AC55" s="43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="56" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A56" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B56" s="38" t="s">
         <v>260</v>
@@ -9853,13 +9860,13 @@
         <v>0</v>
       </c>
       <c r="AA56" s="38" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AB56" s="42" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="AC56" s="43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="57" spans="1:29" x14ac:dyDescent="0.2">
@@ -9869,7 +9876,7 @@
     </row>
     <row r="58" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A58" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B58" s="56" t="s">
         <v>191</v>
@@ -9912,10 +9919,10 @@
         <v>288</v>
       </c>
       <c r="AB58" s="42" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="AC58" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="59" spans="1:29" ht="34" x14ac:dyDescent="0.2">
@@ -10034,7 +10041,7 @@
     </row>
     <row r="62" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A62" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B62" s="38" t="s">
         <v>192</v>
@@ -10075,10 +10082,10 @@
         <v>289</v>
       </c>
       <c r="AB62" s="42" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="AC62" s="43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="63" spans="1:29" x14ac:dyDescent="0.2">
@@ -10088,7 +10095,7 @@
     </row>
     <row r="64" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B64" s="56" t="s">
         <v>178</v>
@@ -10128,13 +10135,13 @@
         <v>0.6</v>
       </c>
       <c r="AA64" s="38" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="AB64" s="42" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="AC64" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="65" spans="1:32" ht="34" x14ac:dyDescent="0.2">
@@ -10244,10 +10251,10 @@
     </row>
     <row r="68" spans="1:32" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B68" s="38" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C68" s="31" t="s">
         <v>162</v>
@@ -10256,13 +10263,13 @@
         <v>49</v>
       </c>
       <c r="AA68" s="38" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="AB68" s="42" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AC68" s="43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="69" spans="1:32" x14ac:dyDescent="0.2">
@@ -10272,7 +10279,7 @@
     </row>
     <row r="70" spans="1:32" ht="34" x14ac:dyDescent="0.2">
       <c r="A70" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B70" s="56" t="s">
         <v>232</v>
@@ -10315,10 +10322,10 @@
         <v>290</v>
       </c>
       <c r="AB70" s="42" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="AC70" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="71" spans="1:32" ht="34" x14ac:dyDescent="0.2">
@@ -10425,7 +10432,7 @@
     </row>
     <row r="75" spans="1:32" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B75" s="56" t="s">
         <v>230</v>
@@ -10464,13 +10471,13 @@
         <v>0</v>
       </c>
       <c r="AA75" s="38" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="AB75" s="42" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="AC75" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="76" spans="1:32" ht="34" x14ac:dyDescent="0.2">
@@ -10590,7 +10597,7 @@
     </row>
     <row r="79" spans="1:32" ht="34" x14ac:dyDescent="0.2">
       <c r="A79" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B79" s="38" t="s">
         <v>231</v>
@@ -10630,13 +10637,13 @@
         <v>0</v>
       </c>
       <c r="AA79" s="45" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="AB79" s="42" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="AC79" s="43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="AF79" t="s">
         <v>106</v>
@@ -10656,10 +10663,10 @@
     </row>
     <row r="81" spans="1:30" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B81" s="37" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C81" s="55" t="s">
         <v>174</v>
@@ -10689,13 +10696,13 @@
         <v>0</v>
       </c>
       <c r="AA81" s="38" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="AB81" s="42" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="AC81" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AD81" t="s">
         <v>86</v>
@@ -10703,10 +10710,10 @@
     </row>
     <row r="82" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="A82" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B82" s="37" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C82" s="55"/>
       <c r="F82" s="14" t="s">
@@ -10769,13 +10776,13 @@
         <v>0</v>
       </c>
       <c r="AA82" s="38" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="AB82" s="42" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="AC82" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="83" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -11018,10 +11025,10 @@
     </row>
     <row r="88" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="A88" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B88" s="37" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C88" s="55" t="s">
         <v>174</v>
@@ -11082,21 +11089,21 @@
         <v>0.6</v>
       </c>
       <c r="AA88" s="37" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="AB88" s="42" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AC88" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="89" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="A89" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B89" s="37" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C89" s="55"/>
       <c r="F89" s="14" t="s">
@@ -11155,13 +11162,13 @@
         <v>0.36</v>
       </c>
       <c r="AA89" s="37" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AB89" s="42" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="AC89" s="43" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="90" spans="1:30" ht="34" x14ac:dyDescent="0.2">
@@ -11295,7 +11302,7 @@
     </row>
     <row r="93" spans="1:30" ht="51" x14ac:dyDescent="0.2">
       <c r="A93" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B93" s="57" t="s">
         <v>202</v>
@@ -11335,13 +11342,13 @@
         <v>9.8621113109027395E-2</v>
       </c>
       <c r="AA93" s="37" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="AB93" s="42" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AC93" s="43" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="94" spans="1:30" ht="51" x14ac:dyDescent="0.2">
@@ -11460,10 +11467,10 @@
     </row>
     <row r="97" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A97" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B97" s="37" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="C97" s="28"/>
       <c r="F97" s="14"/>
@@ -11496,13 +11503,13 @@
         <v>0.17633270956878355</v>
       </c>
       <c r="AA97" s="37" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="AB97" s="42" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="AC97" s="43" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
     </row>
     <row r="98" spans="1:29" x14ac:dyDescent="0.2">
@@ -11512,7 +11519,7 @@
     </row>
     <row r="99" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A99" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B99" s="57" t="s">
         <v>207</v>
@@ -11552,13 +11559,13 @@
         <v>113.71737449773644</v>
       </c>
       <c r="AA99" s="38" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="AB99" s="42" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AC99" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="100" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -11683,7 +11690,7 @@
     </row>
     <row r="104" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A104" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B104" s="57" t="s">
         <v>208</v>
@@ -11724,13 +11731,13 @@
         <v>28.429343624434111</v>
       </c>
       <c r="AA104" s="38" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="AB104" s="42" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="AC104" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="105" spans="1:29" ht="17" x14ac:dyDescent="0.2">
@@ -11953,7 +11960,7 @@
     </row>
     <row r="112" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A112" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B112" s="38" t="s">
         <v>234</v>
@@ -12021,18 +12028,18 @@
         <v>24936000</v>
       </c>
       <c r="AA112" s="38" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="AB112" s="42" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AC112" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="113" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A113" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B113" s="38" t="s">
         <v>181</v>
@@ -12098,18 +12105,18 @@
         <v>1</v>
       </c>
       <c r="AA113" s="38" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="AB113" s="42" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AC113" s="43" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="114" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A114" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B114" s="38" t="s">
         <v>182</v>
@@ -12177,18 +12184,18 @@
         <v>0.92</v>
       </c>
       <c r="AA114" s="38" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="AB114" s="42" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AC114" s="43" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="115" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A115" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B115" s="38" t="s">
         <v>235</v>
@@ -12256,18 +12263,18 @@
         <v>15778712.754563004</v>
       </c>
       <c r="AA115" s="38" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="AB115" s="42" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AC115" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="116" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A116" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B116" s="38" t="s">
         <v>238</v>
@@ -12335,18 +12342,18 @@
         <v>63.276839727955583</v>
       </c>
       <c r="AA116" s="38" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="AB116" s="42" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="AC116" s="43" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="117" spans="1:29" ht="68" x14ac:dyDescent="0.2">
       <c r="A117" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B117" s="38" t="s">
         <v>276</v>
@@ -12414,13 +12421,13 @@
         <v>25.475946727955581</v>
       </c>
       <c r="AA117" s="38" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
       <c r="AB117" s="46" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AC117" s="43" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="118" spans="1:29" x14ac:dyDescent="0.2">
@@ -12451,7 +12458,7 @@
     </row>
     <row r="120" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A120" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B120" s="38" t="s">
         <v>240</v>
@@ -12524,7 +12531,7 @@
     </row>
     <row r="121" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A121" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B121" s="38" t="s">
         <v>239</v>
@@ -12564,18 +12571,18 @@
         <v>215.49749504124878</v>
       </c>
       <c r="AA121" s="38" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="AB121" s="42" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="AC121" s="43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="122" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A122" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B122" s="38" t="s">
         <v>236</v>
@@ -12643,18 +12650,18 @@
         <v>15778928.252058046</v>
       </c>
       <c r="AA122" s="38" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="AB122" s="42" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="AC122" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="123" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A123" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B123" s="38" t="s">
         <v>237</v>
@@ -12722,18 +12729,18 @@
         <v>3944732.0630145115</v>
       </c>
       <c r="AA123" s="38" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="AB123" s="42" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="AC123" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="124" spans="1:29" ht="17" x14ac:dyDescent="0.2">
       <c r="A124" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B124" s="38" t="s">
         <v>275</v>
@@ -12801,18 +12808,18 @@
         <v>7340.1134084428477</v>
       </c>
       <c r="AA124" s="38" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="AB124" s="42" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="AC124" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="125" spans="1:29" ht="51" x14ac:dyDescent="0.2">
       <c r="A125" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B125" s="38" t="s">
         <v>259</v>
@@ -12880,18 +12887,18 @@
         <v>1044</v>
       </c>
       <c r="AA125" s="38" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="AB125" s="42" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="AC125" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="126" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A126" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B126" s="38" t="s">
         <v>277</v>
@@ -12959,18 +12966,18 @@
         <v>4407.2793859099929</v>
       </c>
       <c r="AA126" s="38" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="AB126" s="42" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="AC126" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="127" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A127" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B127" s="38" t="s">
         <v>252</v>
@@ -13010,18 +13017,18 @@
         <v>9842.1904497703563</v>
       </c>
       <c r="AA127" s="38" t="s">
+        <v>324</v>
+      </c>
+      <c r="AB127" s="42" t="s">
         <v>325</v>
       </c>
-      <c r="AB127" s="42" t="s">
-        <v>326</v>
-      </c>
       <c r="AC127" s="43" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="128" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A128" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B128" s="38" t="s">
         <v>253</v>
@@ -13089,18 +13096,18 @@
         <v>0.44779456447246724</v>
       </c>
       <c r="AA128" s="38" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="AB128" s="42" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="AC128" s="43" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="129" spans="1:30" ht="68" x14ac:dyDescent="0.2">
       <c r="A129" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B129" s="38" t="s">
         <v>183</v>
@@ -13168,13 +13175,13 @@
         <v>5088667.5032287594</v>
       </c>
       <c r="AA129" s="38" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="AB129" s="42" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="AC129" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="130" spans="1:30" x14ac:dyDescent="0.2">
@@ -13204,7 +13211,7 @@
     </row>
     <row r="132" spans="1:30" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B132" s="38" t="s">
         <v>254</v>
@@ -13244,19 +13251,21 @@
         <v>2510157.8095502295</v>
       </c>
       <c r="AA132" s="38" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="AB132" s="42" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="AC132" s="43" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="133" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A133" s="50"/>
+      <c r="A133" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B133" s="38" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="C133" s="28" t="s">
         <v>174</v>
@@ -13290,11 +13299,20 @@
         <f>MIN(Y132,Y35*Z79)</f>
         <v>0</v>
       </c>
-      <c r="AA133" s="38"/>
-      <c r="AB133" s="42"/>
-      <c r="AC133" s="43"/>
+      <c r="AA133" s="38" t="s">
+        <v>489</v>
+      </c>
+      <c r="AB133" s="42" t="s">
+        <v>490</v>
+      </c>
+      <c r="AC133" s="43" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="134" spans="1:30" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B134" s="38" t="s">
         <v>255</v>
       </c>
@@ -13333,16 +13351,19 @@
         <v>388638.22348903998</v>
       </c>
       <c r="AA134" s="38" t="s">
-        <v>438</v>
+        <v>488</v>
       </c>
       <c r="AB134" s="42" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="AC134" s="43" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="135" spans="1:30" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B135" s="38" t="s">
         <v>266</v>
       </c>
@@ -13381,18 +13402,21 @@
         <v>2121519.5860611894</v>
       </c>
       <c r="AA135" s="38" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="AB135" s="42" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AC135" s="43" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="136" spans="1:30" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A136" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B136" s="38" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="C136" s="28" t="s">
         <v>174</v>
@@ -13429,16 +13453,19 @@
         <v>0</v>
       </c>
       <c r="AA136" s="38" t="s">
-        <v>434</v>
+        <v>487</v>
       </c>
       <c r="AB136" s="42" t="s">
-        <v>410</v>
+        <v>486</v>
       </c>
       <c r="AC136" s="43" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="137" spans="1:30" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A137" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B137" s="38" t="s">
         <v>262</v>
       </c>
@@ -13505,16 +13532,19 @@
         <v>336166.07900932123</v>
       </c>
       <c r="AA137" s="38" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="AB137" s="42" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="AC137" s="43" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="138" spans="1:30" ht="34" x14ac:dyDescent="0.2">
+      <c r="A138" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B138" s="38" t="s">
         <v>267</v>
       </c>
@@ -13581,13 +13611,13 @@
         <v>336166.07900932123</v>
       </c>
       <c r="AA138" s="38" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="AB138" s="42" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="AC138" s="43" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="139" spans="1:30" ht="17" x14ac:dyDescent="0.2">
@@ -13613,7 +13643,7 @@
     </row>
     <row r="140" spans="1:30" ht="119" x14ac:dyDescent="0.2">
       <c r="A140" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B140" s="38" t="s">
         <v>270</v>
@@ -13681,13 +13711,13 @@
         <v>0.40958701751064658</v>
       </c>
       <c r="AA140" s="38" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="AB140" s="42" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="AC140" s="43" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="AD140">
         <v>20</v>
@@ -13695,7 +13725,7 @@
     </row>
     <row r="141" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="A141" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B141" s="38" t="s">
         <v>184</v>
@@ -13763,13 +13793,13 @@
         <v>6.6061710417515754E-2</v>
       </c>
       <c r="AA141" s="39" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="AB141" s="42" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="AC141" s="43" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="AD141">
         <v>20</v>
@@ -13786,7 +13816,7 @@
     </row>
     <row r="143" spans="1:30" ht="51" x14ac:dyDescent="0.2">
       <c r="A143" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B143" s="38" t="s">
         <v>186</v>
@@ -13854,13 +13884,13 @@
         <v>336166.07900932123</v>
       </c>
       <c r="AA143" s="38" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="AB143" s="42" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="AC143" s="43" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="AD143">
         <v>20</v>
@@ -13868,7 +13898,7 @@
     </row>
     <row r="144" spans="1:30" ht="34" x14ac:dyDescent="0.2">
       <c r="A144" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B144" s="38" t="s">
         <v>187</v>
@@ -13936,18 +13966,18 @@
         <v>388638.22348903998</v>
       </c>
       <c r="AA144" s="38" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="AB144" s="42" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="AC144" s="43" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
     </row>
     <row r="145" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A145" s="50" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B145" s="38" t="s">
         <v>188</v>
@@ -14015,13 +14045,13 @@
         <v>0.86498460185247705</v>
       </c>
       <c r="AA145" s="38" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AB145" s="42" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="AC145" s="43" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="146" spans="1:29" x14ac:dyDescent="0.2">
@@ -14050,6 +14080,9 @@
       <c r="AC147" s="43"/>
     </row>
     <row r="148" spans="1:29" ht="51" x14ac:dyDescent="0.2">
+      <c r="A148" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B148" s="38" t="s">
         <v>268</v>
       </c>
@@ -14116,16 +14149,19 @@
         <v>24233.450635277597</v>
       </c>
       <c r="AA148" s="38" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="AB148" s="42" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AC148" s="43" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="149" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A149" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B149" s="38" t="s">
         <v>284</v>
       </c>
@@ -14189,16 +14225,19 @@
         <v>6058.3626588193993</v>
       </c>
       <c r="AA149" s="38" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="AB149" s="42" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AC149" s="43" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="150" spans="1:29" ht="51" x14ac:dyDescent="0.2">
+      <c r="A150" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B150" s="38" t="s">
         <v>269</v>
       </c>
@@ -14265,16 +14304,19 @@
         <v>84041.519752330307</v>
       </c>
       <c r="AA150" s="38" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="AB150" s="42" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="AC150" s="43" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="151" spans="1:29" ht="34" x14ac:dyDescent="0.2">
+      <c r="A151" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B151" s="38" t="s">
         <v>176</v>
       </c>
@@ -14341,16 +14383,19 @@
         <v>1888.8340225328548</v>
       </c>
       <c r="AA151" s="38" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="AB151" s="42" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="AC151" s="43" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="152" spans="1:29" ht="34" x14ac:dyDescent="0.2">
+      <c r="A152" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B152" s="38" t="s">
         <v>177</v>
       </c>
@@ -14417,16 +14462,19 @@
         <v>1373.5803521107118</v>
       </c>
       <c r="AA152" s="38" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AB152" s="42" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="AC152" s="43" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="153" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A153" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B153" s="38" t="s">
         <v>283</v>
       </c>
@@ -14490,13 +14538,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="AA153" s="38" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="AB153" s="42" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="AC153" s="43" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="154" spans="1:29" x14ac:dyDescent="0.2">
@@ -14575,6 +14623,9 @@
       <c r="AC157" s="43"/>
     </row>
     <row r="158" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A158" s="50" t="s">
+        <v>417</v>
+      </c>
       <c r="B158" s="38" t="s">
         <v>271</v>
       </c>
@@ -14582,41 +14633,41 @@
         <v>163</v>
       </c>
       <c r="G158" s="4">
-        <f>G127+G137+H137+G136</f>
+        <f>G127+G133+G136+G137+H137</f>
         <v>2000000.0000000002</v>
       </c>
       <c r="J158" s="4">
-        <f>J127+J137+K137</f>
+        <f>J127+J133+J136+J137+K137</f>
         <v>2050000</v>
       </c>
       <c r="M158" s="4">
-        <f>M127+M137+N137</f>
+        <f>M127+M133+M136+M137+N137</f>
         <v>2110000</v>
       </c>
       <c r="P158" s="4">
-        <f>P127+P137+Q137</f>
+        <f>P127+P133+P136+P137+Q137</f>
         <v>2210000</v>
       </c>
       <c r="S158" s="4">
-        <f>S127+S137+T137</f>
+        <f>S127+S133+S136+S137+T137</f>
         <v>3000000</v>
       </c>
       <c r="V158" s="4">
-        <f>V127+V137+W137</f>
+        <f>V127+V133+V136+V137+W137</f>
         <v>2360235.9978943658</v>
       </c>
       <c r="Y158" s="4">
-        <f>Y127+Y137+Z137</f>
+        <f>Y127+Y133+Y136+Y137+Z137</f>
         <v>398480.41393881035</v>
       </c>
       <c r="AA158" s="38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="AB158" s="42" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="AC158" s="43" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="159" spans="1:29" x14ac:dyDescent="0.2">
@@ -14654,19 +14705,19 @@
     </row>
     <row r="160" spans="1:29" x14ac:dyDescent="0.2">
       <c r="B160" s="38" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C160" s="31" t="s">
         <v>162</v>
       </c>
       <c r="AA160" s="38" t="s">
+        <v>358</v>
+      </c>
+      <c r="AB160" s="42" t="s">
         <v>359</v>
       </c>
-      <c r="AB160" s="42" t="s">
+      <c r="AC160" s="43" t="s">
         <v>360</v>
-      </c>
-      <c r="AC160" s="43" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="161" spans="2:30" x14ac:dyDescent="0.2">

</xml_diff>